<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-08-19T06:40:23.256Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -25,6 +25,9 @@
     <t>功率</t>
   </si>
   <si>
+    <t>刀壓</t>
+  </si>
+  <si>
     <t>速度</t>
   </si>
   <si>
@@ -32,9 +35,6 @@
   </si>
   <si>
     <t>最後更新日期</t>
-  </si>
-  <si>
-    <t>刀壓</t>
   </si>
   <si>
     <t>0.3mm</t>
@@ -52,16 +52,16 @@
     <t>(PS)</t>
   </si>
   <si>
-    <t>FILL</t>
+    <t>A4紙</t>
+  </si>
+  <si>
+    <t>03mm</t>
   </si>
   <si>
     <t>0.5mm</t>
   </si>
   <si>
-    <t>A4紙</t>
-  </si>
-  <si>
-    <t>03mm</t>
+    <t>FILL</t>
   </si>
   <si>
     <t>(PS -3)</t>
@@ -88,10 +88,10 @@
     <t>cut</t>
   </si>
   <si>
-    <t>Keep Detail</t>
+    <t>3mm</t>
   </si>
   <si>
-    <t>3mm</t>
+    <t>Keep Detail</t>
   </si>
   <si>
     <t>4mm</t>
@@ -327,19 +327,19 @@
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -351,10 +351,10 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -375,26 +375,26 @@
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -688,13 +688,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -710,7 +710,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -722,16 +722,16 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -748,16 +748,16 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>25.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
       <c r="E4" s="12"/>
@@ -773,10 +773,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="6"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -788,8 +788,8 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="s">
-        <v>13</v>
+      <c r="A6" s="14" t="s">
+        <v>14</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>16</v>
@@ -823,8 +823,8 @@
       <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -849,8 +849,8 @@
       <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -861,7 +861,7 @@
     </row>
     <row r="9">
       <c r="A9" s="21"/>
-      <c r="B9" s="9"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="12"/>
@@ -881,7 +881,7 @@
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="9"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -894,23 +894,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>5.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>5.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
       <c r="E11" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,19 +920,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -944,19 +944,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>32.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>5.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -972,7 +972,7 @@
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="6"/>
+      <c r="E14" s="9"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -984,12 +984,12 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
       <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1054,7 +1054,7 @@
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="6"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1067,12 +1067,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="6"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1084,19 +1084,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <v>5.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1108,13 +1108,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="6"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1130,7 +1130,7 @@
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="6"/>
+      <c r="E22" s="9"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1142,12 +1142,12 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
       <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -1222,10 +1222,10 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
-        <v>14</v>
+      <c r="A27" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C27" s="13"/>
@@ -1244,13 +1244,13 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="10">
         <v>100.0</v>
       </c>
       <c r="D28" s="13"/>
@@ -1268,13 +1268,13 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="10">
         <v>20.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
       <c r="D29" s="13"/>
@@ -17107,13 +17107,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17143,16 +17143,16 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>3.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -17170,16 +17170,16 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
       <c r="E4" s="7"/>
@@ -17195,12 +17195,12 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
       <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -17214,22 +17214,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>18.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
       <c r="E6" s="7"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,22 +17239,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="10">
         <v>18.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>3.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
       <c r="E7" s="11"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,9 +17265,9 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
       <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -17281,8 +17281,8 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="s">
-        <v>13</v>
+      <c r="A9" s="14" t="s">
+        <v>14</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
@@ -17387,7 +17387,7 @@
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
-      <c r="E13" s="22"/>
+      <c r="E13" s="25"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17412,7 +17412,7 @@
       <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="22"/>
+      <c r="E14" s="25"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17437,7 +17437,7 @@
       <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="22"/>
+      <c r="E15" s="25"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,7 +17450,7 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="25"/>
+      <c r="A16" s="28"/>
       <c r="E16" s="7"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -17467,11 +17467,11 @@
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
       <c r="E17" s="7"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -17485,16 +17485,16 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
       <c r="E18" s="7"/>
@@ -17510,16 +17510,16 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>40.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
       <c r="E19" s="7"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="22"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17583,7 +17583,7 @@
       <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="22"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17608,7 +17608,7 @@
       <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="22"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17639,7 +17639,7 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
@@ -17657,16 +17657,16 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
       <c r="E26" s="7"/>
@@ -17682,16 +17682,16 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <v>60.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="10">
         <v>2.0</v>
       </c>
       <c r="E27" s="11">
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="22"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17757,7 +17757,7 @@
       <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="22"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17875,10 +17875,10 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
-        <v>14</v>
+      <c r="A36" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C36" s="13"/>
@@ -17896,13 +17896,13 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <v>100.0</v>
       </c>
       <c r="D37" s="13"/>
@@ -17919,13 +17919,13 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="10">
         <v>20.0</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <v>100.0</v>
       </c>
       <c r="D38" s="13"/>
@@ -34573,13 +34573,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34595,7 +34595,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34607,16 +34607,16 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -34633,16 +34633,16 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>10.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>2.0</v>
       </c>
       <c r="E4" s="12">
@@ -34659,16 +34659,16 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="10">
         <v>20.0</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>20.0</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="10">
         <v>1.0</v>
       </c>
       <c r="E5" s="12">
@@ -34685,16 +34685,16 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>12</v>
+      <c r="A6" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>20.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
       <c r="E6" s="12">
@@ -34712,10 +34712,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="6"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="9"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34727,8 +34727,8 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="s">
-        <v>13</v>
+      <c r="A8" s="14" t="s">
+        <v>14</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>16</v>
@@ -34762,8 +34762,8 @@
       <c r="E9" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34788,8 +34788,8 @@
       <c r="E10" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34800,7 +34800,7 @@
     </row>
     <row r="11">
       <c r="A11" s="21"/>
-      <c r="B11" s="9"/>
+      <c r="B11" s="10"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="12"/>
@@ -34816,9 +34816,9 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34830,12 +34830,12 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
       <c r="E13" s="12"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -34848,16 +34848,16 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>20.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>10.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
       <c r="E14" s="12">
@@ -34874,12 +34874,12 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>12</v>
+      <c r="A15" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
       <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -34893,7 +34893,7 @@
     </row>
     <row r="16">
       <c r="A16" s="21"/>
-      <c r="B16" s="9"/>
+      <c r="B16" s="10"/>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="12"/>
@@ -34913,7 +34913,7 @@
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="9"/>
+      <c r="D17" s="10"/>
       <c r="E17" s="12"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -34926,23 +34926,23 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
       <c r="E18" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34952,19 +34952,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>5.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>15.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34976,19 +34976,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <v>32.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -35004,7 +35004,7 @@
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="6"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35016,12 +35016,12 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
       <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -35086,7 +35086,7 @@
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="6"/>
+      <c r="E25" s="9"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35099,12 +35099,12 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
-      <c r="E26" s="6"/>
+      <c r="E26" s="9"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35116,19 +35116,19 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <v>5.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="10">
         <v>1.0</v>
       </c>
-      <c r="E27" s="6"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35140,13 +35140,13 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="6"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35162,7 +35162,7 @@
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
-      <c r="E29" s="6"/>
+      <c r="E29" s="9"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35174,12 +35174,12 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
       <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -35254,10 +35254,10 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="s">
-        <v>14</v>
+      <c r="A34" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C34" s="13"/>
@@ -35276,13 +35276,13 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="10">
         <v>2.0</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="10">
         <v>100.0</v>
       </c>
       <c r="D35" s="13"/>
@@ -35300,13 +35300,13 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="10">
         <v>20.0</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="10">
         <v>100.0</v>
       </c>
       <c r="D36" s="13"/>
@@ -51135,16 +51135,16 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51156,12 +51156,12 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="9"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="10"/>
       <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
@@ -51173,16 +51173,16 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="8">
         <v>60.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
       <c r="E3" s="7"/>
@@ -51212,10 +51212,10 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -51230,16 +51230,16 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>6.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>100.0</v>
       </c>
-      <c r="D6" s="9"/>
+      <c r="D6" s="10"/>
       <c r="E6" s="11">
         <v>46241.84478354167</v>
       </c>
@@ -51253,20 +51253,20 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="10">
         <v>8.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>60.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
       <c r="E7" s="11">
-        <v>46156.860351111114</v>
+        <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -51296,9 +51296,9 @@
       <c r="A9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
       <c r="E9" s="7"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -51310,16 +51310,16 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="10">
         <v>10.0</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="10">
         <v>45.0</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="10">
         <v>1.0</v>
       </c>
       <c r="E10" s="11">
@@ -51335,16 +51335,16 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>11.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>20.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
       <c r="E11" s="11">
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="24"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,14 +51375,14 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
       <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -51394,16 +51394,16 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14" ht="20.25" customHeight="1">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>5.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>60.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
       <c r="E14" s="11">
@@ -51419,16 +51419,16 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="10">
         <v>30.0</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="10">
         <v>1.0</v>
       </c>
       <c r="E15" s="11"/>
@@ -51442,23 +51442,23 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="10">
         <v>5.0</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="10">
         <v>30.0</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="10">
         <v>4.0</v>
       </c>
       <c r="E16" s="11">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="14" t="s">
-        <v>24</v>
+      <c r="F16" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51469,16 +51469,16 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="10">
         <v>12.0</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="10">
         <v>20.0</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="10">
         <v>1.0</v>
       </c>
       <c r="E17" s="11">
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="24"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,7 +51510,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -51526,16 +51526,16 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="8">
         <v>6.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <v>45.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
       <c r="E20" s="11">
@@ -51551,16 +51551,16 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="8">
         <v>18.0</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="8">
         <v>20.0</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="10">
         <v>1.0</v>
       </c>
       <c r="E21" s="11">
@@ -51576,7 +51576,7 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="8"/>
+      <c r="A22" s="6"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -51591,10 +51591,10 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="26" t="s">
-        <v>13</v>
+      <c r="A23" s="24" t="s">
+        <v>14</v>
       </c>
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="27" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="13"/>
@@ -51612,16 +51612,16 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="8">
         <v>6.0</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="8">
         <v>50.0</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="10">
         <v>1.0</v>
       </c>
       <c r="E24" s="11">
@@ -51637,16 +51637,16 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="8">
         <v>8.0</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C25" s="8">
         <v>30.0</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="10">
         <v>1.0</v>
       </c>
       <c r="E25" s="11">
@@ -51662,23 +51662,23 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="8">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>30.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>4.0</v>
       </c>
       <c r="E26" s="11">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="14" t="s">
-        <v>24</v>
+      <c r="F26" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51689,16 +51689,16 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="8">
         <v>17.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="8">
         <v>15.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="10">
         <v>1.0</v>
       </c>
       <c r="E27" s="11">
@@ -51714,7 +51714,7 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8"/>
+      <c r="A28" s="6"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
@@ -51729,10 +51729,10 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="26" t="s">
+      <c r="A29" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="29" t="s">
+      <c r="B29" s="27" t="s">
         <v>22</v>
       </c>
       <c r="C29" s="13"/>
@@ -51748,16 +51748,16 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
+      <c r="A30" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="8">
         <v>6.0</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C30" s="8">
         <v>50.0</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="10">
         <v>1.0</v>
       </c>
       <c r="E30" s="11">
@@ -51773,16 +51773,16 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="10">
+      <c r="B31" s="8">
         <v>8.0</v>
       </c>
-      <c r="C31" s="10">
+      <c r="C31" s="8">
         <v>30.0</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="10">
         <v>1.0</v>
       </c>
       <c r="E31" s="7"/>
@@ -51796,16 +51796,16 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="10">
+      <c r="B32" s="8">
         <v>15.0</v>
       </c>
-      <c r="C32" s="10">
+      <c r="C32" s="8">
         <v>10.0</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="10">
         <v>2.0</v>
       </c>
       <c r="E32" s="11">
@@ -51821,7 +51821,7 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="8"/>
+      <c r="A33" s="6"/>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
@@ -51836,13 +51836,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="s">
+      <c r="A34" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
       <c r="D34" s="16"/>
-      <c r="E34" s="22"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51890,7 +51890,7 @@
       <c r="D36" s="41">
         <v>1.0</v>
       </c>
-      <c r="E36" s="22"/>
+      <c r="E36" s="25"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51901,16 +51901,16 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="10">
         <v>10.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <v>150.0</v>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="10">
         <v>1.0</v>
       </c>
       <c r="E37" s="11">
@@ -51958,16 +51958,16 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="s">
+      <c r="A40" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="10">
         <v>40.0</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="10">
         <v>15.0</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="10">
         <v>1.0</v>
       </c>
       <c r="E40" s="11">
@@ -52015,16 +52015,16 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="s">
+      <c r="A43" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="10">
         <v>9.0</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C43" s="10">
         <v>20.0</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="10">
         <v>1.0</v>
       </c>
       <c r="E43" s="11">
@@ -52040,16 +52040,16 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="10">
         <v>55.0</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="10">
         <v>20.0</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="10">
         <v>1.0</v>
       </c>
       <c r="E44" s="11">
@@ -52065,22 +52065,22 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="s">
+      <c r="A45" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B45" s="10">
         <v>10.0</v>
       </c>
-      <c r="C45" s="9">
+      <c r="C45" s="10">
         <v>250.0</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45" s="10">
         <v>1.0</v>
       </c>
       <c r="E45" s="11">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="14" t="s">
+      <c r="F45" s="15" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52108,7 +52108,7 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
@@ -52124,16 +52124,16 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="s">
+      <c r="A48" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="10">
         <v>55.0</v>
       </c>
-      <c r="C48" s="9">
+      <c r="C48" s="10">
         <v>10.0</v>
       </c>
-      <c r="D48" s="9">
+      <c r="D48" s="10">
         <v>1.0</v>
       </c>
       <c r="E48" s="11">
@@ -52181,16 +52181,16 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="s">
+      <c r="A51" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="9">
+      <c r="B51" s="10">
         <v>60.0</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="10">
         <v>10.0</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="10">
         <v>1.0</v>
       </c>
       <c r="E51" s="11">
@@ -52221,9 +52221,7 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="42" t="s">
-        <v>33</v>
-      </c>
+      <c r="A53" s="42"/>
       <c r="B53" s="13"/>
       <c r="C53" s="13"/>
       <c r="D53" s="13"/>
@@ -52238,21 +52236,13 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="s">
-        <v>12</v>
+      <c r="A54" s="42" t="s">
+        <v>33</v>
       </c>
-      <c r="B54" s="10">
-        <v>70.0</v>
-      </c>
-      <c r="C54" s="10">
-        <v>300.0</v>
-      </c>
-      <c r="D54" s="10">
-        <v>1.0</v>
-      </c>
-      <c r="E54" s="11">
-        <v>46223.80899857639</v>
-      </c>
+      <c r="B54" s="13"/>
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="7"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52263,20 +52253,20 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="s">
-        <v>8</v>
+      <c r="A55" s="6" t="s">
+        <v>15</v>
       </c>
-      <c r="B55" s="10">
-        <v>10.0</v>
+      <c r="B55" s="8">
+        <v>70.0</v>
       </c>
-      <c r="C55" s="10">
-        <v>20.0</v>
+      <c r="C55" s="8">
+        <v>300.0</v>
       </c>
-      <c r="D55" s="10">
+      <c r="D55" s="8">
         <v>1.0</v>
       </c>
       <c r="E55" s="11">
-        <v>46223.80911148148</v>
+        <v>46223.80899857639</v>
       </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
@@ -52288,20 +52278,20 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="s">
-        <v>9</v>
+      <c r="A56" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="B56" s="10">
-        <v>70.0</v>
-      </c>
-      <c r="C56" s="10">
+      <c r="B56" s="8">
         <v>10.0</v>
       </c>
-      <c r="D56" s="10">
+      <c r="C56" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="D56" s="8">
         <v>1.0</v>
       </c>
       <c r="E56" s="11">
-        <v>46207.72572512731</v>
+        <v>46223.80911148148</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52313,11 +52303,21 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="8"/>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="7"/>
+      <c r="A57" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B57" s="8">
+        <v>70.0</v>
+      </c>
+      <c r="C57" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="D57" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E57" s="11">
+        <v>46207.72572512731</v>
+      </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -52328,17 +52328,11 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B58" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="11">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="A58" s="6"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="10"/>
+      <c r="E58" s="7"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52349,16 +52343,16 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="8">
-        <v>50.0</v>
+      <c r="A59" s="6" t="s">
+        <v>34</v>
       </c>
-      <c r="B59" s="9">
-        <v>100.0</v>
+      <c r="B59" s="10" t="s">
+        <v>35</v>
       </c>
-      <c r="C59" s="13"/>
-      <c r="D59" s="13"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="10"/>
       <c r="E59" s="11">
-        <v>45946.87887299768</v>
+        <v>45946.87875708334</v>
       </c>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
@@ -52370,13 +52364,17 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="43" t="s">
-        <v>36</v>
+      <c r="A60" s="6">
+        <v>50.0</v>
       </c>
-      <c r="B60" s="44"/>
-      <c r="C60" s="44"/>
-      <c r="D60" s="44"/>
-      <c r="E60" s="45"/>
+      <c r="B60" s="10">
+        <v>100.0</v>
+      </c>
+      <c r="C60" s="13"/>
+      <c r="D60" s="13"/>
+      <c r="E60" s="11">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -52387,21 +52385,13 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="39" t="s">
-        <v>37</v>
+      <c r="A61" s="43" t="s">
+        <v>36</v>
       </c>
-      <c r="B61" s="39">
-        <v>100.0</v>
-      </c>
-      <c r="C61" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="D61" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="E61" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B61" s="44"/>
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="E61" s="45"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -52412,11 +52402,21 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="40"/>
-      <c r="B62" s="40"/>
-      <c r="C62" s="4"/>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
+      <c r="A62" s="39" t="s">
+        <v>37</v>
+      </c>
+      <c r="B62" s="39">
+        <v>100.0</v>
+      </c>
+      <c r="C62" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="D62" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E62" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -52427,9 +52427,7 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="39" t="s">
-        <v>38</v>
-      </c>
+      <c r="A63" s="40"/>
       <c r="B63" s="40"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
@@ -52444,21 +52442,13 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="s">
-        <v>9</v>
+      <c r="A64" s="39" t="s">
+        <v>38</v>
       </c>
-      <c r="B64" s="39">
-        <v>50.0</v>
-      </c>
-      <c r="C64" s="14">
-        <v>20.0</v>
-      </c>
-      <c r="D64" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="E64" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B64" s="40"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
@@ -52469,18 +52459,20 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="39" t="s">
-        <v>39</v>
+      <c r="A65" s="6" t="s">
+        <v>9</v>
       </c>
       <c r="B65" s="39">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
-      <c r="C65" s="14">
-        <v>16.0</v>
+      <c r="C65" s="15">
+        <v>20.0</v>
       </c>
-      <c r="D65" s="4"/>
+      <c r="D65" s="15">
+        <v>1.0</v>
+      </c>
       <c r="E65" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
@@ -52492,11 +52484,19 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="40"/>
-      <c r="B66" s="40"/>
-      <c r="C66" s="4"/>
+      <c r="A66" s="39" t="s">
+        <v>39</v>
+      </c>
+      <c r="B66" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="C66" s="15">
+        <v>16.0</v>
+      </c>
       <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
+      <c r="E66" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -52507,17 +52507,11 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="B67" s="39" t="s">
-        <v>25</v>
-      </c>
+      <c r="A67" s="40"/>
+      <c r="B67" s="40"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E67" s="4"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -52529,19 +52523,15 @@
     </row>
     <row r="68">
       <c r="A68" s="39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
-      <c r="B68" s="39">
-        <v>5.0</v>
+      <c r="B68" s="39" t="s">
+        <v>24</v>
       </c>
-      <c r="C68" s="14">
-        <v>80.0</v>
-      </c>
-      <c r="D68" s="14">
-        <v>1.0</v>
-      </c>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
       <c r="E68" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
@@ -52554,19 +52544,19 @@
     </row>
     <row r="69">
       <c r="A69" s="39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B69" s="39">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
-      <c r="C69" s="14">
-        <v>10.0</v>
+      <c r="C69" s="15">
+        <v>80.0</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69" s="15">
         <v>1.0</v>
       </c>
       <c r="E69" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
@@ -52579,19 +52569,19 @@
     </row>
     <row r="70">
       <c r="A70" s="39" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="B70" s="39">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
-      <c r="C70" s="14">
+      <c r="C70" s="15">
         <v>10.0</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70" s="15">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
@@ -52603,11 +52593,21 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="40"/>
-      <c r="B71" s="40"/>
-      <c r="C71" s="4"/>
-      <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
+      <c r="A71" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="B71" s="39">
+        <v>30.0</v>
+      </c>
+      <c r="C71" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D71" s="15">
+        <v>1.0</v>
+      </c>
+      <c r="E71" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -52618,17 +52618,11 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="B72" s="39" t="s">
-        <v>33</v>
-      </c>
+      <c r="A72" s="40"/>
+      <c r="B72" s="40"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
-      <c r="E72" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E72" s="4"/>
       <c r="F72" s="4"/>
       <c r="G72" s="4"/>
       <c r="H72" s="4"/>
@@ -52640,18 +52634,16 @@
     </row>
     <row r="73">
       <c r="A73" s="39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
-      <c r="B73" s="39">
-        <v>5.0</v>
+      <c r="B73" s="39" t="s">
+        <v>33</v>
       </c>
-      <c r="C73" s="14">
-        <v>80.0</v>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D73" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="E73" s="4"/>
       <c r="F73" s="4"/>
       <c r="G73" s="4"/>
       <c r="H73" s="4"/>
@@ -52663,15 +52655,15 @@
     </row>
     <row r="74">
       <c r="A74" s="39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B74" s="39">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
-      <c r="C74" s="14">
-        <v>10.0</v>
+      <c r="C74" s="15">
+        <v>80.0</v>
       </c>
-      <c r="D74" s="14">
+      <c r="D74" s="15">
         <v>1.0</v>
       </c>
       <c r="E74" s="4"/>
@@ -52686,20 +52678,18 @@
     </row>
     <row r="75">
       <c r="A75" s="39" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="B75" s="39">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
-      <c r="C75" s="14">
+      <c r="C75" s="15">
         <v>10.0</v>
       </c>
-      <c r="D75" s="14">
-        <v>6.0</v>
+      <c r="D75" s="15">
+        <v>1.0</v>
       </c>
-      <c r="E75" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E75" s="4"/>
       <c r="F75" s="4"/>
       <c r="G75" s="4"/>
       <c r="H75" s="4"/>
@@ -52710,11 +52700,21 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76">
-      <c r="A76" s="40"/>
-      <c r="B76" s="40"/>
-      <c r="C76" s="4"/>
-      <c r="D76" s="4"/>
-      <c r="E76" s="4"/>
+      <c r="A76" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="B76" s="39">
+        <v>20.0</v>
+      </c>
+      <c r="C76" s="15">
+        <v>10.0</v>
+      </c>
+      <c r="D76" s="15">
+        <v>6.0</v>
+      </c>
+      <c r="E76" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F76" s="4"/>
       <c r="G76" s="4"/>
       <c r="H76" s="4"/>
@@ -52725,7 +52725,7 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="39"/>
+      <c r="A77" s="40"/>
       <c r="B77" s="40"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
@@ -52740,7 +52740,7 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="40"/>
+      <c r="A78" s="39"/>
       <c r="B78" s="40"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
@@ -52755,8 +52755,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="4"/>
-      <c r="B79" s="4"/>
+      <c r="A79" s="40"/>
+      <c r="B79" s="40"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
@@ -66824,6 +66824,21 @@
       <c r="L1016" s="4"/>
       <c r="M1016" s="4"/>
     </row>
+    <row r="1017">
+      <c r="A1017" s="4"/>
+      <c r="B1017" s="4"/>
+      <c r="C1017" s="4"/>
+      <c r="D1017" s="4"/>
+      <c r="E1017" s="4"/>
+      <c r="F1017" s="4"/>
+      <c r="G1017" s="4"/>
+      <c r="H1017" s="4"/>
+      <c r="I1017" s="4"/>
+      <c r="J1017" s="4"/>
+      <c r="K1017" s="4"/>
+      <c r="L1017" s="4"/>
+      <c r="M1017" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-08-19T06:40:31.159Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,18 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="43">
   <si>
     <t>項目</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>功率</t>
-  </si>
-  <si>
-    <t>刀壓</t>
   </si>
   <si>
     <t>速度</t>
@@ -34,7 +28,13 @@
     <t>次數</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>最後更新日期</t>
+  </si>
+  <si>
+    <t>刀壓</t>
   </si>
   <si>
     <t>0.3mm</t>
@@ -49,7 +49,16 @@
     <t>Cut(detail)</t>
   </si>
   <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
     <t>(PS)</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -58,19 +67,7 @@
     <t>03mm</t>
   </si>
   <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
     <t>Cut</t>
-  </si>
-  <si>
-    <t>0.3 mm</t>
   </si>
   <si>
     <t>1mm</t>
@@ -79,22 +76,25 @@
     <t>Fill</t>
   </si>
   <si>
+    <t>0.3 mm</t>
+  </si>
+  <si>
     <t>2mm</t>
+  </si>
+  <si>
+    <t>3mm</t>
   </si>
   <si>
     <t>PS</t>
   </si>
   <si>
+    <t>4mm</t>
+  </si>
+  <si>
     <t>cut</t>
   </si>
   <si>
-    <t>3mm</t>
-  </si>
-  <si>
     <t>Keep Detail</t>
-  </si>
-  <si>
-    <t>4mm</t>
   </si>
   <si>
     <t>(0.9 Power)</t>
@@ -209,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -327,37 +327,37 @@
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -375,26 +375,26 @@
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -685,16 +685,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -710,7 +710,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -722,19 +722,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -748,19 +748,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>25.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -773,10 +773,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -788,14 +788,14 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
       <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -811,20 +811,20 @@
       <c r="A7" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="15">
         <v>4.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="15">
         <v>10.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="15">
         <v>1.0</v>
       </c>
       <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -837,20 +837,20 @@
       <c r="A8" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <v>25.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="15">
         <v>5.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
       <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -861,10 +861,10 @@
     </row>
     <row r="9">
       <c r="A9" s="21"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="12"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +877,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="12"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -894,23 +894,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>5.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="9">
         <v>5.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,19 +920,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="9">
         <v>5.0</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="9">
         <v>15.0</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="9">
         <v>1.0</v>
       </c>
-      <c r="E12" s="9"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -944,19 +944,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>32.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>5.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="9"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -969,10 +969,10 @@
     </row>
     <row r="14">
       <c r="A14" s="21"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="9"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -984,12 +984,12 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
       <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1005,13 +1005,13 @@
       <c r="A16" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="15">
         <v>5.0</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="15">
         <v>5.0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="15">
         <v>1.0</v>
       </c>
       <c r="E16" s="17"/>
@@ -1029,13 +1029,13 @@
       <c r="A17" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="15">
         <v>50.0</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="15">
         <v>5.0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="15">
         <v>1.0</v>
       </c>
       <c r="E17" s="17"/>
@@ -1051,10 +1051,10 @@
     </row>
     <row r="18">
       <c r="A18" s="21"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="9"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1067,12 +1067,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="9"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1084,19 +1084,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>5.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="9"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1108,13 +1108,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="22">
       <c r="A22" s="21"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="9"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1142,12 +1142,12 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="s">
-        <v>26</v>
+      <c r="A23" s="13" t="s">
+        <v>24</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
       <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -1163,13 +1163,13 @@
       <c r="A24" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="15">
         <v>5.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
       <c r="E24" s="17"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,14 +1222,14 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
-        <v>12</v>
+      <c r="A27" s="9" t="s">
+        <v>15</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
       <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
@@ -1244,16 +1244,16 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="9">
         <v>2.0</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="13"/>
+      <c r="D28" s="14"/>
       <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
@@ -1268,16 +1268,16 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="9">
         <v>20.0</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="13"/>
+      <c r="D29" s="14"/>
       <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17104,16 +17104,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17143,19 +17143,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>3.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17170,16 +17170,16 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
       <c r="E4" s="7"/>
@@ -17195,12 +17195,12 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>11</v>
+      <c r="A5" s="8" t="s">
+        <v>12</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
       <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -17214,22 +17214,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>18.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
       <c r="E6" s="7"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,22 +17239,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <v>18.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>3.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17265,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="11"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,12 +17281,12 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="s">
-        <v>14</v>
+      <c r="A9" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
       <c r="E9" s="20"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -17303,13 +17303,13 @@
       <c r="A10" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <v>4.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <v>15.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
       <c r="E10" s="20">
@@ -17330,13 +17330,13 @@
       <c r="A11" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="15">
         <v>25.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="15">
         <v>10.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="15">
         <v>1.0</v>
       </c>
       <c r="E11" s="20">
@@ -17355,15 +17355,15 @@
     </row>
     <row r="12">
       <c r="A12" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <v>4.0</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="15">
         <v>10.0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="15">
         <v>1.0</v>
       </c>
       <c r="E12" s="20">
@@ -17382,12 +17382,12 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="25"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="22"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17403,16 +17403,16 @@
       <c r="A14" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="15">
         <v>2.0</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="15">
         <v>18.0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="15">
         <v>1.0</v>
       </c>
-      <c r="E14" s="25"/>
+      <c r="E14" s="22"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17428,16 +17428,16 @@
       <c r="A15" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="15">
         <v>18.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="15">
         <v>4.0</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="15">
         <v>1.0</v>
       </c>
-      <c r="E15" s="25"/>
+      <c r="E15" s="22"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,7 +17450,7 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="28"/>
+      <c r="A16" s="23"/>
       <c r="E16" s="7"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -17465,13 +17465,13 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
-      <c r="B17" s="29" t="s">
-        <v>11</v>
+      <c r="B17" s="25" t="s">
+        <v>12</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
       <c r="E17" s="7"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -17485,16 +17485,16 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
       <c r="E18" s="7"/>
@@ -17510,16 +17510,16 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>40.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
       <c r="E19" s="7"/>
@@ -17536,9 +17536,9 @@
     </row>
     <row r="20">
       <c r="A20" s="21"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
       <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="25"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="22"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17574,16 +17574,16 @@
       <c r="A22" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="15">
         <v>8.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="15">
         <v>15.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="15">
         <v>1.0</v>
       </c>
-      <c r="E22" s="25"/>
+      <c r="E22" s="22"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17599,16 +17599,16 @@
       <c r="A23" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <v>55.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="15">
         <v>2.0</v>
       </c>
-      <c r="E23" s="25"/>
+      <c r="E23" s="22"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17622,9 +17622,9 @@
     </row>
     <row r="24">
       <c r="A24" s="21"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
       <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -17639,11 +17639,11 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
       <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -17657,16 +17657,16 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
       <c r="E26" s="7"/>
@@ -17682,19 +17682,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>60.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="12">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17710,9 +17710,9 @@
     </row>
     <row r="28">
       <c r="A28" s="21"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
       <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="s">
-        <v>26</v>
+      <c r="A29" s="13" t="s">
+        <v>24</v>
       </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="25"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="22"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17748,16 +17748,16 @@
       <c r="A30" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="15">
         <v>18.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="15">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="15">
         <v>1.0</v>
       </c>
-      <c r="E30" s="25"/>
+      <c r="E30" s="22"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17875,14 +17875,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
-        <v>12</v>
+      <c r="A36" s="9" t="s">
+        <v>15</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17896,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="s">
+      <c r="A37" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="9">
         <v>2.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="14"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17919,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
+      <c r="A38" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="9">
         <v>20.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="14"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34570,16 +34570,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34595,7 +34595,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34607,19 +34607,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34633,19 +34633,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>10.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>2.0</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="11">
         <v>46232.916719409724</v>
       </c>
       <c r="F4" s="4"/>
@@ -34659,19 +34659,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>20.0</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>20.0</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>1.0</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="11">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34685,19 +34685,19 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>15</v>
+      <c r="A6" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>20.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="11">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34712,10 +34712,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34727,14 +34727,14 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
       <c r="E8" s="17"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -34750,20 +34750,20 @@
       <c r="A9" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="15">
         <v>4.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="15">
         <v>10.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="15">
         <v>1.0</v>
       </c>
       <c r="E9" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34776,20 +34776,20 @@
       <c r="A10" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <v>20.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <v>10.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
       <c r="E10" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34800,10 +34800,10 @@
     </row>
     <row r="11">
       <c r="A11" s="21"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="12"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34816,9 +34816,9 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
-      <c r="E12" s="9"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34830,13 +34830,13 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="12"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34848,19 +34848,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>20.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>10.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="11">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34874,13 +34874,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="s">
-        <v>15</v>
+      <c r="A15" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="12"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34893,10 +34893,10 @@
     </row>
     <row r="16">
       <c r="A16" s="21"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="12"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34909,12 +34909,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="12"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34926,23 +34926,23 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34952,19 +34952,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>5.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>15.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="9"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34976,19 +34976,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>32.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="9"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -35001,10 +35001,10 @@
     </row>
     <row r="21">
       <c r="A21" s="21"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35016,12 +35016,12 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
       <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -35037,13 +35037,13 @@
       <c r="A23" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <v>5.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="15">
         <v>1.0</v>
       </c>
       <c r="E23" s="17"/>
@@ -35061,13 +35061,13 @@
       <c r="A24" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="15">
         <v>50.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
       <c r="E24" s="17"/>
@@ -35083,10 +35083,10 @@
     </row>
     <row r="25">
       <c r="A25" s="21"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35099,12 +35099,12 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="9"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35116,19 +35116,19 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>5.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>1.0</v>
       </c>
-      <c r="E27" s="9"/>
+      <c r="E27" s="6"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35140,13 +35140,13 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35159,10 +35159,10 @@
     </row>
     <row r="29">
       <c r="A29" s="21"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="9"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35174,12 +35174,12 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="s">
-        <v>26</v>
+      <c r="A30" s="13" t="s">
+        <v>24</v>
       </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
       <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -35195,13 +35195,13 @@
       <c r="A31" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="15">
         <v>5.0</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="15">
         <v>5.0</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="15">
         <v>1.0</v>
       </c>
       <c r="E31" s="17"/>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35254,14 +35254,14 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="s">
-        <v>12</v>
+      <c r="A34" s="9" t="s">
+        <v>15</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
       <c r="E34" s="34">
         <v>46051.96156388889</v>
       </c>
@@ -35276,16 +35276,16 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="9">
         <v>2.0</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="9">
         <v>100.0</v>
       </c>
-      <c r="D35" s="13"/>
+      <c r="D35" s="14"/>
       <c r="E35" s="34">
         <v>46100.83597384259</v>
       </c>
@@ -35300,16 +35300,16 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="10">
+      <c r="B36" s="9">
         <v>20.0</v>
       </c>
-      <c r="C36" s="10">
+      <c r="C36" s="9">
         <v>100.0</v>
       </c>
-      <c r="D36" s="13"/>
+      <c r="D36" s="14"/>
       <c r="E36" s="34">
         <v>46100.83604224537</v>
       </c>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="13"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,19 +51132,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51156,12 +51156,12 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="9"/>
       <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
@@ -51173,16 +51173,16 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>60.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
       <c r="E3" s="7"/>
@@ -51197,9 +51197,9 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
       <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -51212,14 +51212,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="11"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51230,17 +51230,17 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>6.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>100.0</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="11">
+      <c r="D6" s="9"/>
+      <c r="E6" s="12">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51253,19 +51253,19 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <v>8.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>60.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="12">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51279,9 +51279,9 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="5"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
       <c r="E8" s="7"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -51294,11 +51294,11 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
       <c r="E9" s="7"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -51310,19 +51310,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="9">
         <v>10.0</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="9">
         <v>45.0</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="12">
         <v>46106.73232292824</v>
       </c>
       <c r="F10" s="4"/>
@@ -51335,19 +51335,19 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>11.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="9">
         <v>20.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="12">
         <v>46106.732369062505</v>
       </c>
       <c r="F11" s="4"/>
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="27"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,15 +51375,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="s">
-        <v>18</v>
+      <c r="A13" s="28" t="s">
+        <v>20</v>
       </c>
-      <c r="B13" s="27" t="s">
-        <v>22</v>
+      <c r="B13" s="29" t="s">
+        <v>23</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="12"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51394,19 +51394,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14" ht="20.25" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>20</v>
+      <c r="A14" s="8" t="s">
+        <v>19</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>5.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>60.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="12">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51419,19 +51419,19 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="9">
         <v>5.0</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="9">
         <v>30.0</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="9">
         <v>1.0</v>
       </c>
-      <c r="E15" s="11"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51442,23 +51442,23 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>23</v>
+      <c r="A16" s="8" t="s">
+        <v>25</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="9">
         <v>5.0</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="9">
         <v>30.0</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="9">
         <v>4.0</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="15" t="s">
-        <v>25</v>
+      <c r="F16" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51469,19 +51469,19 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="9">
         <v>12.0</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="9">
         <v>20.0</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="9">
         <v>1.0</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="12">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="27"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,11 +51510,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
       <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -51526,19 +51526,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="10">
         <v>6.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="10">
         <v>45.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="12">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51551,19 +51551,19 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="10">
         <v>18.0</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="10">
         <v>20.0</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="9">
         <v>1.0</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="12">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51576,10 +51576,10 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="6"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
       <c r="E22" s="7"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -51591,15 +51591,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="24" t="s">
-        <v>14</v>
+      <c r="A23" s="28" t="s">
+        <v>11</v>
       </c>
-      <c r="B23" s="27" t="s">
-        <v>22</v>
+      <c r="B23" s="29" t="s">
+        <v>23</v>
       </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="11">
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="12">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51612,19 +51612,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="s">
-        <v>20</v>
+      <c r="A24" s="8" t="s">
+        <v>19</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="10">
         <v>6.0</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C24" s="10">
         <v>50.0</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="12">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51637,19 +51637,19 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="10">
         <v>8.0</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="10">
         <v>30.0</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="9">
         <v>1.0</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="12">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51662,23 +51662,23 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="10">
         <v>30.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>4.0</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="15" t="s">
-        <v>25</v>
+      <c r="F26" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51689,19 +51689,19 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="10">
         <v>17.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="10">
         <v>15.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>1.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="12">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51714,10 +51714,10 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="6"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
       <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -51729,14 +51729,14 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="24" t="s">
-        <v>19</v>
+      <c r="A29" s="28" t="s">
+        <v>18</v>
       </c>
-      <c r="B29" s="27" t="s">
-        <v>22</v>
+      <c r="B29" s="29" t="s">
+        <v>23</v>
       </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
       <c r="E29" s="7"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -51748,19 +51748,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="s">
-        <v>20</v>
+      <c r="A30" s="8" t="s">
+        <v>19</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="10">
         <v>6.0</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C30" s="10">
         <v>50.0</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="9">
         <v>1.0</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="12">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51773,16 +51773,16 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="10">
         <v>8.0</v>
       </c>
-      <c r="C31" s="8">
+      <c r="C31" s="10">
         <v>30.0</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="9">
         <v>1.0</v>
       </c>
       <c r="E31" s="7"/>
@@ -51796,19 +51796,19 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="10">
         <v>15.0</v>
       </c>
-      <c r="C32" s="8">
+      <c r="C32" s="10">
         <v>10.0</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="9">
         <v>2.0</v>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="12">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51821,10 +51821,10 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="6"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
       <c r="E33" s="7"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51836,13 +51836,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="s">
-        <v>19</v>
+      <c r="A34" s="13" t="s">
+        <v>18</v>
       </c>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="25"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="22"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51890,7 +51890,7 @@
       <c r="D36" s="41">
         <v>1.0</v>
       </c>
-      <c r="E36" s="25"/>
+      <c r="E36" s="22"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51901,19 +51901,19 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="s">
-        <v>20</v>
+      <c r="A37" s="8" t="s">
+        <v>19</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="9">
         <v>10.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="9">
         <v>150.0</v>
       </c>
-      <c r="D37" s="10">
+      <c r="D37" s="9">
         <v>1.0</v>
       </c>
-      <c r="E37" s="11">
+      <c r="E37" s="12">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51927,9 +51927,9 @@
     </row>
     <row r="38">
       <c r="A38" s="21"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
       <c r="E38" s="7"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51944,9 +51944,9 @@
       <c r="A39" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
       <c r="E39" s="7"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -51958,19 +51958,19 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B40" s="10">
+      <c r="B40" s="9">
         <v>40.0</v>
       </c>
-      <c r="C40" s="10">
+      <c r="C40" s="9">
         <v>15.0</v>
       </c>
-      <c r="D40" s="10">
+      <c r="D40" s="9">
         <v>1.0</v>
       </c>
-      <c r="E40" s="11">
+      <c r="E40" s="12">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51984,9 +51984,9 @@
     </row>
     <row r="41">
       <c r="A41" s="5"/>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
       <c r="E41" s="7"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -52001,9 +52001,9 @@
       <c r="A42" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
       <c r="E42" s="7"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -52015,19 +52015,19 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="s">
+      <c r="A43" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="9">
         <v>9.0</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="9">
         <v>20.0</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="11">
+      <c r="E43" s="12">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52040,19 +52040,19 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B44" s="10">
+      <c r="B44" s="9">
         <v>55.0</v>
       </c>
-      <c r="C44" s="10">
+      <c r="C44" s="9">
         <v>20.0</v>
       </c>
-      <c r="D44" s="10">
+      <c r="D44" s="9">
         <v>1.0</v>
       </c>
-      <c r="E44" s="11">
+      <c r="E44" s="12">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52065,22 +52065,22 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="s">
+      <c r="A45" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B45" s="10">
+      <c r="B45" s="9">
         <v>10.0</v>
       </c>
-      <c r="C45" s="10">
+      <c r="C45" s="9">
         <v>250.0</v>
       </c>
-      <c r="D45" s="10">
+      <c r="D45" s="9">
         <v>1.0</v>
       </c>
-      <c r="E45" s="11">
+      <c r="E45" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="15" t="s">
+      <c r="F45" s="16" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52093,9 +52093,9 @@
     </row>
     <row r="46">
       <c r="A46" s="42"/>
-      <c r="B46" s="13"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
       <c r="E46" s="7"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -52108,11 +52108,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
       <c r="E47" s="7"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -52124,19 +52124,19 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="s">
+      <c r="A48" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B48" s="10">
+      <c r="B48" s="9">
         <v>55.0</v>
       </c>
-      <c r="C48" s="10">
+      <c r="C48" s="9">
         <v>10.0</v>
       </c>
-      <c r="D48" s="10">
+      <c r="D48" s="9">
         <v>1.0</v>
       </c>
-      <c r="E48" s="11">
+      <c r="E48" s="12">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52150,9 +52150,9 @@
     </row>
     <row r="49">
       <c r="A49" s="42"/>
-      <c r="B49" s="13"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
       <c r="E49" s="7"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
@@ -52165,11 +52165,11 @@
     </row>
     <row r="50">
       <c r="A50" s="42" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
-      <c r="B50" s="13"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="14"/>
       <c r="E50" s="7"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52181,19 +52181,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="10">
+      <c r="B51" s="9">
         <v>60.0</v>
       </c>
-      <c r="C51" s="10">
+      <c r="C51" s="9">
         <v>10.0</v>
       </c>
-      <c r="D51" s="10">
+      <c r="D51" s="9">
         <v>1.0</v>
       </c>
-      <c r="E51" s="11">
+      <c r="E51" s="12">
         <v>46203.63265940972</v>
       </c>
       <c r="F51" s="4"/>
@@ -52206,10 +52206,12 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="42"/>
-      <c r="B52" s="13"/>
-      <c r="C52" s="13"/>
-      <c r="D52" s="13"/>
+      <c r="A52" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B52" s="14"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="14"/>
       <c r="E52" s="7"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -52222,9 +52224,9 @@
     </row>
     <row r="53">
       <c r="A53" s="42"/>
-      <c r="B53" s="13"/>
-      <c r="C53" s="13"/>
-      <c r="D53" s="13"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="14"/>
+      <c r="D53" s="14"/>
       <c r="E53" s="7"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52239,9 +52241,9 @@
       <c r="A54" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
+      <c r="B54" s="14"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="14"/>
       <c r="E54" s="7"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
@@ -52253,19 +52255,19 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="s">
-        <v>15</v>
+      <c r="A55" s="8" t="s">
+        <v>13</v>
       </c>
-      <c r="B55" s="8">
+      <c r="B55" s="10">
         <v>70.0</v>
       </c>
-      <c r="C55" s="8">
+      <c r="C55" s="10">
         <v>300.0</v>
       </c>
-      <c r="D55" s="8">
+      <c r="D55" s="10">
         <v>1.0</v>
       </c>
-      <c r="E55" s="11">
+      <c r="E55" s="12">
         <v>46223.80899857639</v>
       </c>
       <c r="F55" s="4"/>
@@ -52278,19 +52280,19 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="s">
+      <c r="A56" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B56" s="8">
+      <c r="B56" s="10">
         <v>10.0</v>
       </c>
-      <c r="C56" s="8">
+      <c r="C56" s="10">
         <v>20.0</v>
       </c>
-      <c r="D56" s="8">
+      <c r="D56" s="10">
         <v>1.0</v>
       </c>
-      <c r="E56" s="11">
+      <c r="E56" s="12">
         <v>46223.80911148148</v>
       </c>
       <c r="F56" s="4"/>
@@ -52303,19 +52305,19 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="s">
+      <c r="A57" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B57" s="8">
+      <c r="B57" s="10">
         <v>70.0</v>
       </c>
-      <c r="C57" s="8">
+      <c r="C57" s="10">
         <v>10.0</v>
       </c>
-      <c r="D57" s="8">
+      <c r="D57" s="10">
         <v>1.0</v>
       </c>
-      <c r="E57" s="11">
+      <c r="E57" s="12">
         <v>46207.72572512731</v>
       </c>
       <c r="F57" s="4"/>
@@ -52328,10 +52330,10 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="6"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
+      <c r="A58" s="8"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
       <c r="E58" s="7"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
@@ -52343,15 +52345,15 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="s">
+      <c r="A59" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="10" t="s">
+      <c r="B59" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="11">
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="12">
         <v>45946.87875708334</v>
       </c>
       <c r="F59" s="4"/>
@@ -52364,15 +52366,15 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="6">
+      <c r="A60" s="8">
         <v>50.0</v>
       </c>
-      <c r="B60" s="10">
+      <c r="B60" s="9">
         <v>100.0</v>
       </c>
-      <c r="C60" s="13"/>
-      <c r="D60" s="13"/>
-      <c r="E60" s="11">
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="12">
         <v>45946.87887299768</v>
       </c>
       <c r="F60" s="4"/>
@@ -52408,10 +52410,10 @@
       <c r="B62" s="39">
         <v>100.0</v>
       </c>
-      <c r="C62" s="15">
+      <c r="C62" s="16">
         <v>1.0</v>
       </c>
-      <c r="D62" s="15">
+      <c r="D62" s="16">
         <v>2.0</v>
       </c>
       <c r="E62" s="46">
@@ -52459,16 +52461,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="s">
+      <c r="A65" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B65" s="39">
         <v>50.0</v>
       </c>
-      <c r="C65" s="15">
+      <c r="C65" s="16">
         <v>20.0</v>
       </c>
-      <c r="D65" s="15">
+      <c r="D65" s="16">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52490,7 +52492,7 @@
       <c r="B66" s="39">
         <v>15.0</v>
       </c>
-      <c r="C66" s="15">
+      <c r="C66" s="16">
         <v>16.0</v>
       </c>
       <c r="D66" s="4"/>
@@ -52526,7 +52528,7 @@
         <v>40</v>
       </c>
       <c r="B68" s="39" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -52549,10 +52551,10 @@
       <c r="B69" s="39">
         <v>5.0</v>
       </c>
-      <c r="C69" s="15">
+      <c r="C69" s="16">
         <v>80.0</v>
       </c>
-      <c r="D69" s="15">
+      <c r="D69" s="16">
         <v>1.0</v>
       </c>
       <c r="E69" s="46">
@@ -52574,10 +52576,10 @@
       <c r="B70" s="39">
         <v>15.0</v>
       </c>
-      <c r="C70" s="15">
+      <c r="C70" s="16">
         <v>10.0</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="16">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52599,10 +52601,10 @@
       <c r="B71" s="39">
         <v>30.0</v>
       </c>
-      <c r="C71" s="15">
+      <c r="C71" s="16">
         <v>10.0</v>
       </c>
-      <c r="D71" s="15">
+      <c r="D71" s="16">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52660,10 +52662,10 @@
       <c r="B74" s="39">
         <v>5.0</v>
       </c>
-      <c r="C74" s="15">
+      <c r="C74" s="16">
         <v>80.0</v>
       </c>
-      <c r="D74" s="15">
+      <c r="D74" s="16">
         <v>1.0</v>
       </c>
       <c r="E74" s="4"/>
@@ -52683,10 +52685,10 @@
       <c r="B75" s="39">
         <v>15.0</v>
       </c>
-      <c r="C75" s="15">
+      <c r="C75" s="16">
         <v>10.0</v>
       </c>
-      <c r="D75" s="15">
+      <c r="D75" s="16">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52706,10 +52708,10 @@
       <c r="B76" s="39">
         <v>20.0</v>
       </c>
-      <c r="C76" s="15">
+      <c r="C76" s="16">
         <v>10.0</v>
       </c>
-      <c r="D76" s="15">
+      <c r="D76" s="16">
         <v>6.0</v>
       </c>
       <c r="E76" s="46">

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-08-19T06:40:33.366Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,6 +19,9 @@
     <t>項目</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>功率</t>
   </si>
   <si>
@@ -28,13 +31,10 @@
     <t>次數</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
+    <t>刀壓</t>
   </si>
   <si>
     <t>最後更新日期</t>
-  </si>
-  <si>
-    <t>刀壓</t>
   </si>
   <si>
     <t>0.3mm</t>
@@ -43,10 +43,13 @@
     <t>Line</t>
   </si>
   <si>
+    <t>Cut(detail)</t>
+  </si>
+  <si>
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
+    <t>FILL</t>
   </si>
   <si>
     <t>0.5mm</t>
@@ -55,28 +58,34 @@
     <t>(PS)</t>
   </si>
   <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
     <t>A4紙</t>
   </si>
   <si>
     <t>03mm</t>
   </si>
   <si>
+    <t>(PS -3)</t>
+  </si>
+  <si>
     <t>Cut</t>
+  </si>
+  <si>
+    <t>0.3 mm</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>Fill</t>
   </si>
   <si>
     <t>1mm</t>
   </si>
   <si>
-    <t>Fill</t>
+    <t>cut</t>
   </si>
   <si>
-    <t>0.3 mm</t>
+    <t>Keep Detail</t>
   </si>
   <si>
     <t>2mm</t>
@@ -85,28 +94,19 @@
     <t>3mm</t>
   </si>
   <si>
-    <t>PS</t>
-  </si>
-  <si>
     <t>4mm</t>
   </si>
   <si>
-    <t>cut</t>
+    <t>(0.9 Power)</t>
   </si>
   <si>
-    <t>Keep Detail</t>
-  </si>
-  <si>
-    <t>(0.9 Power)</t>
+    <t>６</t>
   </si>
   <si>
     <t>甲板紙</t>
   </si>
   <si>
     <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>６</t>
   </si>
   <si>
     <t>1.5mm</t>
@@ -209,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -330,9 +330,6 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -342,34 +339,49 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -379,23 +391,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -415,6 +415,9 @@
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -429,9 +432,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -685,16 +685,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -722,16 +722,16 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -748,16 +748,16 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>25.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
       <c r="E4" s="11"/>
@@ -773,9 +773,9 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
       <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -788,14 +788,14 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="s">
-        <v>11</v>
+      <c r="A6" s="14" t="s">
+        <v>12</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>14</v>
+      <c r="B6" s="16" t="s">
+        <v>16</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
       <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -808,23 +808,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="21">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,23 +834,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="s">
-        <v>9</v>
+      <c r="A8" s="19" t="s">
+        <v>10</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="21">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,10 +860,10 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="21"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
       <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -877,11 +877,11 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="9"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="8"/>
       <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -894,23 +894,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>5.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="8">
         <v>5.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>1.0</v>
       </c>
       <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,16 +920,16 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <v>5.0</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>15.0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>1.0</v>
       </c>
       <c r="E12" s="6"/>
@@ -944,16 +944,16 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>9</v>
+      <c r="A13" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="8">
         <v>32.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="8">
         <v>5.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="8">
         <v>1.0</v>
       </c>
       <c r="E13" s="6"/>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="21"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -984,12 +984,12 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>21</v>
+      <c r="A15" s="14" t="s">
+        <v>24</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
       <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1002,16 +1002,16 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
       <c r="E16" s="17"/>
@@ -1026,16 +1026,16 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="s">
-        <v>9</v>
+      <c r="A17" s="19" t="s">
+        <v>10</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
       <c r="E17" s="17"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="21"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1067,11 +1067,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1084,16 +1084,16 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>5.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -1108,12 +1108,12 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>9</v>
+      <c r="A21" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="21"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
+      <c r="A22" s="25"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1142,12 +1142,12 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
-        <v>24</v>
+      <c r="A23" s="14" t="s">
+        <v>26</v>
       </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
       <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -1160,16 +1160,16 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
       <c r="E24" s="17"/>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="25">
       <c r="A25" s="30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B25" s="31">
         <v>55.0</v>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,14 +1222,14 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
-        <v>15</v>
+      <c r="A27" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
       <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
@@ -1244,16 +1244,16 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="8">
         <v>2.0</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="8">
         <v>100.0</v>
       </c>
-      <c r="D28" s="14"/>
+      <c r="D28" s="13"/>
       <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
@@ -1268,16 +1268,16 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="8">
         <v>20.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="8">
         <v>100.0</v>
       </c>
-      <c r="D29" s="14"/>
+      <c r="D29" s="13"/>
       <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="14"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="14"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17104,16 +17104,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17130,7 +17130,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17143,16 +17143,16 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>3.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
       <c r="E3" s="12">
@@ -17170,19 +17170,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="7"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17195,13 +17195,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>12</v>
+      <c r="A5" s="7" t="s">
+        <v>13</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17214,22 +17214,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>18.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,22 +17239,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>9</v>
+      <c r="A7" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>18.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="8">
         <v>3.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="8">
         <v>1.0</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,9 +17265,9 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
       <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -17281,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>11</v>
+      <c r="A9" s="14" t="s">
+        <v>12</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="20"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="22"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17300,19 +17300,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="22">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,19 +17327,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="s">
-        <v>9</v>
+      <c r="A11" s="19" t="s">
+        <v>10</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="22">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17354,19 +17354,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="s">
-        <v>19</v>
+      <c r="A12" s="19" t="s">
+        <v>20</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="22">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17381,13 +17381,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="s">
-        <v>12</v>
+      <c r="A13" s="19" t="s">
+        <v>13</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="22"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17400,19 +17400,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="22"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,19 +17425,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="s">
-        <v>9</v>
+      <c r="A15" s="19" t="s">
+        <v>10</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="22"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="23"/>
-      <c r="E16" s="7"/>
+      <c r="A16" s="27"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17465,14 +17465,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
-      <c r="B17" s="25" t="s">
-        <v>12</v>
+      <c r="B17" s="28" t="s">
+        <v>13</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="7"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17485,19 +17485,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="7"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17510,19 +17510,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>9</v>
+      <c r="A19" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <v>40.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="8">
         <v>5.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
-      <c r="E19" s="7"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="21"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="7"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="s">
-        <v>21</v>
+      <c r="A21" s="14" t="s">
+        <v>24</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="22"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17571,19 +17571,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="22"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,19 +17596,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
-        <v>9</v>
+      <c r="A23" s="19" t="s">
+        <v>10</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="22"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="21"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="7"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="10"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17639,12 +17639,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="7"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="10"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17657,19 +17657,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="8">
         <v>10.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="8">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="8">
         <v>1.0</v>
       </c>
-      <c r="E26" s="7"/>
+      <c r="E26" s="10"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17682,16 +17682,16 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>9</v>
+      <c r="A27" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="8">
         <v>60.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="8">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="8">
         <v>2.0</v>
       </c>
       <c r="E27" s="12">
@@ -17709,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="21"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="7"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="s">
-        <v>24</v>
+      <c r="A29" s="14" t="s">
+        <v>26</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="22"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17745,19 +17745,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <v>18.0</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="22"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17771,7 +17771,7 @@
     </row>
     <row r="31">
       <c r="A31" s="30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B31" s="31">
         <v>70.0</v>
@@ -17812,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="36" t="s">
-        <v>28</v>
+      <c r="A33" s="37" t="s">
+        <v>29</v>
       </c>
-      <c r="B33" s="37">
+      <c r="B33" s="38">
         <v>5.0</v>
       </c>
-      <c r="C33" s="37">
+      <c r="C33" s="38">
         <v>10.0</v>
       </c>
-      <c r="D33" s="37">
+      <c r="D33" s="38">
         <v>2.0</v>
       </c>
-      <c r="E33" s="38">
+      <c r="E33" s="39">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="39" t="s">
-        <v>29</v>
+      <c r="F33" s="40" t="s">
+        <v>30</v>
       </c>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="40"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="40"/>
-      <c r="N33" s="40"/>
-      <c r="O33" s="40"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17875,14 +17875,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
-        <v>15</v>
+      <c r="A36" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17896,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="8">
         <v>2.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="8">
         <v>100.0</v>
       </c>
-      <c r="D37" s="14"/>
+      <c r="D37" s="13"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17919,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="8">
         <v>20.0</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="8">
         <v>100.0</v>
       </c>
-      <c r="D38" s="14"/>
+      <c r="D38" s="13"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34570,16 +34570,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34607,16 +34607,16 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
       <c r="E3" s="11">
@@ -34633,16 +34633,16 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>10</v>
+      <c r="A4" s="7" t="s">
+        <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>10.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>2.0</v>
       </c>
       <c r="E4" s="11">
@@ -34659,16 +34659,16 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>9</v>
+      <c r="A5" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>20.0</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="8">
         <v>20.0</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="8">
         <v>1.0</v>
       </c>
       <c r="E5" s="11">
@@ -34685,16 +34685,16 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>13</v>
+      <c r="A6" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>20.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>1.0</v>
       </c>
       <c r="E6" s="11">
@@ -34712,9 +34712,9 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
       <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -34727,14 +34727,14 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>11</v>
+      <c r="A8" s="14" t="s">
+        <v>12</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>14</v>
+      <c r="B8" s="16" t="s">
+        <v>16</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
       <c r="E8" s="17"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -34747,23 +34747,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="16">
         <v>4.0</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="16">
         <v>10.0</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="21">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34773,23 +34773,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="s">
-        <v>9</v>
+      <c r="A10" s="19" t="s">
+        <v>10</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <v>20.0</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>10.0</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="21">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,10 +34799,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="21"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
       <c r="E11" s="11"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -34816,7 +34816,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34830,12 +34830,12 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
       <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -34848,16 +34848,16 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
-        <v>9</v>
+      <c r="A14" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>20.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>10.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>1.0</v>
       </c>
       <c r="E14" s="11">
@@ -34874,12 +34874,12 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>13</v>
+      <c r="A15" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
       <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -34892,10 +34892,10 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="21"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
       <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34909,11 +34909,11 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="9"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="8"/>
       <c r="E17" s="11"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -34926,23 +34926,23 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="8">
         <v>1.0</v>
       </c>
       <c r="E18" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34952,16 +34952,16 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <v>5.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="8">
         <v>15.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="8">
         <v>1.0</v>
       </c>
       <c r="E19" s="6"/>
@@ -34976,16 +34976,16 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>9</v>
+      <c r="A20" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>32.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -35000,10 +35000,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="21"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35016,12 +35016,12 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>21</v>
+      <c r="A22" s="14" t="s">
+        <v>24</v>
       </c>
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
       <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -35034,16 +35034,16 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>5.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>1.0</v>
       </c>
       <c r="E23" s="17"/>
@@ -35058,16 +35058,16 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="s">
-        <v>9</v>
+      <c r="A24" s="19" t="s">
+        <v>10</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <v>50.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
       <c r="E24" s="17"/>
@@ -35082,10 +35082,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="21"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
+      <c r="A25" s="25"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35099,11 +35099,11 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35116,16 +35116,16 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="8">
         <v>5.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="8">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="8">
         <v>1.0</v>
       </c>
       <c r="E27" s="6"/>
@@ -35140,12 +35140,12 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>9</v>
+      <c r="A28" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35158,10 +35158,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="21"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35174,12 +35174,12 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
-        <v>24</v>
+      <c r="A30" s="14" t="s">
+        <v>26</v>
       </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
       <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -35192,16 +35192,16 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="15">
+      <c r="B31" s="16">
         <v>5.0</v>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="16">
         <v>5.0</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="16">
         <v>1.0</v>
       </c>
       <c r="E31" s="17"/>
@@ -35217,7 +35217,7 @@
     </row>
     <row r="32">
       <c r="A32" s="30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B32" s="31">
         <v>55.0</v>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="14"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35254,14 +35254,14 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="s">
-        <v>15</v>
+      <c r="A34" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
       <c r="E34" s="34">
         <v>46051.96156388889</v>
       </c>
@@ -35276,16 +35276,16 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="8">
         <v>2.0</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="8">
         <v>100.0</v>
       </c>
-      <c r="D35" s="14"/>
+      <c r="D35" s="13"/>
       <c r="E35" s="34">
         <v>46100.83597384259</v>
       </c>
@@ -35300,16 +35300,16 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="8">
         <v>20.0</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="8">
         <v>100.0</v>
       </c>
-      <c r="D36" s="14"/>
+      <c r="D36" s="13"/>
       <c r="E36" s="34">
         <v>46100.83604224537</v>
       </c>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,19 +51132,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>5</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51156,13 +51156,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="7"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51173,19 +51173,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>9</v>
+      <c r="A3" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>60.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="7"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51197,10 +51197,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="7"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51212,13 +51212,13 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
       <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -51230,16 +51230,16 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>6.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>100.0</v>
       </c>
-      <c r="D6" s="9"/>
+      <c r="D6" s="8"/>
       <c r="E6" s="12">
         <v>46241.84478354167</v>
       </c>
@@ -51253,16 +51253,16 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>8.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="8">
         <v>60.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="8">
         <v>1.0</v>
       </c>
       <c r="E7" s="12">
@@ -51279,10 +51279,10 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="5"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="7"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51294,12 +51294,12 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="7"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="10"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51310,16 +51310,16 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>10.0</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="8">
         <v>45.0</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>1.0</v>
       </c>
       <c r="E10" s="12">
@@ -51335,16 +51335,16 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>11.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="8">
         <v>20.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>1.0</v>
       </c>
       <c r="E11" s="12">
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="27"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="20"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,14 +51375,14 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="s">
-        <v>20</v>
+      <c r="A13" s="23" t="s">
+        <v>18</v>
       </c>
-      <c r="B13" s="29" t="s">
-        <v>23</v>
+      <c r="B13" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
       <c r="E13" s="12"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -51394,16 +51394,16 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14" ht="20.25" customHeight="1">
-      <c r="A14" s="8" t="s">
-        <v>19</v>
+      <c r="A14" s="7" t="s">
+        <v>20</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>5.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>60.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>1.0</v>
       </c>
       <c r="E14" s="12">
@@ -51419,16 +51419,16 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="8">
         <v>5.0</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="8">
         <v>30.0</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="8">
         <v>1.0</v>
       </c>
       <c r="E15" s="12"/>
@@ -51442,23 +51442,23 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>25</v>
+      <c r="A16" s="7" t="s">
+        <v>22</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <v>5.0</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="8">
         <v>30.0</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="8">
         <v>4.0</v>
       </c>
       <c r="E16" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="16" t="s">
-        <v>26</v>
+      <c r="F16" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51469,16 +51469,16 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="8">
         <v>12.0</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="8">
         <v>20.0</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="8">
         <v>1.0</v>
       </c>
       <c r="E17" s="12">
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="27"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="20"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,12 +51510,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="7"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51526,16 +51526,16 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>6.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>45.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="8">
         <v>1.0</v>
       </c>
       <c r="E20" s="12">
@@ -51551,16 +51551,16 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>9</v>
+      <c r="A21" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="9">
         <v>18.0</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="9">
         <v>20.0</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="8">
         <v>1.0</v>
       </c>
       <c r="E21" s="12">
@@ -51576,11 +51576,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="8"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="7"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="10"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51591,14 +51591,14 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="s">
-        <v>11</v>
+      <c r="A23" s="23" t="s">
+        <v>12</v>
       </c>
-      <c r="B23" s="29" t="s">
-        <v>23</v>
+      <c r="B23" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
       <c r="E23" s="12">
         <v>46155.850816817125</v>
       </c>
@@ -51612,16 +51612,16 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>19</v>
+      <c r="A24" s="7" t="s">
+        <v>20</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="9">
         <v>6.0</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="9">
         <v>50.0</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="8">
         <v>1.0</v>
       </c>
       <c r="E24" s="12">
@@ -51637,16 +51637,16 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="9">
         <v>8.0</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C25" s="9">
         <v>30.0</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="8">
         <v>1.0</v>
       </c>
       <c r="E25" s="12">
@@ -51662,23 +51662,23 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="9">
         <v>30.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="8">
         <v>4.0</v>
       </c>
       <c r="E26" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="16" t="s">
-        <v>26</v>
+      <c r="F26" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51689,16 +51689,16 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>17.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="9">
         <v>15.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="8">
         <v>1.0</v>
       </c>
       <c r="E27" s="12">
@@ -51714,11 +51714,11 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="7"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51729,15 +51729,15 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="s">
-        <v>18</v>
+      <c r="A29" s="23" t="s">
+        <v>21</v>
       </c>
-      <c r="B29" s="29" t="s">
-        <v>23</v>
+      <c r="B29" s="24" t="s">
+        <v>19</v>
       </c>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="7"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="10"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51748,16 +51748,16 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>19</v>
+      <c r="A30" s="7" t="s">
+        <v>20</v>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="9">
         <v>6.0</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C30" s="9">
         <v>50.0</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="8">
         <v>1.0</v>
       </c>
       <c r="E30" s="12">
@@ -51773,19 +51773,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="10">
+      <c r="B31" s="9">
         <v>8.0</v>
       </c>
-      <c r="C31" s="10">
+      <c r="C31" s="9">
         <v>30.0</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="8">
         <v>1.0</v>
       </c>
-      <c r="E31" s="7"/>
+      <c r="E31" s="10"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51796,16 +51796,16 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
-        <v>9</v>
+      <c r="A32" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B32" s="10">
+      <c r="B32" s="9">
         <v>15.0</v>
       </c>
-      <c r="C32" s="10">
+      <c r="C32" s="9">
         <v>10.0</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="8">
         <v>2.0</v>
       </c>
       <c r="E32" s="12">
@@ -51821,11 +51821,11 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="8"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="7"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="10"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51836,13 +51836,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="s">
-        <v>18</v>
+      <c r="A34" s="14" t="s">
+        <v>21</v>
       </c>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="22"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="26"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51853,19 +51853,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="41" t="s">
-        <v>30</v>
+      <c r="B35" s="36" t="s">
+        <v>28</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="36">
         <v>40.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="36">
         <v>1.0</v>
       </c>
-      <c r="E35" s="20">
+      <c r="E35" s="22">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51878,19 +51878,19 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="s">
-        <v>9</v>
+      <c r="A36" s="19" t="s">
+        <v>10</v>
       </c>
-      <c r="B36" s="41">
+      <c r="B36" s="36">
         <v>30.0</v>
       </c>
-      <c r="C36" s="41">
+      <c r="C36" s="36">
         <v>15.0</v>
       </c>
-      <c r="D36" s="41">
+      <c r="D36" s="36">
         <v>1.0</v>
       </c>
-      <c r="E36" s="22"/>
+      <c r="E36" s="26"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51901,16 +51901,16 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>19</v>
+      <c r="A37" s="7" t="s">
+        <v>20</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="8">
         <v>10.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="8">
         <v>150.0</v>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="8">
         <v>1.0</v>
       </c>
       <c r="E37" s="12">
@@ -51926,11 +51926,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="21"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="7"/>
+      <c r="A38" s="25"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="10"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51944,10 +51944,10 @@
       <c r="A39" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="7"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="10"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51958,16 +51958,16 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="s">
-        <v>9</v>
+      <c r="A40" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="8">
         <v>40.0</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="8">
         <v>15.0</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="8">
         <v>1.0</v>
       </c>
       <c r="E40" s="12">
@@ -51984,10 +51984,10 @@
     </row>
     <row r="41">
       <c r="A41" s="5"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="7"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="10"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51999,12 +51999,12 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="7"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="10"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -52015,16 +52015,16 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="s">
+      <c r="A43" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="8">
         <v>9.0</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C43" s="8">
         <v>20.0</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="8">
         <v>1.0</v>
       </c>
       <c r="E43" s="12">
@@ -52040,16 +52040,16 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="s">
-        <v>9</v>
+      <c r="A44" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="8">
         <v>55.0</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="8">
         <v>20.0</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="8">
         <v>1.0</v>
       </c>
       <c r="E44" s="12">
@@ -52065,22 +52065,22 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="s">
+      <c r="A45" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B45" s="8">
         <v>10.0</v>
       </c>
-      <c r="C45" s="9">
+      <c r="C45" s="8">
         <v>250.0</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45" s="8">
         <v>1.0</v>
       </c>
       <c r="E45" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="16" t="s">
+      <c r="F45" s="15" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52093,10 +52093,10 @@
     </row>
     <row r="46">
       <c r="A46" s="42"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="7"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="10"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52108,12 +52108,12 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="7"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="10"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52124,16 +52124,16 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="s">
-        <v>9</v>
+      <c r="A48" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="8">
         <v>55.0</v>
       </c>
-      <c r="C48" s="9">
+      <c r="C48" s="8">
         <v>10.0</v>
       </c>
-      <c r="D48" s="9">
+      <c r="D48" s="8">
         <v>1.0</v>
       </c>
       <c r="E48" s="12">
@@ -52150,10 +52150,10 @@
     </row>
     <row r="49">
       <c r="A49" s="42"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="7"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="10"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52165,12 +52165,12 @@
     </row>
     <row r="50">
       <c r="A50" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="7"/>
+      <c r="B50" s="13"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="10"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52181,16 +52181,16 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="s">
-        <v>9</v>
+      <c r="A51" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B51" s="9">
+      <c r="B51" s="8">
         <v>60.0</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="8">
         <v>10.0</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="8">
         <v>1.0</v>
       </c>
       <c r="E51" s="12">
@@ -52206,13 +52206,19 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="s">
+      <c r="A52" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="7"/>
+      <c r="B52" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="C52" s="8">
+        <v>50.0</v>
+      </c>
+      <c r="D52" s="13"/>
+      <c r="E52" s="12">
+        <v>46253.61147633102</v>
+      </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -52224,10 +52230,10 @@
     </row>
     <row r="53">
       <c r="A53" s="42"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="7"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="10"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52241,10 +52247,10 @@
       <c r="A54" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="7"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="10"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52255,16 +52261,16 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="s">
-        <v>13</v>
+      <c r="A55" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B55" s="10">
+      <c r="B55" s="9">
         <v>70.0</v>
       </c>
-      <c r="C55" s="10">
+      <c r="C55" s="9">
         <v>300.0</v>
       </c>
-      <c r="D55" s="10">
+      <c r="D55" s="9">
         <v>1.0</v>
       </c>
       <c r="E55" s="12">
@@ -52280,16 +52286,16 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="s">
+      <c r="A56" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B56" s="10">
+      <c r="B56" s="9">
         <v>10.0</v>
       </c>
-      <c r="C56" s="10">
+      <c r="C56" s="9">
         <v>20.0</v>
       </c>
-      <c r="D56" s="10">
+      <c r="D56" s="9">
         <v>1.0</v>
       </c>
       <c r="E56" s="12">
@@ -52305,16 +52311,16 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="s">
-        <v>9</v>
+      <c r="A57" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B57" s="10">
+      <c r="B57" s="9">
         <v>70.0</v>
       </c>
-      <c r="C57" s="10">
+      <c r="C57" s="9">
         <v>10.0</v>
       </c>
-      <c r="D57" s="10">
+      <c r="D57" s="9">
         <v>1.0</v>
       </c>
       <c r="E57" s="12">
@@ -52330,11 +52336,11 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="8"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="7"/>
+      <c r="A58" s="7"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="10"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52345,14 +52351,14 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="B59" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
       <c r="E59" s="12">
         <v>45946.87875708334</v>
       </c>
@@ -52366,14 +52372,14 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="8">
+      <c r="A60" s="7">
         <v>50.0</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60" s="8">
         <v>100.0</v>
       </c>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
+      <c r="C60" s="13"/>
+      <c r="D60" s="13"/>
       <c r="E60" s="12">
         <v>45946.87887299768</v>
       </c>
@@ -52404,16 +52410,16 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="39" t="s">
+      <c r="A62" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B62" s="39">
+      <c r="B62" s="40">
         <v>100.0</v>
       </c>
-      <c r="C62" s="16">
+      <c r="C62" s="15">
         <v>1.0</v>
       </c>
-      <c r="D62" s="16">
+      <c r="D62" s="15">
         <v>2.0</v>
       </c>
       <c r="E62" s="46">
@@ -52429,8 +52435,8 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="40"/>
-      <c r="B63" s="40"/>
+      <c r="A63" s="41"/>
+      <c r="B63" s="41"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
@@ -52444,10 +52450,10 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="39" t="s">
+      <c r="A64" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B64" s="40"/>
+      <c r="B64" s="41"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
@@ -52461,16 +52467,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="s">
-        <v>9</v>
+      <c r="A65" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B65" s="39">
+      <c r="B65" s="40">
         <v>50.0</v>
       </c>
-      <c r="C65" s="16">
+      <c r="C65" s="15">
         <v>20.0</v>
       </c>
-      <c r="D65" s="16">
+      <c r="D65" s="15">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52486,13 +52492,13 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="39" t="s">
+      <c r="A66" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B66" s="39">
+      <c r="B66" s="40">
         <v>15.0</v>
       </c>
-      <c r="C66" s="16">
+      <c r="C66" s="15">
         <v>16.0</v>
       </c>
       <c r="D66" s="4"/>
@@ -52509,8 +52515,8 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="40"/>
-      <c r="B67" s="40"/>
+      <c r="A67" s="41"/>
+      <c r="B67" s="41"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
@@ -52524,11 +52530,11 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="39" t="s">
+      <c r="A68" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="39" t="s">
-        <v>22</v>
+      <c r="B68" s="40" t="s">
+        <v>25</v>
       </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -52545,16 +52551,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="39" t="s">
+      <c r="A69" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="39">
+      <c r="B69" s="40">
         <v>5.0</v>
       </c>
-      <c r="C69" s="16">
+      <c r="C69" s="15">
         <v>80.0</v>
       </c>
-      <c r="D69" s="16">
+      <c r="D69" s="15">
         <v>1.0</v>
       </c>
       <c r="E69" s="46">
@@ -52570,16 +52576,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="39" t="s">
+      <c r="A70" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B70" s="39">
+      <c r="B70" s="40">
         <v>15.0</v>
       </c>
-      <c r="C70" s="16">
+      <c r="C70" s="15">
         <v>10.0</v>
       </c>
-      <c r="D70" s="16">
+      <c r="D70" s="15">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52595,16 +52601,16 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="39" t="s">
+      <c r="A71" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="B71" s="39">
+      <c r="B71" s="40">
         <v>30.0</v>
       </c>
-      <c r="C71" s="16">
+      <c r="C71" s="15">
         <v>10.0</v>
       </c>
-      <c r="D71" s="16">
+      <c r="D71" s="15">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52620,8 +52626,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="40"/>
-      <c r="B72" s="40"/>
+      <c r="A72" s="41"/>
+      <c r="B72" s="41"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52635,10 +52641,10 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="39" t="s">
+      <c r="A73" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B73" s="39" t="s">
+      <c r="B73" s="40" t="s">
         <v>33</v>
       </c>
       <c r="C73" s="4"/>
@@ -52656,16 +52662,16 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="39" t="s">
+      <c r="A74" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B74" s="39">
+      <c r="B74" s="40">
         <v>5.0</v>
       </c>
-      <c r="C74" s="16">
+      <c r="C74" s="15">
         <v>80.0</v>
       </c>
-      <c r="D74" s="16">
+      <c r="D74" s="15">
         <v>1.0</v>
       </c>
       <c r="E74" s="4"/>
@@ -52679,16 +52685,16 @@
       <c r="M74" s="4"/>
     </row>
     <row r="75">
-      <c r="A75" s="39" t="s">
+      <c r="A75" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B75" s="39">
+      <c r="B75" s="40">
         <v>15.0</v>
       </c>
-      <c r="C75" s="16">
+      <c r="C75" s="15">
         <v>10.0</v>
       </c>
-      <c r="D75" s="16">
+      <c r="D75" s="15">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52702,16 +52708,16 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76">
-      <c r="A76" s="39" t="s">
+      <c r="A76" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="B76" s="39">
+      <c r="B76" s="40">
         <v>20.0</v>
       </c>
-      <c r="C76" s="16">
+      <c r="C76" s="15">
         <v>10.0</v>
       </c>
-      <c r="D76" s="16">
+      <c r="D76" s="15">
         <v>6.0</v>
       </c>
       <c r="E76" s="46">
@@ -52727,8 +52733,8 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="40"/>
-      <c r="B77" s="40"/>
+      <c r="A77" s="41"/>
+      <c r="B77" s="41"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
@@ -52742,8 +52748,8 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="39"/>
-      <c r="B78" s="40"/>
+      <c r="A78" s="40"/>
+      <c r="B78" s="41"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
@@ -52757,8 +52763,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="40"/>
-      <c r="B79" s="40"/>
+      <c r="A79" s="41"/>
+      <c r="B79" s="41"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-08-19T06:40:35.376Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,9 +19,6 @@
     <t>項目</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>功率</t>
   </si>
   <si>
@@ -29,9 +26,6 @@
   </si>
   <si>
     <t>次數</t>
-  </si>
-  <si>
-    <t>刀壓</t>
   </si>
   <si>
     <t>最後更新日期</t>
@@ -49,13 +43,37 @@
     <t>Cut-1/2</t>
   </si>
   <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
     <t>FILL</t>
   </si>
   <si>
-    <t>0.5mm</t>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>(PS)</t>
+  </si>
+  <si>
+    <t>1mm</t>
+  </si>
+  <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
+    <t>刀壓</t>
+  </si>
+  <si>
+    <t>2mm</t>
+  </si>
+  <si>
+    <t>3mm</t>
+  </si>
+  <si>
+    <t>Fill</t>
+  </si>
+  <si>
+    <t>4mm</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -64,10 +82,10 @@
     <t>03mm</t>
   </si>
   <si>
-    <t>(PS -3)</t>
+    <t>Cut</t>
   </si>
   <si>
-    <t>Cut</t>
+    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>0.3 mm</t>
@@ -76,37 +94,19 @@
     <t>PS</t>
   </si>
   <si>
-    <t>Fill</t>
-  </si>
-  <si>
-    <t>1mm</t>
-  </si>
-  <si>
     <t>cut</t>
   </si>
   <si>
     <t>Keep Detail</t>
   </si>
   <si>
-    <t>2mm</t>
-  </si>
-  <si>
-    <t>3mm</t>
-  </si>
-  <si>
-    <t>4mm</t>
-  </si>
-  <si>
-    <t>(0.9 Power)</t>
-  </si>
-  <si>
-    <t>６</t>
-  </si>
-  <si>
     <t>甲板紙</t>
   </si>
   <si>
     <t>反轉cut, 鏡射</t>
+  </si>
+  <si>
+    <t>６</t>
   </si>
   <si>
     <t>1.5mm</t>
@@ -209,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -336,25 +336,13 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -363,42 +351,38 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -412,11 +396,24 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -432,6 +429,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -685,16 +685,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -708,7 +708,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -723,7 +723,7 @@
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B3" s="8">
         <v>2.0</v>
@@ -734,7 +734,7 @@
       <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="9">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -749,7 +749,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" s="8">
         <v>25.0</v>
@@ -760,7 +760,7 @@
       <c r="D4" s="8">
         <v>1.0</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="9"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -788,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="s">
-        <v>12</v>
+      <c r="A6" s="11" t="s">
+        <v>9</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>16</v>
+      <c r="B6" s="12" t="s">
+        <v>11</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="13"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -808,23 +808,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="s">
-        <v>8</v>
+      <c r="A7" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="12">
         <v>4.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="12">
         <v>10.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="12">
         <v>1.0</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="16">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,23 +834,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="s">
-        <v>10</v>
+      <c r="A8" s="15" t="s">
+        <v>8</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="12">
         <v>25.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="12">
         <v>5.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="12">
         <v>1.0</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="16">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="25"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="8"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="11"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="9"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +877,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
       <c r="D10" s="8"/>
-      <c r="E10" s="11"/>
+      <c r="E10" s="9"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -895,7 +895,7 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B11" s="8">
         <v>5.0</v>
@@ -906,11 +906,11 @@
       <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -921,7 +921,7 @@
     </row>
     <row r="12">
       <c r="A12" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B12" s="8">
         <v>5.0</v>
@@ -945,7 +945,7 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B13" s="8">
         <v>32.0</v>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="25"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -984,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="s">
-        <v>24</v>
+      <c r="A15" s="11" t="s">
+        <v>16</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="13"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1002,19 +1002,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="s">
-        <v>8</v>
+      <c r="A16" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="12">
         <v>5.0</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="12">
         <v>5.0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="12">
         <v>1.0</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="13"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,19 +1026,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="s">
-        <v>10</v>
+      <c r="A17" s="15" t="s">
+        <v>8</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="12">
         <v>50.0</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="12">
         <v>5.0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="12">
         <v>1.0</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="13"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="25"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1067,11 +1067,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1085,7 +1085,7 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B20" s="8">
         <v>5.0</v>
@@ -1109,11 +1109,11 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="25"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1142,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="s">
-        <v>26</v>
+      <c r="A23" s="11" t="s">
+        <v>19</v>
       </c>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="13"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1160,19 +1160,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="s">
-        <v>8</v>
+      <c r="A24" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="12">
         <v>5.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="12">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="12">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="13"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1184,17 +1184,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="s">
-        <v>10</v>
+      <c r="A25" s="23" t="s">
+        <v>8</v>
       </c>
-      <c r="B25" s="31">
+      <c r="B25" s="25">
         <v>55.0</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="25">
         <v>2.0</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="33"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="27"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="19"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1223,14 +1223,14 @@
     </row>
     <row r="27">
       <c r="A27" s="8" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="34">
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="28">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1245,7 +1245,7 @@
     </row>
     <row r="28">
       <c r="A28" s="8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B28" s="8">
         <v>2.0</v>
@@ -1253,8 +1253,8 @@
       <c r="C28" s="8">
         <v>100.0</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="34">
+      <c r="D28" s="19"/>
+      <c r="E28" s="28">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1269,7 +1269,7 @@
     </row>
     <row r="29">
       <c r="A29" s="8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B29" s="8">
         <v>20.0</v>
@@ -1277,8 +1277,8 @@
       <c r="C29" s="8">
         <v>100.0</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="34">
+      <c r="D29" s="19"/>
+      <c r="E29" s="28">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="19"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="A31" s="19"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17104,16 +17104,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17128,7 +17128,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="4"/>
@@ -17144,7 +17144,7 @@
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B3" s="8">
         <v>3.0</v>
@@ -17155,7 +17155,7 @@
       <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="14">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17171,7 +17171,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" s="8">
         <v>20.0</v>
@@ -17196,7 +17196,7 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -17215,7 +17215,7 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B6" s="8">
         <v>2.0</v>
@@ -17227,9 +17227,9 @@
         <v>1.0</v>
       </c>
       <c r="E6" s="10"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17240,7 +17240,7 @@
     </row>
     <row r="7">
       <c r="A7" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" s="8">
         <v>18.0</v>
@@ -17251,10 +17251,10 @@
       <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17268,7 +17268,7 @@
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
-      <c r="E8" s="12"/>
+      <c r="E8" s="14"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="s">
-        <v>12</v>
+      <c r="A9" s="11" t="s">
+        <v>9</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="22"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="21"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17300,19 +17300,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="s">
-        <v>8</v>
+      <c r="A10" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="12">
         <v>4.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="12">
         <v>15.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="12">
         <v>1.0</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="21">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,19 +17327,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="s">
-        <v>10</v>
+      <c r="A11" s="15" t="s">
+        <v>8</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="12">
         <v>25.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="12">
         <v>10.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="12">
         <v>1.0</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="21">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17354,19 +17354,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="s">
-        <v>20</v>
+      <c r="A12" s="15" t="s">
+        <v>18</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="12">
         <v>4.0</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="12">
         <v>10.0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="12">
         <v>1.0</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="21">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17381,13 +17381,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="s">
-        <v>13</v>
+      <c r="A13" s="15" t="s">
+        <v>12</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="26"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="24"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17400,19 +17400,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="s">
-        <v>8</v>
+      <c r="A14" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="12">
         <v>2.0</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="12">
         <v>18.0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="12">
         <v>1.0</v>
       </c>
-      <c r="E14" s="26"/>
+      <c r="E14" s="24"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,19 +17425,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="s">
-        <v>10</v>
+      <c r="A15" s="15" t="s">
+        <v>8</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="12">
         <v>18.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="12">
         <v>4.0</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="12">
         <v>1.0</v>
       </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="24"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,7 +17450,7 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="27"/>
+      <c r="A16" s="29"/>
       <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -17465,10 +17465,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
-      <c r="B17" s="28" t="s">
-        <v>13</v>
+      <c r="B17" s="30" t="s">
+        <v>12</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
@@ -17486,7 +17486,7 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B18" s="8">
         <v>5.0</v>
@@ -17511,7 +17511,7 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B19" s="8">
         <v>40.0</v>
@@ -17535,10 +17535,10 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="25"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
       <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
-        <v>24</v>
+      <c r="A21" s="11" t="s">
+        <v>16</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="26"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="24"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17571,19 +17571,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="s">
-        <v>8</v>
+      <c r="A22" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="12">
         <v>8.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="12">
         <v>15.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="12">
         <v>1.0</v>
       </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="24"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,19 +17596,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="s">
-        <v>10</v>
+      <c r="A23" s="15" t="s">
+        <v>8</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="12">
         <v>55.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="12">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="12">
         <v>2.0</v>
       </c>
-      <c r="E23" s="26"/>
+      <c r="E23" s="24"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,10 +17621,10 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="25"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
       <c r="E24" s="10"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -17639,11 +17639,11 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="10"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -17658,7 +17658,7 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B26" s="8">
         <v>10.0</v>
@@ -17683,7 +17683,7 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B27" s="8">
         <v>60.0</v>
@@ -17694,7 +17694,7 @@
       <c r="D27" s="8">
         <v>2.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="14">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,10 +17709,10 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="25"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
       <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="s">
-        <v>26</v>
+      <c r="A29" s="11" t="s">
+        <v>19</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="26"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="24"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17745,19 +17745,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="s">
-        <v>8</v>
+      <c r="A30" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="12">
         <v>18.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="12">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="12">
         <v>1.0</v>
       </c>
-      <c r="E30" s="26"/>
+      <c r="E30" s="24"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17770,16 +17770,16 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="s">
-        <v>10</v>
+      <c r="A31" s="23" t="s">
+        <v>8</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="25">
         <v>70.0</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="25">
         <v>5.0</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="25">
         <v>1.0</v>
       </c>
       <c r="E31" s="35"/>
@@ -17812,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" s="37">
+        <v>5.0</v>
+      </c>
+      <c r="C33" s="37">
+        <v>10.0</v>
+      </c>
+      <c r="D33" s="37">
+        <v>2.0</v>
+      </c>
+      <c r="E33" s="38">
+        <v>46043.55545597222</v>
+      </c>
+      <c r="F33" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B33" s="38">
-        <v>5.0</v>
-      </c>
-      <c r="C33" s="38">
-        <v>10.0</v>
-      </c>
-      <c r="D33" s="38">
-        <v>2.0</v>
-      </c>
-      <c r="E33" s="39">
-        <v>46043.55545597222</v>
-      </c>
-      <c r="F33" s="40" t="s">
-        <v>30</v>
-      </c>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="40"/>
+      <c r="M33" s="40"/>
+      <c r="N33" s="40"/>
+      <c r="O33" s="40"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17876,13 +17876,13 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17897,7 +17897,7 @@
     </row>
     <row r="37">
       <c r="A37" s="8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B37" s="8">
         <v>2.0</v>
@@ -17905,7 +17905,7 @@
       <c r="C37" s="8">
         <v>100.0</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="19"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17920,7 +17920,7 @@
     </row>
     <row r="38">
       <c r="A38" s="8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B38" s="8">
         <v>20.0</v>
@@ -17928,7 +17928,7 @@
       <c r="C38" s="8">
         <v>100.0</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34570,16 +34570,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34593,7 +34593,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -34608,7 +34608,7 @@
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B3" s="8">
         <v>2.0</v>
@@ -34619,7 +34619,7 @@
       <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="9">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34634,7 +34634,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B4" s="8">
         <v>10.0</v>
@@ -34645,7 +34645,7 @@
       <c r="D4" s="8">
         <v>2.0</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="9">
         <v>46232.916719409724</v>
       </c>
       <c r="F4" s="4"/>
@@ -34660,7 +34660,7 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5" s="8">
         <v>20.0</v>
@@ -34671,7 +34671,7 @@
       <c r="D5" s="8">
         <v>1.0</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="9">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34686,7 +34686,7 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="8">
         <v>2.0</v>
@@ -34697,7 +34697,7 @@
       <c r="D6" s="8">
         <v>1.0</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="9">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34727,15 +34727,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="s">
-        <v>12</v>
+      <c r="A8" s="11" t="s">
+        <v>9</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>16</v>
+      <c r="B8" s="12" t="s">
+        <v>11</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="17"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="13"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34747,23 +34747,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="s">
-        <v>8</v>
+      <c r="A9" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="12">
         <v>4.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="12">
         <v>10.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="12">
         <v>1.0</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="16">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34773,23 +34773,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="s">
-        <v>10</v>
+      <c r="A10" s="15" t="s">
+        <v>8</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="12">
         <v>20.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="12">
         <v>10.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="12">
         <v>1.0</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="16">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,11 +34799,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="25"/>
+      <c r="A11" s="18"/>
       <c r="B11" s="8"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="11"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="9"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34816,7 +34816,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34831,12 +34831,12 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
-      <c r="E13" s="11"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34849,7 +34849,7 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B14" s="8">
         <v>20.0</v>
@@ -34860,7 +34860,7 @@
       <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="9">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34875,12 +34875,12 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
-      <c r="E15" s="11"/>
+      <c r="E15" s="9"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34892,11 +34892,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="25"/>
+      <c r="A16" s="18"/>
       <c r="B16" s="8"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="11"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34909,12 +34909,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
       <c r="D17" s="8"/>
-      <c r="E17" s="11"/>
+      <c r="E17" s="9"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34927,7 +34927,7 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B18" s="8">
         <v>5.0</v>
@@ -34938,11 +34938,11 @@
       <c r="D18" s="8">
         <v>1.0</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34953,7 +34953,7 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B19" s="8">
         <v>5.0</v>
@@ -34977,7 +34977,7 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B20" s="8">
         <v>32.0</v>
@@ -35000,10 +35000,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="25"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35016,13 +35016,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="s">
-        <v>24</v>
+      <c r="A22" s="11" t="s">
+        <v>16</v>
       </c>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="17"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="13"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35034,19 +35034,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="s">
-        <v>8</v>
+      <c r="A23" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="12">
         <v>5.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="12">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="12">
         <v>1.0</v>
       </c>
-      <c r="E23" s="17"/>
+      <c r="E23" s="13"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35058,19 +35058,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="s">
-        <v>10</v>
+      <c r="A24" s="15" t="s">
+        <v>8</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="12">
         <v>50.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="12">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="12">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="13"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,10 +35082,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="25"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35099,11 +35099,11 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35117,7 +35117,7 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B27" s="8">
         <v>5.0</v>
@@ -35141,11 +35141,11 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35158,10 +35158,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="25"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35174,13 +35174,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="s">
-        <v>26</v>
+      <c r="A30" s="11" t="s">
+        <v>19</v>
       </c>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="17"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35192,19 +35192,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="s">
-        <v>8</v>
+      <c r="A31" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="12">
         <v>5.0</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="12">
         <v>5.0</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="12">
         <v>1.0</v>
       </c>
-      <c r="E31" s="17"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35216,17 +35216,17 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="30" t="s">
-        <v>10</v>
+      <c r="A32" s="23" t="s">
+        <v>8</v>
       </c>
-      <c r="B32" s="31">
+      <c r="B32" s="25">
         <v>55.0</v>
       </c>
-      <c r="C32" s="31">
+      <c r="C32" s="25">
         <v>2.0</v>
       </c>
-      <c r="D32" s="32"/>
-      <c r="E32" s="33"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="27"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
+      <c r="A33" s="19"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35255,14 +35255,14 @@
     </row>
     <row r="34">
       <c r="A34" s="8" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="34">
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="28">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35277,7 +35277,7 @@
     </row>
     <row r="35">
       <c r="A35" s="8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B35" s="8">
         <v>2.0</v>
@@ -35285,8 +35285,8 @@
       <c r="C35" s="8">
         <v>100.0</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="34">
+      <c r="D35" s="19"/>
+      <c r="E35" s="28">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35301,7 +35301,7 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B36" s="8">
         <v>20.0</v>
@@ -35309,8 +35309,8 @@
       <c r="C36" s="8">
         <v>100.0</v>
       </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="34">
+      <c r="D36" s="19"/>
+      <c r="E36" s="28">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="A37" s="19"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="19"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="13"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
+      <c r="A38" s="19"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,19 +51132,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51157,10 +51157,10 @@
     </row>
     <row r="2">
       <c r="A2" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
       <c r="D2" s="8"/>
       <c r="E2" s="10"/>
       <c r="F2" s="4"/>
@@ -51174,12 +51174,12 @@
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="22">
         <v>60.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="22">
         <v>20.0</v>
       </c>
       <c r="D3" s="8">
@@ -51197,9 +51197,9 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
       <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -51212,14 +51212,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="14"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51231,7 +51231,7 @@
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B6" s="8">
         <v>6.0</v>
@@ -51240,7 +51240,7 @@
         <v>100.0</v>
       </c>
       <c r="D6" s="8"/>
-      <c r="E6" s="12">
+      <c r="E6" s="14">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51254,7 +51254,7 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B7" s="8">
         <v>8.0</v>
@@ -51265,7 +51265,7 @@
       <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="14">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51279,9 +51279,9 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="5"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
       <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -51294,7 +51294,7 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -51311,7 +51311,7 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10" s="8">
         <v>10.0</v>
@@ -51322,7 +51322,7 @@
       <c r="D10" s="8">
         <v>1.0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="14">
         <v>46106.73232292824</v>
       </c>
       <c r="F10" s="4"/>
@@ -51336,7 +51336,7 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B11" s="8">
         <v>11.0</v>
@@ -51347,7 +51347,7 @@
       <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="14">
         <v>46106.732369062505</v>
       </c>
       <c r="F11" s="4"/>
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="20"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="32"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,15 +51375,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="s">
-        <v>18</v>
+      <c r="A13" s="33" t="s">
+        <v>24</v>
       </c>
-      <c r="B13" s="24" t="s">
-        <v>19</v>
+      <c r="B13" s="34" t="s">
+        <v>25</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
-      <c r="E13" s="12"/>
+      <c r="E13" s="14"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51395,7 +51395,7 @@
     </row>
     <row r="14" ht="20.25" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B14" s="8">
         <v>5.0</v>
@@ -51406,7 +51406,7 @@
       <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="14">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51420,7 +51420,7 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B15" s="8">
         <v>5.0</v>
@@ -51431,7 +51431,7 @@
       <c r="D15" s="8">
         <v>1.0</v>
       </c>
-      <c r="E15" s="12"/>
+      <c r="E15" s="14"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51443,7 +51443,7 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B16" s="8">
         <v>5.0</v>
@@ -51454,11 +51454,11 @@
       <c r="D16" s="8">
         <v>4.0</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="14">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="15" t="s">
-        <v>23</v>
+      <c r="F16" s="17" t="s">
+        <v>27</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51470,7 +51470,7 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B17" s="8">
         <v>12.0</v>
@@ -51481,7 +51481,7 @@
       <c r="D17" s="8">
         <v>1.0</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="14">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="20"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="32"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,11 +51510,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
       <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -51527,18 +51527,18 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="22">
         <v>6.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="22">
         <v>45.0</v>
       </c>
       <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="14">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51552,18 +51552,18 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
-      <c r="B21" s="9">
+      <c r="B21" s="22">
         <v>18.0</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="22">
         <v>20.0</v>
       </c>
       <c r="D21" s="8">
         <v>1.0</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="14">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51577,9 +51577,9 @@
     </row>
     <row r="22">
       <c r="A22" s="7"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
       <c r="E22" s="10"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -51591,15 +51591,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="s">
-        <v>12</v>
+      <c r="A23" s="33" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="24" t="s">
-        <v>19</v>
+      <c r="B23" s="34" t="s">
+        <v>25</v>
       </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="12">
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="14">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51613,18 +51613,18 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="22">
         <v>6.0</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="22">
         <v>50.0</v>
       </c>
       <c r="D24" s="8">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="14">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51638,18 +51638,18 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="22">
         <v>8.0</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="22">
         <v>30.0</v>
       </c>
       <c r="D25" s="8">
         <v>1.0</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="14">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51663,22 +51663,22 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="22">
         <v>10.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="22">
         <v>30.0</v>
       </c>
       <c r="D26" s="8">
         <v>4.0</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="14">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="15" t="s">
-        <v>23</v>
+      <c r="F26" s="17" t="s">
+        <v>27</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51690,18 +51690,18 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="22">
         <v>17.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="22">
         <v>15.0</v>
       </c>
       <c r="D27" s="8">
         <v>1.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="14">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51715,9 +51715,9 @@
     </row>
     <row r="28">
       <c r="A28" s="7"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
       <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -51729,14 +51729,14 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="s">
-        <v>21</v>
+      <c r="A29" s="33" t="s">
+        <v>13</v>
       </c>
-      <c r="B29" s="24" t="s">
-        <v>19</v>
+      <c r="B29" s="34" t="s">
+        <v>25</v>
       </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
       <c r="E29" s="10"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -51749,18 +51749,18 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="22">
         <v>6.0</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="22">
         <v>50.0</v>
       </c>
       <c r="D30" s="8">
         <v>1.0</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="14">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51774,12 +51774,12 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="22">
         <v>8.0</v>
       </c>
-      <c r="C31" s="9">
+      <c r="C31" s="22">
         <v>30.0</v>
       </c>
       <c r="D31" s="8">
@@ -51797,18 +51797,18 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="22">
         <v>15.0</v>
       </c>
-      <c r="C32" s="9">
+      <c r="C32" s="22">
         <v>10.0</v>
       </c>
       <c r="D32" s="8">
         <v>2.0</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="14">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51822,9 +51822,9 @@
     </row>
     <row r="33">
       <c r="A33" s="7"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
       <c r="E33" s="10"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51836,13 +51836,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="s">
-        <v>21</v>
+      <c r="A34" s="11" t="s">
+        <v>13</v>
       </c>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="26"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="24"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51853,19 +51853,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="s">
-        <v>8</v>
+      <c r="A35" s="15" t="s">
+        <v>6</v>
       </c>
-      <c r="B35" s="36" t="s">
-        <v>28</v>
+      <c r="B35" s="41" t="s">
+        <v>30</v>
       </c>
-      <c r="C35" s="36">
+      <c r="C35" s="41">
         <v>40.0</v>
       </c>
-      <c r="D35" s="36">
+      <c r="D35" s="41">
         <v>1.0</v>
       </c>
-      <c r="E35" s="22">
+      <c r="E35" s="21">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51878,19 +51878,19 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="s">
-        <v>10</v>
+      <c r="A36" s="15" t="s">
+        <v>8</v>
       </c>
-      <c r="B36" s="36">
+      <c r="B36" s="41">
         <v>30.0</v>
       </c>
-      <c r="C36" s="36">
+      <c r="C36" s="41">
         <v>15.0</v>
       </c>
-      <c r="D36" s="36">
+      <c r="D36" s="41">
         <v>1.0</v>
       </c>
-      <c r="E36" s="26"/>
+      <c r="E36" s="24"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51902,7 +51902,7 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B37" s="8">
         <v>10.0</v>
@@ -51913,7 +51913,7 @@
       <c r="D37" s="8">
         <v>1.0</v>
       </c>
-      <c r="E37" s="12">
+      <c r="E37" s="14">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51926,10 +51926,10 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="25"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="10"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51944,9 +51944,9 @@
       <c r="A39" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
       <c r="E39" s="10"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -51959,7 +51959,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B40" s="8">
         <v>40.0</v>
@@ -51970,7 +51970,7 @@
       <c r="D40" s="8">
         <v>1.0</v>
       </c>
-      <c r="E40" s="12">
+      <c r="E40" s="14">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51984,9 +51984,9 @@
     </row>
     <row r="41">
       <c r="A41" s="5"/>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
+      <c r="B41" s="19"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
       <c r="E41" s="10"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -51999,11 +51999,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
+      <c r="B42" s="19"/>
+      <c r="C42" s="19"/>
+      <c r="D42" s="19"/>
       <c r="E42" s="10"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -52016,7 +52016,7 @@
     </row>
     <row r="43">
       <c r="A43" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B43" s="8">
         <v>9.0</v>
@@ -52027,7 +52027,7 @@
       <c r="D43" s="8">
         <v>1.0</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="14">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52041,7 +52041,7 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B44" s="8">
         <v>55.0</v>
@@ -52052,7 +52052,7 @@
       <c r="D44" s="8">
         <v>1.0</v>
       </c>
-      <c r="E44" s="12">
+      <c r="E44" s="14">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52066,7 +52066,7 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B45" s="8">
         <v>10.0</v>
@@ -52077,10 +52077,10 @@
       <c r="D45" s="8">
         <v>1.0</v>
       </c>
-      <c r="E45" s="12">
+      <c r="E45" s="14">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="15" t="s">
+      <c r="F45" s="17" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52093,9 +52093,9 @@
     </row>
     <row r="46">
       <c r="A46" s="42"/>
-      <c r="B46" s="13"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
+      <c r="B46" s="19"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
       <c r="E46" s="10"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -52108,11 +52108,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
       <c r="E47" s="10"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -52125,7 +52125,7 @@
     </row>
     <row r="48">
       <c r="A48" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B48" s="8">
         <v>55.0</v>
@@ -52136,7 +52136,7 @@
       <c r="D48" s="8">
         <v>1.0</v>
       </c>
-      <c r="E48" s="12">
+      <c r="E48" s="14">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52150,9 +52150,9 @@
     </row>
     <row r="49">
       <c r="A49" s="42"/>
-      <c r="B49" s="13"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
       <c r="E49" s="10"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
@@ -52165,11 +52165,11 @@
     </row>
     <row r="50">
       <c r="A50" s="42" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
-      <c r="B50" s="13"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
       <c r="E50" s="10"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52182,7 +52182,7 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B51" s="8">
         <v>60.0</v>
@@ -52193,7 +52193,7 @@
       <c r="D51" s="8">
         <v>1.0</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="14">
         <v>46203.63265940972</v>
       </c>
       <c r="F51" s="4"/>
@@ -52207,7 +52207,7 @@
     </row>
     <row r="52">
       <c r="A52" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B52" s="8">
         <v>10.0</v>
@@ -52215,9 +52215,11 @@
       <c r="C52" s="8">
         <v>50.0</v>
       </c>
-      <c r="D52" s="13"/>
-      <c r="E52" s="12">
-        <v>46253.61147633102</v>
+      <c r="D52" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E52" s="14">
+        <v>46253.61151159722</v>
       </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -52230,9 +52232,9 @@
     </row>
     <row r="53">
       <c r="A53" s="42"/>
-      <c r="B53" s="13"/>
-      <c r="C53" s="13"/>
-      <c r="D53" s="13"/>
+      <c r="B53" s="19"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="19"/>
       <c r="E53" s="10"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52247,9 +52249,9 @@
       <c r="A54" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
       <c r="E54" s="10"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
@@ -52262,18 +52264,18 @@
     </row>
     <row r="55">
       <c r="A55" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
-      <c r="B55" s="9">
+      <c r="B55" s="22">
         <v>70.0</v>
       </c>
-      <c r="C55" s="9">
+      <c r="C55" s="22">
         <v>300.0</v>
       </c>
-      <c r="D55" s="9">
+      <c r="D55" s="22">
         <v>1.0</v>
       </c>
-      <c r="E55" s="12">
+      <c r="E55" s="14">
         <v>46223.80899857639</v>
       </c>
       <c r="F55" s="4"/>
@@ -52287,18 +52289,18 @@
     </row>
     <row r="56">
       <c r="A56" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
-      <c r="B56" s="9">
+      <c r="B56" s="22">
         <v>10.0</v>
       </c>
-      <c r="C56" s="9">
+      <c r="C56" s="22">
         <v>20.0</v>
       </c>
-      <c r="D56" s="9">
+      <c r="D56" s="22">
         <v>1.0</v>
       </c>
-      <c r="E56" s="12">
+      <c r="E56" s="14">
         <v>46223.80911148148</v>
       </c>
       <c r="F56" s="4"/>
@@ -52312,18 +52314,18 @@
     </row>
     <row r="57">
       <c r="A57" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
-      <c r="B57" s="9">
+      <c r="B57" s="22">
         <v>70.0</v>
       </c>
-      <c r="C57" s="9">
+      <c r="C57" s="22">
         <v>10.0</v>
       </c>
-      <c r="D57" s="9">
+      <c r="D57" s="22">
         <v>1.0</v>
       </c>
-      <c r="E57" s="12">
+      <c r="E57" s="14">
         <v>46207.72572512731</v>
       </c>
       <c r="F57" s="4"/>
@@ -52359,7 +52361,7 @@
       </c>
       <c r="C59" s="8"/>
       <c r="D59" s="8"/>
-      <c r="E59" s="12">
+      <c r="E59" s="14">
         <v>45946.87875708334</v>
       </c>
       <c r="F59" s="4"/>
@@ -52378,9 +52380,9 @@
       <c r="B60" s="8">
         <v>100.0</v>
       </c>
-      <c r="C60" s="13"/>
-      <c r="D60" s="13"/>
-      <c r="E60" s="12">
+      <c r="C60" s="19"/>
+      <c r="D60" s="19"/>
+      <c r="E60" s="14">
         <v>45946.87887299768</v>
       </c>
       <c r="F60" s="4"/>
@@ -52410,16 +52412,16 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="40" t="s">
+      <c r="A62" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="B62" s="40">
+      <c r="B62" s="39">
         <v>100.0</v>
       </c>
-      <c r="C62" s="15">
+      <c r="C62" s="17">
         <v>1.0</v>
       </c>
-      <c r="D62" s="15">
+      <c r="D62" s="17">
         <v>2.0</v>
       </c>
       <c r="E62" s="46">
@@ -52435,8 +52437,8 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="41"/>
-      <c r="B63" s="41"/>
+      <c r="A63" s="40"/>
+      <c r="B63" s="40"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
@@ -52450,10 +52452,10 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="40" t="s">
+      <c r="A64" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="B64" s="41"/>
+      <c r="B64" s="40"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
@@ -52468,15 +52470,15 @@
     </row>
     <row r="65">
       <c r="A65" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
-      <c r="B65" s="40">
+      <c r="B65" s="39">
         <v>50.0</v>
       </c>
-      <c r="C65" s="15">
+      <c r="C65" s="17">
         <v>20.0</v>
       </c>
-      <c r="D65" s="15">
+      <c r="D65" s="17">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52492,13 +52494,13 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="40" t="s">
+      <c r="A66" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B66" s="40">
+      <c r="B66" s="39">
         <v>15.0</v>
       </c>
-      <c r="C66" s="15">
+      <c r="C66" s="17">
         <v>16.0</v>
       </c>
       <c r="D66" s="4"/>
@@ -52515,8 +52517,8 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="41"/>
-      <c r="B67" s="41"/>
+      <c r="A67" s="40"/>
+      <c r="B67" s="40"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
@@ -52530,11 +52532,11 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="40" t="s">
+      <c r="A68" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="40" t="s">
-        <v>25</v>
+      <c r="B68" s="39" t="s">
+        <v>17</v>
       </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -52551,16 +52553,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="40" t="s">
+      <c r="A69" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="40">
+      <c r="B69" s="39">
         <v>5.0</v>
       </c>
-      <c r="C69" s="15">
+      <c r="C69" s="17">
         <v>80.0</v>
       </c>
-      <c r="D69" s="15">
+      <c r="D69" s="17">
         <v>1.0</v>
       </c>
       <c r="E69" s="46">
@@ -52576,16 +52578,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="40" t="s">
+      <c r="A70" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="B70" s="40">
+      <c r="B70" s="39">
         <v>15.0</v>
       </c>
-      <c r="C70" s="15">
+      <c r="C70" s="17">
         <v>10.0</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="17">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52601,16 +52603,16 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="40" t="s">
-        <v>17</v>
+      <c r="A71" s="39" t="s">
+        <v>22</v>
       </c>
-      <c r="B71" s="40">
+      <c r="B71" s="39">
         <v>30.0</v>
       </c>
-      <c r="C71" s="15">
+      <c r="C71" s="17">
         <v>10.0</v>
       </c>
-      <c r="D71" s="15">
+      <c r="D71" s="17">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52626,8 +52628,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="41"/>
-      <c r="B72" s="41"/>
+      <c r="A72" s="40"/>
+      <c r="B72" s="40"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52641,10 +52643,10 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="40" t="s">
+      <c r="A73" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="B73" s="40" t="s">
+      <c r="B73" s="39" t="s">
         <v>33</v>
       </c>
       <c r="C73" s="4"/>
@@ -52662,16 +52664,16 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="40" t="s">
+      <c r="A74" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="B74" s="40">
+      <c r="B74" s="39">
         <v>5.0</v>
       </c>
-      <c r="C74" s="15">
+      <c r="C74" s="17">
         <v>80.0</v>
       </c>
-      <c r="D74" s="15">
+      <c r="D74" s="17">
         <v>1.0</v>
       </c>
       <c r="E74" s="4"/>
@@ -52685,16 +52687,16 @@
       <c r="M74" s="4"/>
     </row>
     <row r="75">
-      <c r="A75" s="40" t="s">
+      <c r="A75" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="B75" s="40">
+      <c r="B75" s="39">
         <v>15.0</v>
       </c>
-      <c r="C75" s="15">
+      <c r="C75" s="17">
         <v>10.0</v>
       </c>
-      <c r="D75" s="15">
+      <c r="D75" s="17">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52708,16 +52710,16 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76">
-      <c r="A76" s="40" t="s">
-        <v>17</v>
+      <c r="A76" s="39" t="s">
+        <v>22</v>
       </c>
-      <c r="B76" s="40">
+      <c r="B76" s="39">
         <v>20.0</v>
       </c>
-      <c r="C76" s="15">
+      <c r="C76" s="17">
         <v>10.0</v>
       </c>
-      <c r="D76" s="15">
+      <c r="D76" s="17">
         <v>6.0</v>
       </c>
       <c r="E76" s="46">
@@ -52733,8 +52735,8 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="41"/>
-      <c r="B77" s="41"/>
+      <c r="A77" s="40"/>
+      <c r="B77" s="40"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
@@ -52748,8 +52750,8 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="40"/>
-      <c r="B78" s="41"/>
+      <c r="A78" s="39"/>
+      <c r="B78" s="40"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
@@ -52763,8 +52765,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="41"/>
-      <c r="B79" s="41"/>
+      <c r="A79" s="40"/>
+      <c r="B79" s="40"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-08-26T10:12:28.664Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -37,34 +37,46 @@
     <t>Line</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
-  </si>
-  <si>
-    <t>Cut-1/2</t>
-  </si>
-  <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
-    <t>(PS)</t>
-  </si>
-  <si>
-    <t>1mm</t>
-  </si>
-  <si>
     <t>遮蓋膠紙</t>
   </si>
   <si>
     <t>刀壓</t>
   </si>
   <si>
+    <t>Cut-1/2</t>
+  </si>
+  <si>
+    <t>Cut(detail)</t>
+  </si>
+  <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
+    <t>(PS)</t>
+  </si>
+  <si>
+    <t>A4紙</t>
+  </si>
+  <si>
+    <t>1mm</t>
+  </si>
+  <si>
+    <t>03mm</t>
+  </si>
+  <si>
+    <t>Cut</t>
+  </si>
+  <si>
     <t>2mm</t>
+  </si>
+  <si>
+    <t>0.3 mm</t>
   </si>
   <si>
     <t>3mm</t>
@@ -73,25 +85,10 @@
     <t>Fill</t>
   </si>
   <si>
-    <t>4mm</t>
+    <t>PS</t>
   </si>
   <si>
-    <t>A4紙</t>
-  </si>
-  <si>
-    <t>03mm</t>
-  </si>
-  <si>
-    <t>Cut</t>
-  </si>
-  <si>
-    <t>(0.9 Power)</t>
-  </si>
-  <si>
-    <t>0.3 mm</t>
-  </si>
-  <si>
-    <t>PS</t>
+    <t>4mm</t>
   </si>
   <si>
     <t>cut</t>
@@ -100,13 +97,16 @@
     <t>Keep Detail</t>
   </si>
   <si>
+    <t>(0.9 Power)</t>
+  </si>
+  <si>
+    <t>６</t>
+  </si>
+  <si>
     <t>甲板紙</t>
   </si>
   <si>
     <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>６</t>
   </si>
   <si>
     <t>1.5mm</t>
@@ -209,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -342,62 +342,40 @@
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -406,14 +384,39 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -429,9 +432,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -749,7 +749,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" s="8">
         <v>25.0</v>
@@ -788,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="12" t="s">
+      <c r="A6" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="13"/>
+      <c r="B6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="15"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -808,23 +808,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="14">
         <v>4.0</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="14">
         <v>10.0</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="14">
         <v>1.0</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="17">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,23 +834,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="s">
-        <v>8</v>
+      <c r="A8" s="16" t="s">
+        <v>9</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="14">
         <v>25.0</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="14">
         <v>5.0</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="14">
         <v>1.0</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="17">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,7 +860,7 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="18"/>
+      <c r="A9" s="20"/>
       <c r="B9" s="8"/>
       <c r="C9" s="19"/>
       <c r="D9" s="19"/>
@@ -877,7 +877,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
@@ -909,8 +909,8 @@
       <c r="E11" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -945,7 +945,7 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B13" s="8">
         <v>32.0</v>
@@ -968,7 +968,7 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="18"/>
+      <c r="A14" s="20"/>
       <c r="B14" s="19"/>
       <c r="C14" s="19"/>
       <c r="D14" s="19"/>
@@ -984,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="s">
-        <v>16</v>
+      <c r="A15" s="13" t="s">
+        <v>19</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="13"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="15"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1002,19 +1002,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="14">
         <v>5.0</v>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="14">
         <v>5.0</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="14">
         <v>1.0</v>
       </c>
-      <c r="E16" s="13"/>
+      <c r="E16" s="15"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,19 +1026,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="s">
-        <v>8</v>
+      <c r="A17" s="16" t="s">
+        <v>9</v>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="14">
         <v>50.0</v>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="14">
         <v>5.0</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="14">
         <v>1.0</v>
       </c>
-      <c r="E17" s="13"/>
+      <c r="E17" s="15"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,7 +1050,7 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="18"/>
+      <c r="A18" s="20"/>
       <c r="B18" s="19"/>
       <c r="C18" s="19"/>
       <c r="D18" s="19"/>
@@ -1067,7 +1067,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
@@ -1109,7 +1109,7 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -1126,7 +1126,7 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18"/>
+      <c r="A22" s="20"/>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
       <c r="D22" s="19"/>
@@ -1142,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="s">
-        <v>19</v>
+      <c r="A23" s="13" t="s">
+        <v>24</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="13"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="15"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1160,19 +1160,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="14">
         <v>5.0</v>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="14">
         <v>5.0</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="14">
         <v>1.0</v>
       </c>
-      <c r="E24" s="13"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1184,17 +1184,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="s">
-        <v>8</v>
+      <c r="A25" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B25" s="25">
+      <c r="B25" s="31">
         <v>55.0</v>
       </c>
-      <c r="C25" s="25">
+      <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="26"/>
-      <c r="E25" s="27"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1223,14 +1223,14 @@
     </row>
     <row r="27">
       <c r="A27" s="8" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="19"/>
-      <c r="E27" s="28">
+      <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1254,7 +1254,7 @@
         <v>100.0</v>
       </c>
       <c r="D28" s="19"/>
-      <c r="E28" s="28">
+      <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1269,7 +1269,7 @@
     </row>
     <row r="29">
       <c r="A29" s="8" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B29" s="8">
         <v>20.0</v>
@@ -1278,7 +1278,7 @@
         <v>100.0</v>
       </c>
       <c r="D29" s="19"/>
-      <c r="E29" s="28">
+      <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -17155,7 +17155,7 @@
       <c r="D3" s="8">
         <v>1.0</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="12">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17171,7 +17171,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" s="8">
         <v>20.0</v>
@@ -17196,7 +17196,7 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -17227,9 +17227,9 @@
         <v>1.0</v>
       </c>
       <c r="E6" s="10"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17240,7 +17240,7 @@
     </row>
     <row r="7">
       <c r="A7" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" s="8">
         <v>18.0</v>
@@ -17251,10 +17251,10 @@
       <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17268,7 +17268,7 @@
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
-      <c r="E8" s="14"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="s">
-        <v>9</v>
+      <c r="A9" s="13" t="s">
+        <v>11</v>
       </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="21"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="22"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17300,19 +17300,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="14">
         <v>4.0</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="14">
         <v>15.0</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="14">
         <v>1.0</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="22">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,19 +17327,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="s">
-        <v>8</v>
+      <c r="A11" s="16" t="s">
+        <v>9</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="14">
         <v>25.0</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="14">
         <v>10.0</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="14">
         <v>1.0</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="22">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17354,19 +17354,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="s">
-        <v>18</v>
+      <c r="A12" s="16" t="s">
+        <v>22</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="14">
         <v>4.0</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="14">
         <v>10.0</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="14">
         <v>1.0</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="22">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17381,13 +17381,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="s">
-        <v>12</v>
+      <c r="A13" s="16" t="s">
+        <v>14</v>
       </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="24"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17400,19 +17400,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="14">
         <v>2.0</v>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="14">
         <v>18.0</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="14">
         <v>1.0</v>
       </c>
-      <c r="E14" s="24"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,19 +17425,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
-        <v>8</v>
+      <c r="A15" s="16" t="s">
+        <v>9</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="14">
         <v>18.0</v>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="14">
         <v>4.0</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="14">
         <v>1.0</v>
       </c>
-      <c r="E15" s="24"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,7 +17450,7 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="29"/>
+      <c r="A16" s="28"/>
       <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -17465,10 +17465,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
-      <c r="B17" s="30" t="s">
-        <v>12</v>
+      <c r="B17" s="29" t="s">
+        <v>14</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
@@ -17511,7 +17511,7 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19" s="8">
         <v>40.0</v>
@@ -17535,7 +17535,7 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="18"/>
+      <c r="A20" s="20"/>
       <c r="B20" s="19"/>
       <c r="C20" s="19"/>
       <c r="D20" s="19"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="s">
-        <v>16</v>
+      <c r="A21" s="13" t="s">
+        <v>19</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="24"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17571,19 +17571,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="14">
         <v>8.0</v>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="14">
         <v>15.0</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="14">
         <v>1.0</v>
       </c>
-      <c r="E22" s="24"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,19 +17596,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
-        <v>8</v>
+      <c r="A23" s="16" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="14">
         <v>55.0</v>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="14">
         <v>5.0</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="14">
         <v>2.0</v>
       </c>
-      <c r="E23" s="24"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,7 +17621,7 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18"/>
+      <c r="A24" s="20"/>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
       <c r="D24" s="19"/>
@@ -17639,7 +17639,7 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B25" s="19"/>
       <c r="C25" s="19"/>
@@ -17683,7 +17683,7 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B27" s="8">
         <v>60.0</v>
@@ -17694,7 +17694,7 @@
       <c r="D27" s="8">
         <v>2.0</v>
       </c>
-      <c r="E27" s="14">
+      <c r="E27" s="12">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,7 +17709,7 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="18"/>
+      <c r="A28" s="20"/>
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
       <c r="D28" s="19"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="s">
-        <v>19</v>
+      <c r="A29" s="13" t="s">
+        <v>24</v>
       </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="24"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17745,19 +17745,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="14">
         <v>18.0</v>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="14">
         <v>5.0</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="14">
         <v>1.0</v>
       </c>
-      <c r="E30" s="24"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17770,16 +17770,16 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="s">
-        <v>8</v>
+      <c r="A31" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="25">
+      <c r="B31" s="31">
         <v>70.0</v>
       </c>
-      <c r="C31" s="25">
+      <c r="C31" s="31">
         <v>5.0</v>
       </c>
-      <c r="D31" s="25">
+      <c r="D31" s="31">
         <v>1.0</v>
       </c>
       <c r="E31" s="35"/>
@@ -17812,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="36" t="s">
-        <v>28</v>
+      <c r="A33" s="37" t="s">
+        <v>29</v>
       </c>
-      <c r="B33" s="37">
+      <c r="B33" s="38">
         <v>5.0</v>
       </c>
-      <c r="C33" s="37">
+      <c r="C33" s="38">
         <v>10.0</v>
       </c>
-      <c r="D33" s="37">
+      <c r="D33" s="38">
         <v>2.0</v>
       </c>
-      <c r="E33" s="38">
+      <c r="E33" s="39">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="39" t="s">
-        <v>29</v>
+      <c r="F33" s="40" t="s">
+        <v>30</v>
       </c>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="40"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="40"/>
-      <c r="N33" s="40"/>
-      <c r="O33" s="40"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17876,10 +17876,10 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C36" s="19"/>
       <c r="D36" s="19"/>
@@ -17920,7 +17920,7 @@
     </row>
     <row r="38">
       <c r="A38" s="8" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B38" s="8">
         <v>20.0</v>
@@ -34634,7 +34634,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B4" s="8">
         <v>10.0</v>
@@ -34660,7 +34660,7 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="8">
         <v>20.0</v>
@@ -34686,7 +34686,7 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6" s="8">
         <v>2.0</v>
@@ -34727,15 +34727,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="12" t="s">
+      <c r="A8" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="13"/>
+      <c r="B8" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="15"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34747,23 +34747,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="14">
         <v>4.0</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="14">
         <v>10.0</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="14">
         <v>1.0</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="17">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34773,23 +34773,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="s">
-        <v>8</v>
+      <c r="A10" s="16" t="s">
+        <v>9</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="14">
         <v>20.0</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="14">
         <v>10.0</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="14">
         <v>1.0</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="17">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,7 +34799,7 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="18"/>
+      <c r="A11" s="20"/>
       <c r="B11" s="8"/>
       <c r="C11" s="19"/>
       <c r="D11" s="19"/>
@@ -34816,7 +34816,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34849,7 +34849,7 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" s="8">
         <v>20.0</v>
@@ -34875,7 +34875,7 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -34892,7 +34892,7 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="18"/>
+      <c r="A16" s="20"/>
       <c r="B16" s="8"/>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -34909,7 +34909,7 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -34941,8 +34941,8 @@
       <c r="E18" s="9">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34977,7 +34977,7 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20" s="8">
         <v>32.0</v>
@@ -35000,7 +35000,7 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="18"/>
+      <c r="A21" s="20"/>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
       <c r="D21" s="19"/>
@@ -35016,13 +35016,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="s">
-        <v>16</v>
+      <c r="A22" s="13" t="s">
+        <v>19</v>
       </c>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="13"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="15"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35034,19 +35034,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="14">
         <v>5.0</v>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="14">
         <v>5.0</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="14">
         <v>1.0</v>
       </c>
-      <c r="E23" s="13"/>
+      <c r="E23" s="15"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35058,19 +35058,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="s">
-        <v>8</v>
+      <c r="A24" s="16" t="s">
+        <v>9</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="14">
         <v>50.0</v>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="14">
         <v>5.0</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="14">
         <v>1.0</v>
       </c>
-      <c r="E24" s="13"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,7 +35082,7 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="18"/>
+      <c r="A25" s="20"/>
       <c r="B25" s="19"/>
       <c r="C25" s="19"/>
       <c r="D25" s="19"/>
@@ -35099,7 +35099,7 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B26" s="19"/>
       <c r="C26" s="19"/>
@@ -35141,7 +35141,7 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
@@ -35158,7 +35158,7 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="18"/>
+      <c r="A29" s="20"/>
       <c r="B29" s="19"/>
       <c r="C29" s="19"/>
       <c r="D29" s="19"/>
@@ -35174,13 +35174,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="s">
-        <v>19</v>
+      <c r="A30" s="13" t="s">
+        <v>24</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="13"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="15"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35192,19 +35192,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="s">
+      <c r="A31" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="14">
         <v>5.0</v>
       </c>
-      <c r="C31" s="12">
+      <c r="C31" s="14">
         <v>5.0</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="14">
         <v>1.0</v>
       </c>
-      <c r="E31" s="13"/>
+      <c r="E31" s="15"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35216,17 +35216,17 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="s">
-        <v>8</v>
+      <c r="A32" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B32" s="25">
+      <c r="B32" s="31">
         <v>55.0</v>
       </c>
-      <c r="C32" s="25">
+      <c r="C32" s="31">
         <v>2.0</v>
       </c>
-      <c r="D32" s="26"/>
-      <c r="E32" s="27"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="33"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35255,14 +35255,14 @@
     </row>
     <row r="34">
       <c r="A34" s="8" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
-      <c r="E34" s="28">
+      <c r="E34" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35286,7 +35286,7 @@
         <v>100.0</v>
       </c>
       <c r="D35" s="19"/>
-      <c r="E35" s="28">
+      <c r="E35" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35301,7 +35301,7 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B36" s="8">
         <v>20.0</v>
@@ -35310,7 +35310,7 @@
         <v>100.0</v>
       </c>
       <c r="D36" s="19"/>
-      <c r="E36" s="28">
+      <c r="E36" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -51132,10 +51132,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -51159,8 +51159,8 @@
       <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
       <c r="D2" s="8"/>
       <c r="E2" s="10"/>
       <c r="F2" s="4"/>
@@ -51174,12 +51174,12 @@
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="11">
         <v>60.0</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="11">
         <v>20.0</v>
       </c>
       <c r="D3" s="8">
@@ -51212,14 +51212,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C5" s="19"/>
       <c r="D5" s="19"/>
-      <c r="E5" s="14"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51240,7 +51240,7 @@
         <v>100.0</v>
       </c>
       <c r="D6" s="8"/>
-      <c r="E6" s="14">
+      <c r="E6" s="12">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51254,7 +51254,7 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B7" s="8">
         <v>8.0</v>
@@ -51265,7 +51265,7 @@
       <c r="D7" s="8">
         <v>1.0</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="12">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51294,7 +51294,7 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -51322,7 +51322,7 @@
       <c r="D10" s="8">
         <v>1.0</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="12">
         <v>46106.73232292824</v>
       </c>
       <c r="F10" s="4"/>
@@ -51336,7 +51336,7 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B11" s="8">
         <v>11.0</v>
@@ -51347,7 +51347,7 @@
       <c r="D11" s="8">
         <v>1.0</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="12">
         <v>46106.732369062505</v>
       </c>
       <c r="F11" s="4"/>
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="31"/>
-      <c r="D12" s="31"/>
-      <c r="E12" s="32"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="24"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,15 +51375,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="s">
-        <v>24</v>
+      <c r="A13" s="25" t="s">
+        <v>20</v>
       </c>
-      <c r="B13" s="34" t="s">
-        <v>25</v>
+      <c r="B13" s="27" t="s">
+        <v>23</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
-      <c r="E13" s="14"/>
+      <c r="E13" s="12"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51395,7 +51395,7 @@
     </row>
     <row r="14" ht="20.25" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B14" s="8">
         <v>5.0</v>
@@ -51406,7 +51406,7 @@
       <c r="D14" s="8">
         <v>1.0</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="12">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51431,7 +51431,7 @@
       <c r="D15" s="8">
         <v>1.0</v>
       </c>
-      <c r="E15" s="14"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51443,7 +51443,7 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" s="8">
         <v>5.0</v>
@@ -51454,11 +51454,11 @@
       <c r="D16" s="8">
         <v>4.0</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="17" t="s">
-        <v>27</v>
+      <c r="F16" s="18" t="s">
+        <v>26</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51470,7 +51470,7 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B17" s="8">
         <v>12.0</v>
@@ -51481,7 +51481,7 @@
       <c r="D17" s="8">
         <v>1.0</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="12">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="32"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="24"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,7 +51510,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
@@ -51529,16 +51529,16 @@
       <c r="A20" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="11">
         <v>6.0</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="11">
         <v>45.0</v>
       </c>
       <c r="D20" s="8">
         <v>1.0</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="12">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51552,18 +51552,18 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="11">
         <v>18.0</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="11">
         <v>20.0</v>
       </c>
       <c r="D21" s="8">
         <v>1.0</v>
       </c>
-      <c r="E21" s="14">
+      <c r="E21" s="12">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51591,15 +51591,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="33" t="s">
-        <v>9</v>
+      <c r="A23" s="25" t="s">
+        <v>11</v>
       </c>
-      <c r="B23" s="34" t="s">
-        <v>25</v>
+      <c r="B23" s="27" t="s">
+        <v>23</v>
       </c>
       <c r="C23" s="19"/>
       <c r="D23" s="19"/>
-      <c r="E23" s="14">
+      <c r="E23" s="12">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51613,18 +51613,18 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="11">
         <v>6.0</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="11">
         <v>50.0</v>
       </c>
       <c r="D24" s="8">
         <v>1.0</v>
       </c>
-      <c r="E24" s="14">
+      <c r="E24" s="12">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51640,16 +51640,16 @@
       <c r="A25" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="22">
+      <c r="B25" s="11">
         <v>8.0</v>
       </c>
-      <c r="C25" s="22">
+      <c r="C25" s="11">
         <v>30.0</v>
       </c>
       <c r="D25" s="8">
         <v>1.0</v>
       </c>
-      <c r="E25" s="14">
+      <c r="E25" s="12">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51663,22 +51663,22 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
-      <c r="B26" s="22">
+      <c r="B26" s="11">
         <v>10.0</v>
       </c>
-      <c r="C26" s="22">
+      <c r="C26" s="11">
         <v>30.0</v>
       </c>
       <c r="D26" s="8">
         <v>4.0</v>
       </c>
-      <c r="E26" s="14">
+      <c r="E26" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="17" t="s">
-        <v>27</v>
+      <c r="F26" s="18" t="s">
+        <v>26</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51690,18 +51690,18 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
-      <c r="B27" s="22">
+      <c r="B27" s="11">
         <v>17.0</v>
       </c>
-      <c r="C27" s="22">
+      <c r="C27" s="11">
         <v>15.0</v>
       </c>
       <c r="D27" s="8">
         <v>1.0</v>
       </c>
-      <c r="E27" s="14">
+      <c r="E27" s="12">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51729,11 +51729,11 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="33" t="s">
-        <v>13</v>
+      <c r="A29" s="25" t="s">
+        <v>16</v>
       </c>
-      <c r="B29" s="34" t="s">
-        <v>25</v>
+      <c r="B29" s="27" t="s">
+        <v>23</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="19"/>
@@ -51749,18 +51749,18 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
-      <c r="B30" s="22">
+      <c r="B30" s="11">
         <v>6.0</v>
       </c>
-      <c r="C30" s="22">
+      <c r="C30" s="11">
         <v>50.0</v>
       </c>
       <c r="D30" s="8">
         <v>1.0</v>
       </c>
-      <c r="E30" s="14">
+      <c r="E30" s="12">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51776,10 +51776,10 @@
       <c r="A31" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="22">
+      <c r="B31" s="11">
         <v>8.0</v>
       </c>
-      <c r="C31" s="22">
+      <c r="C31" s="11">
         <v>30.0</v>
       </c>
       <c r="D31" s="8">
@@ -51797,18 +51797,18 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="B32" s="22">
+      <c r="B32" s="11">
         <v>15.0</v>
       </c>
-      <c r="C32" s="22">
+      <c r="C32" s="11">
         <v>10.0</v>
       </c>
       <c r="D32" s="8">
         <v>2.0</v>
       </c>
-      <c r="E32" s="14">
+      <c r="E32" s="12">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51836,13 +51836,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="s">
-        <v>13</v>
+      <c r="A34" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="24"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="26"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51853,19 +51853,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="s">
+      <c r="A35" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B35" s="41" t="s">
-        <v>30</v>
+      <c r="B35" s="36" t="s">
+        <v>28</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="36">
         <v>40.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="36">
         <v>1.0</v>
       </c>
-      <c r="E35" s="21">
+      <c r="E35" s="22">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51878,19 +51878,19 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="s">
-        <v>8</v>
+      <c r="A36" s="16" t="s">
+        <v>9</v>
       </c>
-      <c r="B36" s="41">
+      <c r="B36" s="36">
         <v>30.0</v>
       </c>
-      <c r="C36" s="41">
+      <c r="C36" s="36">
         <v>15.0</v>
       </c>
-      <c r="D36" s="41">
+      <c r="D36" s="36">
         <v>1.0</v>
       </c>
-      <c r="E36" s="24"/>
+      <c r="E36" s="26"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51902,7 +51902,7 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B37" s="8">
         <v>10.0</v>
@@ -51913,7 +51913,7 @@
       <c r="D37" s="8">
         <v>1.0</v>
       </c>
-      <c r="E37" s="14">
+      <c r="E37" s="12">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51926,7 +51926,7 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="18"/>
+      <c r="A38" s="20"/>
       <c r="B38" s="19"/>
       <c r="C38" s="19"/>
       <c r="D38" s="19"/>
@@ -51959,7 +51959,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B40" s="8">
         <v>40.0</v>
@@ -51970,7 +51970,7 @@
       <c r="D40" s="8">
         <v>1.0</v>
       </c>
-      <c r="E40" s="14">
+      <c r="E40" s="12">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51999,7 +51999,7 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B42" s="19"/>
       <c r="C42" s="19"/>
@@ -52027,7 +52027,7 @@
       <c r="D43" s="8">
         <v>1.0</v>
       </c>
-      <c r="E43" s="14">
+      <c r="E43" s="12">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52041,7 +52041,7 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B44" s="8">
         <v>55.0</v>
@@ -52052,7 +52052,7 @@
       <c r="D44" s="8">
         <v>1.0</v>
       </c>
-      <c r="E44" s="14">
+      <c r="E44" s="12">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52077,10 +52077,10 @@
       <c r="D45" s="8">
         <v>1.0</v>
       </c>
-      <c r="E45" s="14">
+      <c r="E45" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="17" t="s">
+      <c r="F45" s="18" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52108,7 +52108,7 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B47" s="19"/>
       <c r="C47" s="19"/>
@@ -52125,7 +52125,7 @@
     </row>
     <row r="48">
       <c r="A48" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B48" s="8">
         <v>55.0</v>
@@ -52136,7 +52136,7 @@
       <c r="D48" s="8">
         <v>1.0</v>
       </c>
-      <c r="E48" s="14">
+      <c r="E48" s="12">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52165,7 +52165,7 @@
     </row>
     <row r="50">
       <c r="A50" s="42" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B50" s="19"/>
       <c r="C50" s="19"/>
@@ -52182,7 +52182,7 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B51" s="8">
         <v>60.0</v>
@@ -52193,7 +52193,7 @@
       <c r="D51" s="8">
         <v>1.0</v>
       </c>
-      <c r="E51" s="14">
+      <c r="E51" s="12">
         <v>46203.63265940972</v>
       </c>
       <c r="F51" s="4"/>
@@ -52218,7 +52218,7 @@
       <c r="D52" s="8">
         <v>1.0</v>
       </c>
-      <c r="E52" s="14">
+      <c r="E52" s="12">
         <v>46253.61151159722</v>
       </c>
       <c r="F52" s="4"/>
@@ -52264,18 +52264,18 @@
     </row>
     <row r="55">
       <c r="A55" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
-      <c r="B55" s="22">
+      <c r="B55" s="11">
         <v>70.0</v>
       </c>
-      <c r="C55" s="22">
+      <c r="C55" s="11">
         <v>300.0</v>
       </c>
-      <c r="D55" s="22">
+      <c r="D55" s="11">
         <v>1.0</v>
       </c>
-      <c r="E55" s="14">
+      <c r="E55" s="12">
         <v>46223.80899857639</v>
       </c>
       <c r="F55" s="4"/>
@@ -52291,16 +52291,16 @@
       <c r="A56" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B56" s="22">
+      <c r="B56" s="11">
         <v>10.0</v>
       </c>
-      <c r="C56" s="22">
+      <c r="C56" s="11">
         <v>20.0</v>
       </c>
-      <c r="D56" s="22">
+      <c r="D56" s="11">
         <v>1.0</v>
       </c>
-      <c r="E56" s="14">
+      <c r="E56" s="12">
         <v>46223.80911148148</v>
       </c>
       <c r="F56" s="4"/>
@@ -52314,19 +52314,19 @@
     </row>
     <row r="57">
       <c r="A57" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="B57" s="22">
+      <c r="B57" s="11">
         <v>70.0</v>
       </c>
-      <c r="C57" s="22">
-        <v>10.0</v>
+      <c r="C57" s="11">
+        <v>8.0</v>
       </c>
-      <c r="D57" s="22">
+      <c r="D57" s="11">
         <v>1.0</v>
       </c>
-      <c r="E57" s="14">
-        <v>46207.72572512731</v>
+      <c r="E57" s="12">
+        <v>46260.758642430555</v>
       </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
@@ -52361,7 +52361,7 @@
       </c>
       <c r="C59" s="8"/>
       <c r="D59" s="8"/>
-      <c r="E59" s="14">
+      <c r="E59" s="12">
         <v>45946.87875708334</v>
       </c>
       <c r="F59" s="4"/>
@@ -52382,7 +52382,7 @@
       </c>
       <c r="C60" s="19"/>
       <c r="D60" s="19"/>
-      <c r="E60" s="14">
+      <c r="E60" s="12">
         <v>45946.87887299768</v>
       </c>
       <c r="F60" s="4"/>
@@ -52412,16 +52412,16 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="39" t="s">
+      <c r="A62" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B62" s="39">
+      <c r="B62" s="40">
         <v>100.0</v>
       </c>
-      <c r="C62" s="17">
+      <c r="C62" s="18">
         <v>1.0</v>
       </c>
-      <c r="D62" s="17">
+      <c r="D62" s="18">
         <v>2.0</v>
       </c>
       <c r="E62" s="46">
@@ -52437,8 +52437,8 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="40"/>
-      <c r="B63" s="40"/>
+      <c r="A63" s="41"/>
+      <c r="B63" s="41"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
@@ -52452,10 +52452,10 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="39" t="s">
+      <c r="A64" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B64" s="40"/>
+      <c r="B64" s="41"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
@@ -52470,15 +52470,15 @@
     </row>
     <row r="65">
       <c r="A65" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
-      <c r="B65" s="39">
+      <c r="B65" s="40">
         <v>50.0</v>
       </c>
-      <c r="C65" s="17">
+      <c r="C65" s="18">
         <v>20.0</v>
       </c>
-      <c r="D65" s="17">
+      <c r="D65" s="18">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52494,13 +52494,13 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="39" t="s">
+      <c r="A66" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B66" s="39">
+      <c r="B66" s="40">
         <v>15.0</v>
       </c>
-      <c r="C66" s="17">
+      <c r="C66" s="18">
         <v>16.0</v>
       </c>
       <c r="D66" s="4"/>
@@ -52517,8 +52517,8 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="40"/>
-      <c r="B67" s="40"/>
+      <c r="A67" s="41"/>
+      <c r="B67" s="41"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
@@ -52532,11 +52532,11 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="39" t="s">
+      <c r="A68" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="39" t="s">
-        <v>17</v>
+      <c r="B68" s="40" t="s">
+        <v>21</v>
       </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -52553,16 +52553,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="39" t="s">
+      <c r="A69" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="39">
+      <c r="B69" s="40">
         <v>5.0</v>
       </c>
-      <c r="C69" s="17">
+      <c r="C69" s="18">
         <v>80.0</v>
       </c>
-      <c r="D69" s="17">
+      <c r="D69" s="18">
         <v>1.0</v>
       </c>
       <c r="E69" s="46">
@@ -52578,16 +52578,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="39" t="s">
+      <c r="A70" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B70" s="39">
+      <c r="B70" s="40">
         <v>15.0</v>
       </c>
-      <c r="C70" s="17">
+      <c r="C70" s="18">
         <v>10.0</v>
       </c>
-      <c r="D70" s="17">
+      <c r="D70" s="18">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52603,16 +52603,16 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="39" t="s">
-        <v>22</v>
+      <c r="A71" s="40" t="s">
+        <v>18</v>
       </c>
-      <c r="B71" s="39">
+      <c r="B71" s="40">
         <v>30.0</v>
       </c>
-      <c r="C71" s="17">
+      <c r="C71" s="18">
         <v>10.0</v>
       </c>
-      <c r="D71" s="17">
+      <c r="D71" s="18">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52628,8 +52628,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="40"/>
-      <c r="B72" s="40"/>
+      <c r="A72" s="41"/>
+      <c r="B72" s="41"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52643,10 +52643,10 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="39" t="s">
+      <c r="A73" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B73" s="39" t="s">
+      <c r="B73" s="40" t="s">
         <v>33</v>
       </c>
       <c r="C73" s="4"/>
@@ -52664,16 +52664,16 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="39" t="s">
+      <c r="A74" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B74" s="39">
+      <c r="B74" s="40">
         <v>5.0</v>
       </c>
-      <c r="C74" s="17">
+      <c r="C74" s="18">
         <v>80.0</v>
       </c>
-      <c r="D74" s="17">
+      <c r="D74" s="18">
         <v>1.0</v>
       </c>
       <c r="E74" s="4"/>
@@ -52687,16 +52687,16 @@
       <c r="M74" s="4"/>
     </row>
     <row r="75">
-      <c r="A75" s="39" t="s">
+      <c r="A75" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B75" s="39">
+      <c r="B75" s="40">
         <v>15.0</v>
       </c>
-      <c r="C75" s="17">
+      <c r="C75" s="18">
         <v>10.0</v>
       </c>
-      <c r="D75" s="17">
+      <c r="D75" s="18">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52710,16 +52710,16 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76">
-      <c r="A76" s="39" t="s">
-        <v>22</v>
+      <c r="A76" s="40" t="s">
+        <v>18</v>
       </c>
-      <c r="B76" s="39">
+      <c r="B76" s="40">
         <v>20.0</v>
       </c>
-      <c r="C76" s="17">
+      <c r="C76" s="18">
         <v>10.0</v>
       </c>
-      <c r="D76" s="17">
+      <c r="D76" s="18">
         <v>6.0</v>
       </c>
       <c r="E76" s="46">
@@ -52735,8 +52735,8 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="40"/>
-      <c r="B77" s="40"/>
+      <c r="A77" s="41"/>
+      <c r="B77" s="41"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
@@ -52750,8 +52750,8 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="39"/>
-      <c r="B78" s="40"/>
+      <c r="A78" s="40"/>
+      <c r="B78" s="41"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
@@ -52765,8 +52765,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="40"/>
-      <c r="B79" s="40"/>
+      <c r="A79" s="41"/>
+      <c r="B79" s="41"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-09-01T13:12:05.359Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -37,34 +37,43 @@
     <t>Line</t>
   </si>
   <si>
+    <t>Cut-1/2</t>
+  </si>
+  <si>
+    <t>Cut(detail)</t>
+  </si>
+  <si>
+    <t>(PS)</t>
+  </si>
+  <si>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>FILL</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
+  </si>
+  <si>
+    <t>1mm</t>
+  </si>
+  <si>
+    <t>Fill</t>
+  </si>
+  <si>
     <t>遮蓋膠紙</t>
   </si>
   <si>
     <t>刀壓</t>
   </si>
   <si>
-    <t>Cut-1/2</t>
+    <t>2mm</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
-  </si>
-  <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>(PS)</t>
+    <t>3mm</t>
   </si>
   <si>
     <t>A4紙</t>
-  </si>
-  <si>
-    <t>1mm</t>
   </si>
   <si>
     <t>03mm</t>
@@ -73,16 +82,7 @@
     <t>Cut</t>
   </si>
   <si>
-    <t>2mm</t>
-  </si>
-  <si>
     <t>0.3 mm</t>
-  </si>
-  <si>
-    <t>3mm</t>
-  </si>
-  <si>
-    <t>Fill</t>
   </si>
   <si>
     <t>PS</t>
@@ -91,22 +91,22 @@
     <t>4mm</t>
   </si>
   <si>
+    <t>(0.9 Power)</t>
+  </si>
+  <si>
     <t>cut</t>
+  </si>
+  <si>
+    <t>甲板紙</t>
   </si>
   <si>
     <t>Keep Detail</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>６</t>
-  </si>
-  <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>1.5mm</t>
@@ -209,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -330,6 +330,9 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -337,12 +340,6 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -354,6 +351,9 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -363,19 +363,26 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -384,16 +391,9 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -415,9 +415,6 @@
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -432,6 +429,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -722,19 +722,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="10">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -748,19 +748,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>9</v>
+      <c r="A4" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>25.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="9"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -773,9 +773,9 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
       <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -788,14 +788,14 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="s">
-        <v>11</v>
+      <c r="A6" s="12" t="s">
+        <v>10</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
       <c r="E6" s="15"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -811,20 +811,20 @@
       <c r="A7" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="13">
         <v>4.0</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="13">
         <v>10.0</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="13">
         <v>1.0</v>
       </c>
       <c r="E7" s="17">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -835,22 +835,22 @@
     </row>
     <row r="8">
       <c r="A8" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="13">
         <v>25.0</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="13">
         <v>5.0</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="13">
         <v>1.0</v>
       </c>
       <c r="E8" s="17">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="20"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="9"/>
+      <c r="A9" s="19"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="10"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +877,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="10"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -894,23 +894,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="9">
         <v>5.0</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="9">
         <v>5.0</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="10">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,16 +920,16 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="9">
         <v>5.0</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="9">
         <v>15.0</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="9">
         <v>1.0</v>
       </c>
       <c r="E12" s="6"/>
@@ -944,16 +944,16 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>9</v>
+      <c r="A13" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <v>32.0</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="9">
         <v>5.0</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
       <c r="E13" s="6"/>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
+      <c r="A14" s="19"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -984,12 +984,12 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>19</v>
+      <c r="A15" s="12" t="s">
+        <v>17</v>
       </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
       <c r="E15" s="15"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1005,13 +1005,13 @@
       <c r="A16" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="13">
         <v>5.0</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="13">
         <v>5.0</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="13">
         <v>1.0</v>
       </c>
       <c r="E16" s="15"/>
@@ -1027,15 +1027,15 @@
     </row>
     <row r="17">
       <c r="A17" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="13">
         <v>50.0</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="13">
         <v>5.0</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="13">
         <v>1.0</v>
       </c>
       <c r="E17" s="15"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="20"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
+      <c r="A18" s="19"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1067,11 +1067,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1084,16 +1084,16 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>5.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -1108,12 +1108,12 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>9</v>
+      <c r="A21" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="20"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
+      <c r="A22" s="19"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1142,12 +1142,12 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
       <c r="E23" s="15"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -1163,13 +1163,13 @@
       <c r="A24" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="13">
         <v>5.0</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="13">
         <v>5.0</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="13">
         <v>1.0</v>
       </c>
       <c r="E24" s="15"/>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="25">
       <c r="A25" s="30" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B25" s="31">
         <v>55.0</v>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="19"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
+      <c r="A26" s="20"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,14 +1222,14 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>15</v>
+      <c r="A27" s="9" t="s">
+        <v>19</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>27</v>
+      <c r="B27" s="9" t="s">
+        <v>25</v>
       </c>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
       <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
@@ -1244,16 +1244,16 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="9">
         <v>2.0</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="19"/>
+      <c r="D28" s="20"/>
       <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
@@ -1268,16 +1268,16 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>18</v>
+      <c r="A29" s="9" t="s">
+        <v>21</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="9">
         <v>20.0</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="19"/>
+      <c r="D29" s="20"/>
       <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="19"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="19"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17130,7 +17130,7 @@
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17143,19 +17143,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>3.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17170,19 +17170,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>9</v>
+      <c r="A4" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17195,13 +17195,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>14</v>
+      <c r="A5" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="10"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17214,22 +17214,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <v>18.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,22 +17239,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>9</v>
+      <c r="A7" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="9">
         <v>18.0</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="9">
         <v>3.0</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17265,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="12"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>11</v>
+      <c r="A9" s="12" t="s">
+        <v>10</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="22"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="18"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17303,16 +17303,16 @@
       <c r="A10" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="13">
         <v>4.0</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="13">
         <v>15.0</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="13">
         <v>1.0</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="18">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17328,18 +17328,18 @@
     </row>
     <row r="11">
       <c r="A11" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="13">
         <v>25.0</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="13">
         <v>10.0</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="13">
         <v>1.0</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="18">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17355,18 +17355,18 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="13">
         <v>4.0</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="13">
         <v>10.0</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="13">
         <v>1.0</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="18">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17382,12 +17382,12 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="26"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="21"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17403,16 +17403,16 @@
       <c r="A14" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="13">
         <v>2.0</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="13">
         <v>18.0</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="13">
         <v>1.0</v>
       </c>
-      <c r="E14" s="26"/>
+      <c r="E14" s="21"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17426,18 +17426,18 @@
     </row>
     <row r="15">
       <c r="A15" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="13">
         <v>18.0</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="13">
         <v>4.0</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="13">
         <v>1.0</v>
       </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="21"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="28"/>
-      <c r="E16" s="10"/>
+      <c r="A16" s="24"/>
+      <c r="E16" s="7"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17465,14 +17465,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
-      <c r="B17" s="29" t="s">
-        <v>14</v>
+      <c r="B17" s="25" t="s">
+        <v>9</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="10"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="7"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17485,19 +17485,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17510,19 +17510,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>9</v>
+      <c r="A19" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="9">
         <v>40.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="9">
         <v>5.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="10"/>
+      <c r="A20" s="19"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="s">
-        <v>19</v>
+      <c r="A21" s="12" t="s">
+        <v>17</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="26"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="21"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17574,16 +17574,16 @@
       <c r="A22" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="13">
         <v>8.0</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="13">
         <v>15.0</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="13">
         <v>1.0</v>
       </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="21"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17597,18 +17597,18 @@
     </row>
     <row r="23">
       <c r="A23" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="13">
         <v>55.0</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="13">
         <v>5.0</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="13">
         <v>2.0</v>
       </c>
-      <c r="E23" s="26"/>
+      <c r="E23" s="21"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="10"/>
+      <c r="A24" s="19"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17639,12 +17639,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="10"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17657,19 +17657,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="10"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17682,19 +17682,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>9</v>
+      <c r="A27" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>60.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="11">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="10"/>
+      <c r="A28" s="19"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="26"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="21"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17748,16 +17748,16 @@
       <c r="A30" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="13">
         <v>18.0</v>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="13">
         <v>5.0</v>
       </c>
-      <c r="D30" s="14">
+      <c r="D30" s="13">
         <v>1.0</v>
       </c>
-      <c r="E30" s="26"/>
+      <c r="E30" s="21"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17771,7 +17771,7 @@
     </row>
     <row r="31">
       <c r="A31" s="30" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B31" s="31">
         <v>70.0</v>
@@ -17812,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="B33" s="37">
+        <v>5.0</v>
+      </c>
+      <c r="C33" s="37">
+        <v>10.0</v>
+      </c>
+      <c r="D33" s="37">
+        <v>2.0</v>
+      </c>
+      <c r="E33" s="38">
+        <v>46043.55545597222</v>
+      </c>
+      <c r="F33" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B33" s="38">
-        <v>5.0</v>
-      </c>
-      <c r="C33" s="38">
-        <v>10.0</v>
-      </c>
-      <c r="D33" s="38">
-        <v>2.0</v>
-      </c>
-      <c r="E33" s="39">
-        <v>46043.55545597222</v>
-      </c>
-      <c r="F33" s="40" t="s">
-        <v>30</v>
-      </c>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="40"/>
+      <c r="M33" s="40"/>
+      <c r="N33" s="40"/>
+      <c r="O33" s="40"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17875,14 +17875,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>15</v>
+      <c r="A36" s="9" t="s">
+        <v>19</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>27</v>
+      <c r="B36" s="9" t="s">
+        <v>25</v>
       </c>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17896,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="9">
         <v>2.0</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="19"/>
+      <c r="D37" s="20"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17919,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="s">
-        <v>18</v>
+      <c r="A38" s="9" t="s">
+        <v>21</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="9">
         <v>20.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="19"/>
+      <c r="D38" s="20"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34607,19 +34607,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="10">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34633,19 +34633,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>10</v>
+      <c r="A4" s="8" t="s">
+        <v>8</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <v>10.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>2.0</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="10">
         <v>46232.916719409724</v>
       </c>
       <c r="F4" s="4"/>
@@ -34659,19 +34659,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>9</v>
+      <c r="A5" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="9">
         <v>20.0</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="9">
         <v>20.0</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="9">
         <v>1.0</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="10">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34685,19 +34685,19 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>13</v>
+      <c r="A6" s="8" t="s">
+        <v>11</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <v>20.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="10">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34712,9 +34712,9 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
       <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -34727,14 +34727,14 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="s">
-        <v>11</v>
+      <c r="A8" s="12" t="s">
+        <v>10</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
       <c r="E8" s="15"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -34750,20 +34750,20 @@
       <c r="A9" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="13">
         <v>4.0</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="13">
         <v>10.0</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="13">
         <v>1.0</v>
       </c>
       <c r="E9" s="17">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34774,22 +34774,22 @@
     </row>
     <row r="10">
       <c r="A10" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="13">
         <v>20.0</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="13">
         <v>10.0</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="13">
         <v>1.0</v>
       </c>
       <c r="E10" s="17">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,11 +34799,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="20"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="9"/>
+      <c r="A11" s="19"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="10"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34816,7 +34816,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34830,13 +34830,13 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="10"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34848,19 +34848,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>9</v>
+      <c r="A14" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="9">
         <v>20.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="9">
         <v>10.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="10">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34874,13 +34874,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>13</v>
+      <c r="A15" s="8" t="s">
+        <v>11</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="10"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34892,11 +34892,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="20"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="9"/>
+      <c r="A16" s="19"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34909,12 +34909,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="9"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34926,23 +34926,23 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="10">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34952,16 +34952,16 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="9">
         <v>5.0</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="9">
         <v>15.0</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
       <c r="E19" s="6"/>
@@ -34976,16 +34976,16 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>9</v>
+      <c r="A20" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>32.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
       <c r="E20" s="6"/>
@@ -35000,10 +35000,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="20"/>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
+      <c r="A21" s="19"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35016,12 +35016,12 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="s">
-        <v>19</v>
+      <c r="A22" s="12" t="s">
+        <v>17</v>
       </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
       <c r="E22" s="15"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -35037,13 +35037,13 @@
       <c r="A23" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="13">
         <v>5.0</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="13">
         <v>5.0</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="13">
         <v>1.0</v>
       </c>
       <c r="E23" s="15"/>
@@ -35059,15 +35059,15 @@
     </row>
     <row r="24">
       <c r="A24" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="13">
         <v>50.0</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="13">
         <v>5.0</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="13">
         <v>1.0</v>
       </c>
       <c r="E24" s="15"/>
@@ -35082,10 +35082,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
+      <c r="A25" s="19"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35099,11 +35099,11 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35116,16 +35116,16 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>5.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="9">
         <v>1.0</v>
       </c>
       <c r="E27" s="6"/>
@@ -35140,12 +35140,12 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>9</v>
+      <c r="A28" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35158,10 +35158,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="20"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
+      <c r="A29" s="19"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35174,12 +35174,12 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
       <c r="E30" s="15"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -35195,13 +35195,13 @@
       <c r="A31" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="14">
+      <c r="B31" s="13">
         <v>5.0</v>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="13">
         <v>5.0</v>
       </c>
-      <c r="D31" s="14">
+      <c r="D31" s="13">
         <v>1.0</v>
       </c>
       <c r="E31" s="15"/>
@@ -35217,7 +35217,7 @@
     </row>
     <row r="32">
       <c r="A32" s="30" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B32" s="31">
         <v>55.0</v>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="19"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35254,14 +35254,14 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>15</v>
+      <c r="A34" s="9" t="s">
+        <v>19</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>27</v>
+      <c r="B34" s="9" t="s">
+        <v>25</v>
       </c>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
       <c r="E34" s="34">
         <v>46051.96156388889</v>
       </c>
@@ -35276,16 +35276,16 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="9">
         <v>2.0</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="9">
         <v>100.0</v>
       </c>
-      <c r="D35" s="19"/>
+      <c r="D35" s="20"/>
       <c r="E35" s="34">
         <v>46100.83597384259</v>
       </c>
@@ -35300,16 +35300,16 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="s">
-        <v>18</v>
+      <c r="A36" s="9" t="s">
+        <v>21</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="9">
         <v>20.0</v>
       </c>
-      <c r="C36" s="8">
+      <c r="C36" s="9">
         <v>100.0</v>
       </c>
-      <c r="D36" s="19"/>
+      <c r="D36" s="20"/>
       <c r="E36" s="34">
         <v>46100.83604224537</v>
       </c>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="19"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="19"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
+      <c r="A38" s="20"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,10 +51132,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -51156,13 +51156,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="10"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51173,19 +51173,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>9</v>
+      <c r="A3" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="22">
         <v>60.0</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="22">
         <v>20.0</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10"/>
+      <c r="E3" s="7"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51197,10 +51197,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="10"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51212,14 +51212,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="11"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51230,17 +51230,17 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <v>6.0</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <v>100.0</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="12">
+      <c r="D6" s="9"/>
+      <c r="E6" s="11">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51253,19 +51253,19 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="7" t="s">
-        <v>18</v>
+      <c r="A7" s="8" t="s">
+        <v>21</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="9">
         <v>8.0</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="9">
         <v>60.0</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="11">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51279,10 +51279,10 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="5"/>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="10"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="7"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51294,12 +51294,12 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="10"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="7"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51310,19 +51310,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="9">
         <v>10.0</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="9">
         <v>45.0</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="11">
         <v>46106.73232292824</v>
       </c>
       <c r="F10" s="4"/>
@@ -51335,20 +51335,20 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>18</v>
+      <c r="A11" s="8" t="s">
+        <v>21</v>
       </c>
-      <c r="B11" s="8">
-        <v>11.0</v>
+      <c r="B11" s="9">
+        <v>13.0</v>
       </c>
-      <c r="C11" s="8">
-        <v>20.0</v>
+      <c r="C11" s="9">
+        <v>30.0</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="12">
-        <v>46106.732369062505</v>
+      <c r="E11" s="11">
+        <v>46266.88338049769</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="24"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="27"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,15 +51375,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="s">
-        <v>20</v>
+      <c r="A13" s="28" t="s">
+        <v>22</v>
       </c>
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="12"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51394,19 +51394,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14" ht="20.25" customHeight="1">
-      <c r="A14" s="7" t="s">
-        <v>22</v>
+      <c r="A14" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="9">
         <v>5.0</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="9">
         <v>60.0</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="11">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51419,19 +51419,19 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="9">
         <v>5.0</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="9">
         <v>30.0</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="9">
         <v>1.0</v>
       </c>
-      <c r="E15" s="12"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51442,23 +51442,23 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
-        <v>25</v>
+      <c r="A16" s="8" t="s">
+        <v>26</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="9">
         <v>5.0</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="9">
         <v>30.0</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="9">
         <v>4.0</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="11">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="18" t="s">
-        <v>26</v>
+      <c r="F16" s="14" t="s">
+        <v>28</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51469,19 +51469,19 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="s">
-        <v>18</v>
+      <c r="A17" s="8" t="s">
+        <v>21</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="9">
         <v>12.0</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="9">
         <v>20.0</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="9">
         <v>1.0</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="11">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="24"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="27"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,12 +51510,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="10"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51526,19 +51526,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="22">
         <v>6.0</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="22">
         <v>45.0</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="11">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51551,19 +51551,19 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>9</v>
+      <c r="A21" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="22">
         <v>18.0</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="22">
         <v>20.0</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D21" s="9">
         <v>1.0</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="11">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51576,11 +51576,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="7"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="10"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="7"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51591,15 +51591,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="s">
-        <v>11</v>
+      <c r="A23" s="28" t="s">
+        <v>10</v>
       </c>
-      <c r="B23" s="27" t="s">
+      <c r="B23" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="12">
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="11">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51612,19 +51612,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>22</v>
+      <c r="A24" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="22">
         <v>6.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="22">
         <v>50.0</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="11">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51637,19 +51637,19 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="22">
         <v>8.0</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="22">
         <v>30.0</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="9">
         <v>1.0</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="11">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51662,23 +51662,23 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>18</v>
+      <c r="A26" s="8" t="s">
+        <v>21</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="22">
         <v>10.0</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="22">
         <v>30.0</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="9">
         <v>4.0</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="11">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="18" t="s">
-        <v>26</v>
+      <c r="F26" s="14" t="s">
+        <v>28</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51689,19 +51689,19 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>18</v>
+      <c r="A27" s="8" t="s">
+        <v>21</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="22">
         <v>17.0</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="22">
         <v>15.0</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="9">
         <v>1.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="11">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51714,11 +51714,11 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="10"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51729,15 +51729,15 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="25" t="s">
-        <v>16</v>
+      <c r="A29" s="28" t="s">
+        <v>13</v>
       </c>
-      <c r="B29" s="27" t="s">
+      <c r="B29" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="10"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="7"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51748,19 +51748,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>22</v>
+      <c r="A30" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="22">
         <v>6.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="22">
         <v>50.0</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="9">
         <v>1.0</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="11">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51773,19 +51773,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="22">
         <v>8.0</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="22">
         <v>30.0</v>
       </c>
-      <c r="D31" s="8">
+      <c r="D31" s="9">
         <v>1.0</v>
       </c>
-      <c r="E31" s="10"/>
+      <c r="E31" s="7"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51796,19 +51796,19 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="s">
-        <v>9</v>
+      <c r="A32" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="22">
         <v>15.0</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="22">
         <v>10.0</v>
       </c>
-      <c r="D32" s="8">
+      <c r="D32" s="9">
         <v>2.0</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="11">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51821,11 +51821,11 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="7"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="10"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="7"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51836,13 +51836,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="s">
-        <v>16</v>
+      <c r="A34" s="12" t="s">
+        <v>13</v>
       </c>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="26"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="21"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51856,16 +51856,16 @@
       <c r="A35" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B35" s="36" t="s">
-        <v>28</v>
+      <c r="B35" s="41" t="s">
+        <v>30</v>
       </c>
-      <c r="C35" s="36">
+      <c r="C35" s="41">
         <v>40.0</v>
       </c>
-      <c r="D35" s="36">
+      <c r="D35" s="41">
         <v>1.0</v>
       </c>
-      <c r="E35" s="22">
+      <c r="E35" s="18">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51879,18 +51879,18 @@
     </row>
     <row r="36">
       <c r="A36" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B36" s="36">
+      <c r="B36" s="41">
         <v>30.0</v>
       </c>
-      <c r="C36" s="36">
+      <c r="C36" s="41">
         <v>15.0</v>
       </c>
-      <c r="D36" s="36">
+      <c r="D36" s="41">
         <v>1.0</v>
       </c>
-      <c r="E36" s="26"/>
+      <c r="E36" s="21"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51901,19 +51901,19 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="s">
-        <v>22</v>
+      <c r="A37" s="8" t="s">
+        <v>14</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="9">
         <v>10.0</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="9">
         <v>150.0</v>
       </c>
-      <c r="D37" s="8">
+      <c r="D37" s="9">
         <v>1.0</v>
       </c>
-      <c r="E37" s="12">
+      <c r="E37" s="11">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51926,11 +51926,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="20"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="10"/>
+      <c r="A38" s="19"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="7"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51944,10 +51944,10 @@
       <c r="A39" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="19"/>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="10"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51958,19 +51958,19 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="s">
-        <v>9</v>
+      <c r="A40" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B40" s="8">
+      <c r="B40" s="9">
         <v>40.0</v>
       </c>
-      <c r="C40" s="8">
+      <c r="C40" s="9">
         <v>15.0</v>
       </c>
-      <c r="D40" s="8">
+      <c r="D40" s="9">
         <v>1.0</v>
       </c>
-      <c r="E40" s="12">
+      <c r="E40" s="11">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51984,10 +51984,10 @@
     </row>
     <row r="41">
       <c r="A41" s="5"/>
-      <c r="B41" s="19"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="10"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="7"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51999,12 +51999,12 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
-      <c r="B42" s="19"/>
-      <c r="C42" s="19"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="10"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="7"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -52015,19 +52015,19 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
+      <c r="A43" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="9">
         <v>9.0</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43" s="9">
         <v>20.0</v>
       </c>
-      <c r="D43" s="8">
+      <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="11">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52040,19 +52040,19 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="s">
-        <v>9</v>
+      <c r="A44" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B44" s="8">
+      <c r="B44" s="9">
         <v>55.0</v>
       </c>
-      <c r="C44" s="8">
+      <c r="C44" s="9">
         <v>20.0</v>
       </c>
-      <c r="D44" s="8">
+      <c r="D44" s="9">
         <v>1.0</v>
       </c>
-      <c r="E44" s="12">
+      <c r="E44" s="11">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52065,22 +52065,22 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="s">
+      <c r="A45" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="9">
         <v>10.0</v>
       </c>
-      <c r="C45" s="8">
+      <c r="C45" s="9">
         <v>250.0</v>
       </c>
-      <c r="D45" s="8">
+      <c r="D45" s="9">
         <v>1.0</v>
       </c>
-      <c r="E45" s="12">
+      <c r="E45" s="11">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="18" t="s">
+      <c r="F45" s="14" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52093,10 +52093,10 @@
     </row>
     <row r="46">
       <c r="A46" s="42"/>
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="10"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="7"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52108,12 +52108,12 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
-      <c r="B47" s="19"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="10"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="7"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52124,19 +52124,19 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="s">
-        <v>9</v>
+      <c r="A48" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B48" s="8">
+      <c r="B48" s="9">
         <v>55.0</v>
       </c>
-      <c r="C48" s="8">
+      <c r="C48" s="9">
         <v>10.0</v>
       </c>
-      <c r="D48" s="8">
+      <c r="D48" s="9">
         <v>1.0</v>
       </c>
-      <c r="E48" s="12">
+      <c r="E48" s="11">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52150,10 +52150,10 @@
     </row>
     <row r="49">
       <c r="A49" s="42"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="10"/>
+      <c r="B49" s="20"/>
+      <c r="C49" s="20"/>
+      <c r="D49" s="20"/>
+      <c r="E49" s="7"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52167,10 +52167,10 @@
       <c r="A50" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="B50" s="19"/>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="10"/>
+      <c r="B50" s="20"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="20"/>
+      <c r="E50" s="7"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52181,19 +52181,19 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="s">
-        <v>9</v>
+      <c r="A51" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B51" s="8">
+      <c r="B51" s="9">
         <v>60.0</v>
       </c>
-      <c r="C51" s="8">
+      <c r="C51" s="9">
         <v>10.0</v>
       </c>
-      <c r="D51" s="8">
+      <c r="D51" s="9">
         <v>1.0</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="11">
         <v>46203.63265940972</v>
       </c>
       <c r="F51" s="4"/>
@@ -52206,19 +52206,19 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="s">
+      <c r="A52" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B52" s="8">
+      <c r="B52" s="9">
         <v>10.0</v>
       </c>
-      <c r="C52" s="8">
+      <c r="C52" s="9">
         <v>50.0</v>
       </c>
-      <c r="D52" s="8">
+      <c r="D52" s="9">
         <v>1.0</v>
       </c>
-      <c r="E52" s="12">
+      <c r="E52" s="11">
         <v>46253.61151159722</v>
       </c>
       <c r="F52" s="4"/>
@@ -52232,10 +52232,10 @@
     </row>
     <row r="53">
       <c r="A53" s="42"/>
-      <c r="B53" s="19"/>
-      <c r="C53" s="19"/>
-      <c r="D53" s="19"/>
-      <c r="E53" s="10"/>
+      <c r="B53" s="20"/>
+      <c r="C53" s="20"/>
+      <c r="D53" s="20"/>
+      <c r="E53" s="7"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52249,10 +52249,10 @@
       <c r="A54" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B54" s="19"/>
-      <c r="C54" s="19"/>
-      <c r="D54" s="19"/>
-      <c r="E54" s="10"/>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
+      <c r="E54" s="7"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52263,19 +52263,19 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="s">
-        <v>13</v>
+      <c r="A55" s="8" t="s">
+        <v>11</v>
       </c>
-      <c r="B55" s="11">
+      <c r="B55" s="22">
         <v>70.0</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="22">
         <v>300.0</v>
       </c>
-      <c r="D55" s="11">
+      <c r="D55" s="22">
         <v>1.0</v>
       </c>
-      <c r="E55" s="12">
+      <c r="E55" s="11">
         <v>46223.80899857639</v>
       </c>
       <c r="F55" s="4"/>
@@ -52288,19 +52288,19 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="s">
+      <c r="A56" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B56" s="11">
+      <c r="B56" s="22">
         <v>10.0</v>
       </c>
-      <c r="C56" s="11">
+      <c r="C56" s="22">
         <v>20.0</v>
       </c>
-      <c r="D56" s="11">
+      <c r="D56" s="22">
         <v>1.0</v>
       </c>
-      <c r="E56" s="12">
+      <c r="E56" s="11">
         <v>46223.80911148148</v>
       </c>
       <c r="F56" s="4"/>
@@ -52313,19 +52313,19 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="s">
-        <v>9</v>
+      <c r="A57" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B57" s="11">
+      <c r="B57" s="22">
         <v>70.0</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="22">
         <v>8.0</v>
       </c>
-      <c r="D57" s="11">
+      <c r="D57" s="22">
         <v>1.0</v>
       </c>
-      <c r="E57" s="12">
+      <c r="E57" s="11">
         <v>46260.758642430555</v>
       </c>
       <c r="F57" s="4"/>
@@ -52338,11 +52338,11 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="7"/>
-      <c r="B58" s="8"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="8"/>
-      <c r="E58" s="10"/>
+      <c r="A58" s="8"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="7"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52353,15 +52353,15 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="s">
+      <c r="A59" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B59" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C59" s="8"/>
-      <c r="D59" s="8"/>
-      <c r="E59" s="12">
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="11">
         <v>45946.87875708334</v>
       </c>
       <c r="F59" s="4"/>
@@ -52374,15 +52374,15 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="7">
+      <c r="A60" s="8">
         <v>50.0</v>
       </c>
-      <c r="B60" s="8">
+      <c r="B60" s="9">
         <v>100.0</v>
       </c>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="12">
+      <c r="C60" s="20"/>
+      <c r="D60" s="20"/>
+      <c r="E60" s="11">
         <v>45946.87887299768</v>
       </c>
       <c r="F60" s="4"/>
@@ -52412,16 +52412,16 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="40" t="s">
+      <c r="A62" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="B62" s="40">
+      <c r="B62" s="39">
         <v>100.0</v>
       </c>
-      <c r="C62" s="18">
+      <c r="C62" s="14">
         <v>1.0</v>
       </c>
-      <c r="D62" s="18">
+      <c r="D62" s="14">
         <v>2.0</v>
       </c>
       <c r="E62" s="46">
@@ -52437,8 +52437,8 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="41"/>
-      <c r="B63" s="41"/>
+      <c r="A63" s="40"/>
+      <c r="B63" s="40"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
@@ -52452,10 +52452,10 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="40" t="s">
+      <c r="A64" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="B64" s="41"/>
+      <c r="B64" s="40"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
@@ -52469,16 +52469,16 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="7" t="s">
-        <v>9</v>
+      <c r="A65" s="8" t="s">
+        <v>7</v>
       </c>
-      <c r="B65" s="40">
+      <c r="B65" s="39">
         <v>50.0</v>
       </c>
-      <c r="C65" s="18">
+      <c r="C65" s="14">
         <v>20.0</v>
       </c>
-      <c r="D65" s="18">
+      <c r="D65" s="14">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52494,13 +52494,13 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="40" t="s">
+      <c r="A66" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B66" s="40">
+      <c r="B66" s="39">
         <v>15.0</v>
       </c>
-      <c r="C66" s="18">
+      <c r="C66" s="14">
         <v>16.0</v>
       </c>
       <c r="D66" s="4"/>
@@ -52517,8 +52517,8 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="41"/>
-      <c r="B67" s="41"/>
+      <c r="A67" s="40"/>
+      <c r="B67" s="40"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
@@ -52532,11 +52532,11 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="40" t="s">
+      <c r="A68" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="B68" s="40" t="s">
-        <v>21</v>
+      <c r="B68" s="39" t="s">
+        <v>18</v>
       </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -52553,16 +52553,16 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="40" t="s">
+      <c r="A69" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="40">
+      <c r="B69" s="39">
         <v>5.0</v>
       </c>
-      <c r="C69" s="18">
+      <c r="C69" s="14">
         <v>80.0</v>
       </c>
-      <c r="D69" s="18">
+      <c r="D69" s="14">
         <v>1.0</v>
       </c>
       <c r="E69" s="46">
@@ -52578,16 +52578,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="40" t="s">
+      <c r="A70" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="B70" s="40">
+      <c r="B70" s="39">
         <v>15.0</v>
       </c>
-      <c r="C70" s="18">
+      <c r="C70" s="14">
         <v>10.0</v>
       </c>
-      <c r="D70" s="18">
+      <c r="D70" s="14">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52603,16 +52603,16 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="40" t="s">
-        <v>18</v>
+      <c r="A71" s="39" t="s">
+        <v>21</v>
       </c>
-      <c r="B71" s="40">
+      <c r="B71" s="39">
         <v>30.0</v>
       </c>
-      <c r="C71" s="18">
+      <c r="C71" s="14">
         <v>10.0</v>
       </c>
-      <c r="D71" s="18">
+      <c r="D71" s="14">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52628,8 +52628,8 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="41"/>
-      <c r="B72" s="41"/>
+      <c r="A72" s="40"/>
+      <c r="B72" s="40"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
@@ -52643,10 +52643,10 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="40" t="s">
+      <c r="A73" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="B73" s="40" t="s">
+      <c r="B73" s="39" t="s">
         <v>33</v>
       </c>
       <c r="C73" s="4"/>
@@ -52664,16 +52664,16 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="40" t="s">
+      <c r="A74" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="B74" s="40">
+      <c r="B74" s="39">
         <v>5.0</v>
       </c>
-      <c r="C74" s="18">
+      <c r="C74" s="14">
         <v>80.0</v>
       </c>
-      <c r="D74" s="18">
+      <c r="D74" s="14">
         <v>1.0</v>
       </c>
       <c r="E74" s="4"/>
@@ -52687,16 +52687,16 @@
       <c r="M74" s="4"/>
     </row>
     <row r="75">
-      <c r="A75" s="40" t="s">
+      <c r="A75" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="B75" s="40">
+      <c r="B75" s="39">
         <v>15.0</v>
       </c>
-      <c r="C75" s="18">
+      <c r="C75" s="14">
         <v>10.0</v>
       </c>
-      <c r="D75" s="18">
+      <c r="D75" s="14">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52710,16 +52710,16 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76">
-      <c r="A76" s="40" t="s">
-        <v>18</v>
+      <c r="A76" s="39" t="s">
+        <v>21</v>
       </c>
-      <c r="B76" s="40">
+      <c r="B76" s="39">
         <v>20.0</v>
       </c>
-      <c r="C76" s="18">
+      <c r="C76" s="14">
         <v>10.0</v>
       </c>
-      <c r="D76" s="18">
+      <c r="D76" s="14">
         <v>6.0</v>
       </c>
       <c r="E76" s="46">
@@ -52735,8 +52735,8 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="41"/>
-      <c r="B77" s="41"/>
+      <c r="A77" s="40"/>
+      <c r="B77" s="40"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
@@ -52750,8 +52750,8 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="40"/>
-      <c r="B78" s="41"/>
+      <c r="A78" s="39"/>
+      <c r="B78" s="40"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
@@ -52765,8 +52765,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="41"/>
-      <c r="B79" s="41"/>
+      <c r="A79" s="40"/>
+      <c r="B79" s="40"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-09-01T13:12:09.328Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -43,6 +43,9 @@
     <t>Cut(detail)</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>(PS)</t>
   </si>
   <si>
@@ -55,22 +58,16 @@
     <t>(PS -3)</t>
   </si>
   <si>
+    <t>刀壓</t>
+  </si>
+  <si>
     <t>1mm</t>
   </si>
   <si>
     <t>Fill</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
-    <t>刀壓</t>
-  </si>
-  <si>
     <t>2mm</t>
-  </si>
-  <si>
-    <t>3mm</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -79,31 +76,34 @@
     <t>03mm</t>
   </si>
   <si>
+    <t>3mm</t>
+  </si>
+  <si>
     <t>Cut</t>
+  </si>
+  <si>
+    <t>4mm</t>
   </si>
   <si>
     <t>0.3 mm</t>
   </si>
   <si>
+    <t>(0.9 Power)</t>
+  </si>
+  <si>
     <t>PS</t>
   </si>
   <si>
-    <t>4mm</t>
+    <t>甲板紙</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>cut</t>
   </si>
   <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
     <t>Keep Detail</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>６</t>
@@ -351,19 +351,16 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -372,29 +369,20 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -410,6 +398,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -789,14 +789,14 @@
     </row>
     <row r="6">
       <c r="A6" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
-      <c r="E6" s="15"/>
+      <c r="E6" s="14"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -823,8 +823,8 @@
       <c r="E7" s="17">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -849,8 +849,8 @@
       <c r="E8" s="17">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,10 +860,10 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="19"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="9"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
       <c r="E9" s="10"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -877,10 +877,10 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
       <c r="D10" s="9"/>
       <c r="E10" s="10"/>
       <c r="F10" s="4"/>
@@ -909,8 +909,8 @@
       <c r="E11" s="10">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="19"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -987,10 +987,10 @@
       <c r="A15" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="15"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="14"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1014,7 +1014,7 @@
       <c r="D16" s="13">
         <v>1.0</v>
       </c>
-      <c r="E16" s="15"/>
+      <c r="E16" s="14"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1038,7 +1038,7 @@
       <c r="D17" s="13">
         <v>1.0</v>
       </c>
-      <c r="E17" s="15"/>
+      <c r="E17" s="14"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="19"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1067,11 +1067,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1111,9 +1111,9 @@
       <c r="A21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="19"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1143,12 +1143,12 @@
     </row>
     <row r="23">
       <c r="A23" s="12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="15"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="14"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1172,7 +1172,7 @@
       <c r="D24" s="13">
         <v>1.0</v>
       </c>
-      <c r="E24" s="15"/>
+      <c r="E24" s="14"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1184,17 +1184,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="31">
+      <c r="B25" s="27">
         <v>55.0</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="27">
         <v>2.0</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="33"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="29"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="20"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
+      <c r="A26" s="19"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1223,14 +1223,14 @@
     </row>
     <row r="27">
       <c r="A27" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="34">
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="30">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1253,8 +1253,8 @@
       <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="34">
+      <c r="D28" s="19"/>
+      <c r="E28" s="30">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1277,8 +1277,8 @@
       <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="20"/>
-      <c r="E29" s="34">
+      <c r="D29" s="19"/>
+      <c r="E29" s="30">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
+      <c r="A30" s="19"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="20"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
+      <c r="A31" s="19"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17196,7 +17196,7 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -17227,9 +17227,9 @@
         <v>1.0</v>
       </c>
       <c r="E6" s="7"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17252,9 +17252,9 @@
         <v>1.0</v>
       </c>
       <c r="E7" s="11"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17282,12 +17282,12 @@
     </row>
     <row r="9">
       <c r="A9" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="18"/>
+      <c r="E9" s="21"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17312,7 +17312,7 @@
       <c r="D10" s="13">
         <v>1.0</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="21">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17339,7 +17339,7 @@
       <c r="D11" s="13">
         <v>1.0</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="21">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17355,7 +17355,7 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B12" s="13">
         <v>4.0</v>
@@ -17366,7 +17366,7 @@
       <c r="D12" s="13">
         <v>1.0</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="21">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17382,12 +17382,12 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
-      <c r="E13" s="21"/>
+      <c r="E13" s="23"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17412,7 +17412,7 @@
       <c r="D14" s="13">
         <v>1.0</v>
       </c>
-      <c r="E14" s="21"/>
+      <c r="E14" s="23"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17437,7 +17437,7 @@
       <c r="D15" s="13">
         <v>1.0</v>
       </c>
-      <c r="E15" s="21"/>
+      <c r="E15" s="23"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17465,10 +17465,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
@@ -17535,10 +17535,10 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="19"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
       <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -17555,10 +17555,10 @@
       <c r="A21" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="21"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="23"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17583,7 +17583,7 @@
       <c r="D22" s="13">
         <v>1.0</v>
       </c>
-      <c r="E22" s="21"/>
+      <c r="E22" s="23"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17608,7 +17608,7 @@
       <c r="D23" s="13">
         <v>2.0</v>
       </c>
-      <c r="E23" s="21"/>
+      <c r="E23" s="23"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,10 +17621,10 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="19"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
       <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -17639,11 +17639,11 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -17709,10 +17709,10 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="19"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
       <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -17727,12 +17727,12 @@
     </row>
     <row r="29">
       <c r="A29" s="12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="21"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="23"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17757,7 +17757,7 @@
       <c r="D30" s="13">
         <v>1.0</v>
       </c>
-      <c r="E30" s="21"/>
+      <c r="E30" s="23"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17770,16 +17770,16 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="s">
+      <c r="A31" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="27">
         <v>70.0</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="27">
         <v>5.0</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="27">
         <v>1.0</v>
       </c>
       <c r="E31" s="35"/>
@@ -17813,7 +17813,7 @@
     </row>
     <row r="33" ht="20.25" customHeight="1">
       <c r="A33" s="36" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B33" s="37">
         <v>5.0</v>
@@ -17828,7 +17828,7 @@
         <v>46043.55545597222</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G33" s="40"/>
       <c r="H33" s="40"/>
@@ -17876,13 +17876,13 @@
     </row>
     <row r="36">
       <c r="A36" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17905,7 +17905,7 @@
       <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="20"/>
+      <c r="D37" s="19"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17928,7 +17928,7 @@
       <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="20"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34686,7 +34686,7 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="9">
         <v>2.0</v>
@@ -34728,14 +34728,14 @@
     </row>
     <row r="8">
       <c r="A8" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
-      <c r="E8" s="15"/>
+      <c r="E8" s="14"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34762,8 +34762,8 @@
       <c r="E9" s="17">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34788,8 +34788,8 @@
       <c r="E10" s="17">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,10 +34799,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="19"/>
+      <c r="A11" s="18"/>
       <c r="B11" s="9"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
       <c r="E11" s="10"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -34816,7 +34816,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34875,7 +34875,7 @@
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -34892,10 +34892,10 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="19"/>
+      <c r="A16" s="18"/>
       <c r="B16" s="9"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
       <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34909,10 +34909,10 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
       <c r="D17" s="9"/>
       <c r="E17" s="10"/>
       <c r="F17" s="4"/>
@@ -34941,8 +34941,8 @@
       <c r="E18" s="10">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -35000,10 +35000,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="19"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35019,10 +35019,10 @@
       <c r="A22" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="15"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="14"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35046,7 +35046,7 @@
       <c r="D23" s="13">
         <v>1.0</v>
       </c>
-      <c r="E23" s="15"/>
+      <c r="E23" s="14"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35070,7 +35070,7 @@
       <c r="D24" s="13">
         <v>1.0</v>
       </c>
-      <c r="E24" s="15"/>
+      <c r="E24" s="14"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,10 +35082,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="19"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35099,11 +35099,11 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35143,9 +35143,9 @@
       <c r="A28" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35158,10 +35158,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="19"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35175,12 +35175,12 @@
     </row>
     <row r="30">
       <c r="A30" s="12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B30" s="23"/>
-      <c r="C30" s="23"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="15"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="14"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35204,7 +35204,7 @@
       <c r="D31" s="13">
         <v>1.0</v>
       </c>
-      <c r="E31" s="15"/>
+      <c r="E31" s="14"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35216,17 +35216,17 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="30" t="s">
+      <c r="A32" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B32" s="31">
+      <c r="B32" s="27">
         <v>55.0</v>
       </c>
-      <c r="C32" s="31">
+      <c r="C32" s="27">
         <v>2.0</v>
       </c>
-      <c r="D32" s="32"/>
-      <c r="E32" s="33"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="29"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="20"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
+      <c r="A33" s="19"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35255,14 +35255,14 @@
     </row>
     <row r="34">
       <c r="A34" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="34">
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="30">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35285,8 +35285,8 @@
       <c r="C35" s="9">
         <v>100.0</v>
       </c>
-      <c r="D35" s="20"/>
-      <c r="E35" s="34">
+      <c r="D35" s="19"/>
+      <c r="E35" s="30">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35309,8 +35309,8 @@
       <c r="C36" s="9">
         <v>100.0</v>
       </c>
-      <c r="D36" s="20"/>
-      <c r="E36" s="34">
+      <c r="D36" s="19"/>
+      <c r="E36" s="30">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="20"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="20"/>
+      <c r="A37" s="19"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="19"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="20"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
+      <c r="A38" s="19"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,10 +51132,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -51159,8 +51159,8 @@
       <c r="A2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
       <c r="D2" s="9"/>
       <c r="E2" s="7"/>
       <c r="F2" s="4"/>
@@ -51176,10 +51176,10 @@
       <c r="A3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="20">
         <v>60.0</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="20">
         <v>20.0</v>
       </c>
       <c r="D3" s="9">
@@ -51197,9 +51197,9 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
       <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -51212,13 +51212,13 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
       <c r="E5" s="11"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -51279,9 +51279,9 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="5"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
       <c r="E8" s="7"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -51294,7 +51294,7 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -51314,7 +51314,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="9">
-        <v>10.0</v>
+        <v>6.0</v>
       </c>
       <c r="C10" s="9">
         <v>45.0</v>
@@ -51323,7 +51323,7 @@
         <v>1.0</v>
       </c>
       <c r="E10" s="11">
-        <v>46106.73232292824</v>
+        <v>46266.88342763889</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -51348,7 +51348,7 @@
         <v>1.0</v>
       </c>
       <c r="E11" s="11">
-        <v>46266.88338049769</v>
+        <v>46266.88340020833</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="27"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="32"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,11 +51375,11 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="s">
-        <v>22</v>
+      <c r="A13" s="33" t="s">
+        <v>23</v>
       </c>
-      <c r="B13" s="29" t="s">
-        <v>23</v>
+      <c r="B13" s="34" t="s">
+        <v>25</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
@@ -51395,7 +51395,7 @@
     </row>
     <row r="14" ht="20.25" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B14" s="9">
         <v>5.0</v>
@@ -51443,7 +51443,7 @@
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B16" s="9">
         <v>5.0</v>
@@ -51457,8 +51457,8 @@
       <c r="E16" s="11">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="14" t="s">
-        <v>28</v>
+      <c r="F16" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="27"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="32"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,11 +51510,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
       <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -51529,10 +51529,10 @@
       <c r="A20" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="20">
         <v>6.0</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="20">
         <v>45.0</v>
       </c>
       <c r="D20" s="9">
@@ -51554,10 +51554,10 @@
       <c r="A21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="20">
         <v>18.0</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="20">
         <v>20.0</v>
       </c>
       <c r="D21" s="9">
@@ -51577,9 +51577,9 @@
     </row>
     <row r="22">
       <c r="A22" s="8"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
       <c r="E22" s="7"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -51591,14 +51591,14 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="s">
-        <v>10</v>
+      <c r="A23" s="33" t="s">
+        <v>11</v>
       </c>
-      <c r="B23" s="29" t="s">
-        <v>23</v>
+      <c r="B23" s="34" t="s">
+        <v>25</v>
       </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
       <c r="E23" s="11">
         <v>46155.850816817125</v>
       </c>
@@ -51613,12 +51613,12 @@
     </row>
     <row r="24">
       <c r="A24" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="20">
         <v>6.0</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="20">
         <v>50.0</v>
       </c>
       <c r="D24" s="9">
@@ -51640,10 +51640,10 @@
       <c r="A25" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="22">
+      <c r="B25" s="20">
         <v>8.0</v>
       </c>
-      <c r="C25" s="22">
+      <c r="C25" s="20">
         <v>30.0</v>
       </c>
       <c r="D25" s="9">
@@ -51665,10 +51665,10 @@
       <c r="A26" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="22">
+      <c r="B26" s="20">
         <v>10.0</v>
       </c>
-      <c r="C26" s="22">
+      <c r="C26" s="20">
         <v>30.0</v>
       </c>
       <c r="D26" s="9">
@@ -51677,8 +51677,8 @@
       <c r="E26" s="11">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="14" t="s">
-        <v>28</v>
+      <c r="F26" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51692,10 +51692,10 @@
       <c r="A27" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="22">
+      <c r="B27" s="20">
         <v>17.0</v>
       </c>
-      <c r="C27" s="22">
+      <c r="C27" s="20">
         <v>15.0</v>
       </c>
       <c r="D27" s="9">
@@ -51715,9 +51715,9 @@
     </row>
     <row r="28">
       <c r="A28" s="8"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
       <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -51729,14 +51729,14 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="s">
-        <v>13</v>
+      <c r="A29" s="33" t="s">
+        <v>15</v>
       </c>
-      <c r="B29" s="29" t="s">
-        <v>23</v>
+      <c r="B29" s="34" t="s">
+        <v>25</v>
       </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
       <c r="E29" s="7"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -51749,12 +51749,12 @@
     </row>
     <row r="30">
       <c r="A30" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
-      <c r="B30" s="22">
+      <c r="B30" s="20">
         <v>6.0</v>
       </c>
-      <c r="C30" s="22">
+      <c r="C30" s="20">
         <v>50.0</v>
       </c>
       <c r="D30" s="9">
@@ -51776,10 +51776,10 @@
       <c r="A31" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="22">
+      <c r="B31" s="20">
         <v>8.0</v>
       </c>
-      <c r="C31" s="22">
+      <c r="C31" s="20">
         <v>30.0</v>
       </c>
       <c r="D31" s="9">
@@ -51799,10 +51799,10 @@
       <c r="A32" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B32" s="22">
+      <c r="B32" s="20">
         <v>15.0</v>
       </c>
-      <c r="C32" s="22">
+      <c r="C32" s="20">
         <v>10.0</v>
       </c>
       <c r="D32" s="9">
@@ -51822,9 +51822,9 @@
     </row>
     <row r="33">
       <c r="A33" s="8"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
       <c r="E33" s="7"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -51837,12 +51837,12 @@
     </row>
     <row r="34">
       <c r="A34" s="12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
       <c r="D34" s="13"/>
-      <c r="E34" s="21"/>
+      <c r="E34" s="23"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51865,7 +51865,7 @@
       <c r="D35" s="41">
         <v>1.0</v>
       </c>
-      <c r="E35" s="18">
+      <c r="E35" s="21">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51890,7 +51890,7 @@
       <c r="D36" s="41">
         <v>1.0</v>
       </c>
-      <c r="E36" s="21"/>
+      <c r="E36" s="23"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51902,7 +51902,7 @@
     </row>
     <row r="37">
       <c r="A37" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B37" s="9">
         <v>10.0</v>
@@ -51926,10 +51926,10 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="19"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="7"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -51944,9 +51944,9 @@
       <c r="A39" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
       <c r="E39" s="7"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -51984,9 +51984,9 @@
     </row>
     <row r="41">
       <c r="A41" s="5"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
+      <c r="B41" s="19"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
       <c r="E41" s="7"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -52001,9 +52001,9 @@
       <c r="A42" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
+      <c r="B42" s="19"/>
+      <c r="C42" s="19"/>
+      <c r="D42" s="19"/>
       <c r="E42" s="7"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -52080,7 +52080,7 @@
       <c r="E45" s="11">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="14" t="s">
+      <c r="F45" s="15" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52093,9 +52093,9 @@
     </row>
     <row r="46">
       <c r="A46" s="42"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
+      <c r="B46" s="19"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
       <c r="E46" s="7"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -52108,11 +52108,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
       <c r="E47" s="7"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
@@ -52150,9 +52150,9 @@
     </row>
     <row r="49">
       <c r="A49" s="42"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
       <c r="E49" s="7"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
@@ -52165,11 +52165,11 @@
     </row>
     <row r="50">
       <c r="A50" s="42" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
       <c r="E50" s="7"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -52232,9 +52232,9 @@
     </row>
     <row r="53">
       <c r="A53" s="42"/>
-      <c r="B53" s="20"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
+      <c r="B53" s="19"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="19"/>
       <c r="E53" s="7"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
@@ -52249,9 +52249,9 @@
       <c r="A54" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
       <c r="E54" s="7"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
@@ -52264,15 +52264,15 @@
     </row>
     <row r="55">
       <c r="A55" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
-      <c r="B55" s="22">
+      <c r="B55" s="20">
         <v>70.0</v>
       </c>
-      <c r="C55" s="22">
+      <c r="C55" s="20">
         <v>300.0</v>
       </c>
-      <c r="D55" s="22">
+      <c r="D55" s="20">
         <v>1.0</v>
       </c>
       <c r="E55" s="11">
@@ -52291,13 +52291,13 @@
       <c r="A56" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B56" s="22">
+      <c r="B56" s="20">
         <v>10.0</v>
       </c>
-      <c r="C56" s="22">
+      <c r="C56" s="20">
         <v>20.0</v>
       </c>
-      <c r="D56" s="22">
+      <c r="D56" s="20">
         <v>1.0</v>
       </c>
       <c r="E56" s="11">
@@ -52316,13 +52316,13 @@
       <c r="A57" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B57" s="22">
+      <c r="B57" s="20">
         <v>70.0</v>
       </c>
-      <c r="C57" s="22">
+      <c r="C57" s="20">
         <v>8.0</v>
       </c>
-      <c r="D57" s="22">
+      <c r="D57" s="20">
         <v>1.0</v>
       </c>
       <c r="E57" s="11">
@@ -52380,8 +52380,8 @@
       <c r="B60" s="9">
         <v>100.0</v>
       </c>
-      <c r="C60" s="20"/>
-      <c r="D60" s="20"/>
+      <c r="C60" s="19"/>
+      <c r="D60" s="19"/>
       <c r="E60" s="11">
         <v>45946.87887299768</v>
       </c>
@@ -52418,10 +52418,10 @@
       <c r="B62" s="39">
         <v>100.0</v>
       </c>
-      <c r="C62" s="14">
+      <c r="C62" s="15">
         <v>1.0</v>
       </c>
-      <c r="D62" s="14">
+      <c r="D62" s="15">
         <v>2.0</v>
       </c>
       <c r="E62" s="46">
@@ -52475,10 +52475,10 @@
       <c r="B65" s="39">
         <v>50.0</v>
       </c>
-      <c r="C65" s="14">
+      <c r="C65" s="15">
         <v>20.0</v>
       </c>
-      <c r="D65" s="14">
+      <c r="D65" s="15">
         <v>1.0</v>
       </c>
       <c r="E65" s="46">
@@ -52500,7 +52500,7 @@
       <c r="B66" s="39">
         <v>15.0</v>
       </c>
-      <c r="C66" s="14">
+      <c r="C66" s="15">
         <v>16.0</v>
       </c>
       <c r="D66" s="4"/>
@@ -52536,7 +52536,7 @@
         <v>40</v>
       </c>
       <c r="B68" s="39" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -52559,10 +52559,10 @@
       <c r="B69" s="39">
         <v>5.0</v>
       </c>
-      <c r="C69" s="14">
+      <c r="C69" s="15">
         <v>80.0</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69" s="15">
         <v>1.0</v>
       </c>
       <c r="E69" s="46">
@@ -52584,10 +52584,10 @@
       <c r="B70" s="39">
         <v>15.0</v>
       </c>
-      <c r="C70" s="14">
+      <c r="C70" s="15">
         <v>10.0</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70" s="15">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52609,10 +52609,10 @@
       <c r="B71" s="39">
         <v>30.0</v>
       </c>
-      <c r="C71" s="14">
+      <c r="C71" s="15">
         <v>10.0</v>
       </c>
-      <c r="D71" s="14">
+      <c r="D71" s="15">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52670,10 +52670,10 @@
       <c r="B74" s="39">
         <v>5.0</v>
       </c>
-      <c r="C74" s="14">
+      <c r="C74" s="15">
         <v>80.0</v>
       </c>
-      <c r="D74" s="14">
+      <c r="D74" s="15">
         <v>1.0</v>
       </c>
       <c r="E74" s="4"/>
@@ -52693,10 +52693,10 @@
       <c r="B75" s="39">
         <v>15.0</v>
       </c>
-      <c r="C75" s="14">
+      <c r="C75" s="15">
         <v>10.0</v>
       </c>
-      <c r="D75" s="14">
+      <c r="D75" s="15">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52716,10 +52716,10 @@
       <c r="B76" s="39">
         <v>20.0</v>
       </c>
-      <c r="C76" s="14">
+      <c r="C76" s="15">
         <v>10.0</v>
       </c>
-      <c r="D76" s="14">
+      <c r="D76" s="15">
         <v>6.0</v>
       </c>
       <c r="E76" s="46">

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-10-23T06:57:35.079Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -31,43 +31,37 @@
     <t>最後更新日期</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
+    <t>刀壓</t>
+  </si>
+  <si>
     <t>0.3mm</t>
   </si>
   <si>
     <t>Line</t>
   </si>
   <si>
+    <t>Cut(detail)</t>
+  </si>
+  <si>
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
+    <t>FILL</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
   </si>
   <si>
     <t>(PS)</t>
   </si>
   <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
-  </si>
-  <si>
-    <t>刀壓</t>
-  </si>
-  <si>
     <t>1mm</t>
-  </si>
-  <si>
-    <t>Fill</t>
-  </si>
-  <si>
-    <t>2mm</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -76,16 +70,22 @@
     <t>03mm</t>
   </si>
   <si>
-    <t>3mm</t>
+    <t>2mm</t>
   </si>
   <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>4mm</t>
+    <t>0.3 mm</t>
   </si>
   <si>
-    <t>0.3 mm</t>
+    <t>Fill</t>
+  </si>
+  <si>
+    <t>3mm</t>
+  </si>
+  <si>
+    <t>4mm</t>
   </si>
   <si>
     <t>(0.9 Power)</t>
@@ -94,16 +94,16 @@
     <t>PS</t>
   </si>
   <si>
+    <t>cut</t>
+  </si>
+  <si>
+    <t>Keep Detail</t>
+  </si>
+  <si>
     <t>甲板紙</t>
   </si>
   <si>
     <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>cut</t>
-  </si>
-  <si>
-    <t>Keep Detail</t>
   </si>
   <si>
     <t>６</t>
@@ -209,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -330,11 +330,11 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -342,7 +342,7 @@
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -351,11 +351,11 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -363,14 +363,14 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -381,8 +381,7 @@
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -397,16 +396,17 @@
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -708,7 +708,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -722,8 +722,8 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>6</v>
+      <c r="A3" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B3" s="9">
         <v>2.0</v>
@@ -748,8 +748,8 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>7</v>
+      <c r="A4" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B4" s="9">
         <v>25.0</v>
@@ -789,14 +789,14 @@
     </row>
     <row r="6">
       <c r="A6" s="12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
-      <c r="E6" s="14"/>
+      <c r="E6" s="15"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -809,7 +809,7 @@
     </row>
     <row r="7">
       <c r="A7" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B7" s="13">
         <v>4.0</v>
@@ -823,8 +823,8 @@
       <c r="E7" s="17">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -835,7 +835,7 @@
     </row>
     <row r="8">
       <c r="A8" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B8" s="13">
         <v>25.0</v>
@@ -849,8 +849,8 @@
       <c r="E8" s="17">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,10 +860,10 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="18"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="9"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
       <c r="E9" s="10"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
@@ -879,8 +879,8 @@
       <c r="A10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
       <c r="D10" s="9"/>
       <c r="E10" s="10"/>
       <c r="F10" s="4"/>
@@ -894,8 +894,8 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>6</v>
+      <c r="A11" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B11" s="9">
         <v>5.0</v>
@@ -909,8 +909,8 @@
       <c r="E11" s="10">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,8 +920,8 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
-        <v>6</v>
+      <c r="A12" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B12" s="9">
         <v>5.0</v>
@@ -944,8 +944,8 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>7</v>
+      <c r="A13" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B13" s="9">
         <v>32.0</v>
@@ -968,10 +968,10 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="18"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
+      <c r="A14" s="19"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
       <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -985,12 +985,12 @@
     </row>
     <row r="15">
       <c r="A15" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B15" s="22"/>
       <c r="C15" s="22"/>
       <c r="D15" s="22"/>
-      <c r="E15" s="14"/>
+      <c r="E15" s="15"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1003,7 +1003,7 @@
     </row>
     <row r="16">
       <c r="A16" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B16" s="13">
         <v>5.0</v>
@@ -1014,7 +1014,7 @@
       <c r="D16" s="13">
         <v>1.0</v>
       </c>
-      <c r="E16" s="14"/>
+      <c r="E16" s="15"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1027,7 +1027,7 @@
     </row>
     <row r="17">
       <c r="A17" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B17" s="13">
         <v>50.0</v>
@@ -1038,7 +1038,7 @@
       <c r="D17" s="13">
         <v>1.0</v>
       </c>
-      <c r="E17" s="14"/>
+      <c r="E17" s="15"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,10 +1050,10 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="18"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
+      <c r="A18" s="19"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
       <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1067,11 +1067,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
       <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1084,8 +1084,8 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>6</v>
+      <c r="A20" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B20" s="9">
         <v>5.0</v>
@@ -1108,12 +1108,12 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>7</v>
+      <c r="A21" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -1126,10 +1126,10 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
+      <c r="A22" s="19"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
       <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -1143,12 +1143,12 @@
     </row>
     <row r="23">
       <c r="A23" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
       <c r="D23" s="22"/>
-      <c r="E23" s="14"/>
+      <c r="E23" s="15"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1161,7 +1161,7 @@
     </row>
     <row r="24">
       <c r="A24" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B24" s="13">
         <v>5.0</v>
@@ -1172,7 +1172,7 @@
       <c r="D24" s="13">
         <v>1.0</v>
       </c>
-      <c r="E24" s="14"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1184,17 +1184,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="26" t="s">
-        <v>7</v>
+      <c r="A25" s="25" t="s">
+        <v>10</v>
       </c>
-      <c r="B25" s="27">
+      <c r="B25" s="26">
         <v>55.0</v>
       </c>
-      <c r="C25" s="27">
+      <c r="C25" s="26">
         <v>2.0</v>
       </c>
-      <c r="D25" s="28"/>
-      <c r="E25" s="29"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="28"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="19"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
+      <c r="A26" s="20"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1223,14 +1223,14 @@
     </row>
     <row r="27">
       <c r="A27" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B27" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="30">
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="31">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1245,7 +1245,7 @@
     </row>
     <row r="28">
       <c r="A28" s="9" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B28" s="9">
         <v>2.0</v>
@@ -1253,8 +1253,8 @@
       <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="30">
+      <c r="D28" s="20"/>
+      <c r="E28" s="31">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1269,7 +1269,7 @@
     </row>
     <row r="29">
       <c r="A29" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B29" s="9">
         <v>20.0</v>
@@ -1277,8 +1277,8 @@
       <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="19"/>
-      <c r="E29" s="30">
+      <c r="D29" s="20"/>
+      <c r="E29" s="31">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="19"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="19"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17128,9 +17128,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17143,8 +17143,8 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>6</v>
+      <c r="A3" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B3" s="9">
         <v>3.0</v>
@@ -17155,7 +17155,7 @@
       <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="14">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17170,8 +17170,8 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>7</v>
+      <c r="A4" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B4" s="9">
         <v>20.0</v>
@@ -17182,7 +17182,7 @@
       <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="7"/>
+      <c r="E4" s="8"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17195,13 +17195,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>10</v>
+      <c r="A5" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="7"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17214,8 +17214,8 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>6</v>
+      <c r="A6" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B6" s="9">
         <v>2.0</v>
@@ -17226,10 +17226,10 @@
       <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,8 +17239,8 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>7</v>
+      <c r="A7" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B7" s="9">
         <v>18.0</v>
@@ -17251,10 +17251,10 @@
       <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17268,7 +17268,7 @@
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
-      <c r="E8" s="11"/>
+      <c r="E8" s="14"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17282,7 +17282,7 @@
     </row>
     <row r="9">
       <c r="A9" s="12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
@@ -17301,7 +17301,7 @@
     </row>
     <row r="10">
       <c r="A10" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B10" s="13">
         <v>4.0</v>
@@ -17328,7 +17328,7 @@
     </row>
     <row r="11">
       <c r="A11" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B11" s="13">
         <v>25.0</v>
@@ -17355,7 +17355,7 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B12" s="13">
         <v>4.0</v>
@@ -17382,7 +17382,7 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -17401,7 +17401,7 @@
     </row>
     <row r="14">
       <c r="A14" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B14" s="13">
         <v>2.0</v>
@@ -17426,7 +17426,7 @@
     </row>
     <row r="15">
       <c r="A15" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B15" s="13">
         <v>18.0</v>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="24"/>
-      <c r="E16" s="7"/>
+      <c r="A16" s="30"/>
+      <c r="E16" s="8"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17467,12 +17467,12 @@
       <c r="A17" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="25" t="s">
-        <v>10</v>
+      <c r="B17" s="34" t="s">
+        <v>14</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
-      <c r="E17" s="7"/>
+      <c r="E17" s="8"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17485,8 +17485,8 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>6</v>
+      <c r="A18" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B18" s="9">
         <v>5.0</v>
@@ -17497,7 +17497,7 @@
       <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="7"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17510,8 +17510,8 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>7</v>
+      <c r="A19" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B19" s="9">
         <v>40.0</v>
@@ -17522,7 +17522,7 @@
       <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="7"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="18"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="7"/>
+      <c r="A20" s="19"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17553,7 +17553,7 @@
     </row>
     <row r="21">
       <c r="A21" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="22"/>
       <c r="C21" s="22"/>
@@ -17572,7 +17572,7 @@
     </row>
     <row r="22">
       <c r="A22" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B22" s="13">
         <v>8.0</v>
@@ -17597,7 +17597,7 @@
     </row>
     <row r="23">
       <c r="A23" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B23" s="13">
         <v>55.0</v>
@@ -17621,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="7"/>
+      <c r="A24" s="19"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="8"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17639,12 +17639,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="7"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="8"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17657,8 +17657,8 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>6</v>
+      <c r="A26" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B26" s="9">
         <v>10.0</v>
@@ -17669,7 +17669,7 @@
       <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="7"/>
+      <c r="E26" s="8"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17682,8 +17682,8 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>7</v>
+      <c r="A27" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B27" s="9">
         <v>60.0</v>
@@ -17694,7 +17694,7 @@
       <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="14">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="18"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="7"/>
+      <c r="A28" s="19"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17727,7 +17727,7 @@
     </row>
     <row r="29">
       <c r="A29" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
@@ -17746,7 +17746,7 @@
     </row>
     <row r="30">
       <c r="A30" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B30" s="13">
         <v>18.0</v>
@@ -17770,16 +17770,16 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="26" t="s">
-        <v>7</v>
+      <c r="A31" s="25" t="s">
+        <v>10</v>
       </c>
-      <c r="B31" s="27">
+      <c r="B31" s="26">
         <v>70.0</v>
       </c>
-      <c r="C31" s="27">
+      <c r="C31" s="26">
         <v>5.0</v>
       </c>
-      <c r="D31" s="27">
+      <c r="D31" s="26">
         <v>1.0</v>
       </c>
       <c r="E31" s="35"/>
@@ -17813,7 +17813,7 @@
     </row>
     <row r="33" ht="20.25" customHeight="1">
       <c r="A33" s="36" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B33" s="37">
         <v>5.0</v>
@@ -17828,7 +17828,7 @@
         <v>46043.55545597222</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G33" s="40"/>
       <c r="H33" s="40"/>
@@ -17876,13 +17876,13 @@
     </row>
     <row r="36">
       <c r="A36" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17897,7 +17897,7 @@
     </row>
     <row r="37">
       <c r="A37" s="9" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B37" s="9">
         <v>2.0</v>
@@ -17905,7 +17905,7 @@
       <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="19"/>
+      <c r="D37" s="20"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17920,7 +17920,7 @@
     </row>
     <row r="38">
       <c r="A38" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B38" s="9">
         <v>20.0</v>
@@ -17928,7 +17928,7 @@
       <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="19"/>
+      <c r="D38" s="20"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34593,7 +34593,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="4"/>
@@ -34607,8 +34607,8 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>6</v>
+      <c r="A3" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B3" s="9">
         <v>2.0</v>
@@ -34633,8 +34633,8 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>8</v>
+      <c r="A4" s="7" t="s">
+        <v>9</v>
       </c>
       <c r="B4" s="9">
         <v>10.0</v>
@@ -34659,8 +34659,8 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>7</v>
+      <c r="A5" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B5" s="9">
         <v>20.0</v>
@@ -34685,8 +34685,8 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>12</v>
+      <c r="A6" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="B6" s="9">
         <v>2.0</v>
@@ -34728,14 +34728,14 @@
     </row>
     <row r="8">
       <c r="A8" s="12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
-      <c r="E8" s="14"/>
+      <c r="E8" s="15"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34748,7 +34748,7 @@
     </row>
     <row r="9">
       <c r="A9" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B9" s="13">
         <v>4.0</v>
@@ -34762,8 +34762,8 @@
       <c r="E9" s="17">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34774,7 +34774,7 @@
     </row>
     <row r="10">
       <c r="A10" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B10" s="13">
         <v>20.0</v>
@@ -34788,8 +34788,8 @@
       <c r="E10" s="17">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,10 +34799,10 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="18"/>
+      <c r="A11" s="19"/>
       <c r="B11" s="9"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
       <c r="E11" s="10"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -34816,7 +34816,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="4"/>
@@ -34830,8 +34830,8 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>6</v>
+      <c r="A13" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -34848,8 +34848,8 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
-        <v>7</v>
+      <c r="A14" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B14" s="9">
         <v>20.0</v>
@@ -34874,8 +34874,8 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>12</v>
+      <c r="A15" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -34892,10 +34892,10 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="18"/>
+      <c r="A16" s="19"/>
       <c r="B16" s="9"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
       <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -34911,8 +34911,8 @@
       <c r="A17" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
       <c r="D17" s="9"/>
       <c r="E17" s="10"/>
       <c r="F17" s="4"/>
@@ -34926,8 +34926,8 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>6</v>
+      <c r="A18" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B18" s="9">
         <v>5.0</v>
@@ -34941,8 +34941,8 @@
       <c r="E18" s="10">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34952,8 +34952,8 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>6</v>
+      <c r="A19" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B19" s="9">
         <v>5.0</v>
@@ -34976,8 +34976,8 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>7</v>
+      <c r="A20" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B20" s="9">
         <v>32.0</v>
@@ -35000,10 +35000,10 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="18"/>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
+      <c r="A21" s="19"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
       <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -35017,12 +35017,12 @@
     </row>
     <row r="22">
       <c r="A22" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B22" s="22"/>
       <c r="C22" s="22"/>
       <c r="D22" s="22"/>
-      <c r="E22" s="14"/>
+      <c r="E22" s="15"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35035,7 +35035,7 @@
     </row>
     <row r="23">
       <c r="A23" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B23" s="13">
         <v>5.0</v>
@@ -35046,7 +35046,7 @@
       <c r="D23" s="13">
         <v>1.0</v>
       </c>
-      <c r="E23" s="14"/>
+      <c r="E23" s="15"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35059,7 +35059,7 @@
     </row>
     <row r="24">
       <c r="A24" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B24" s="13">
         <v>50.0</v>
@@ -35070,7 +35070,7 @@
       <c r="D24" s="13">
         <v>1.0</v>
       </c>
-      <c r="E24" s="14"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,10 +35082,10 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="18"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
+      <c r="A25" s="19"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
       <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -35099,11 +35099,11 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
       <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -35116,8 +35116,8 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>6</v>
+      <c r="A27" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B27" s="9">
         <v>5.0</v>
@@ -35140,12 +35140,12 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>7</v>
+      <c r="A28" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -35158,10 +35158,10 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="18"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
+      <c r="A29" s="19"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
       <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -35175,12 +35175,12 @@
     </row>
     <row r="30">
       <c r="A30" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B30" s="22"/>
       <c r="C30" s="22"/>
       <c r="D30" s="22"/>
-      <c r="E30" s="14"/>
+      <c r="E30" s="15"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35193,7 +35193,7 @@
     </row>
     <row r="31">
       <c r="A31" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B31" s="13">
         <v>5.0</v>
@@ -35204,7 +35204,7 @@
       <c r="D31" s="13">
         <v>1.0</v>
       </c>
-      <c r="E31" s="14"/>
+      <c r="E31" s="15"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35216,17 +35216,17 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="26" t="s">
-        <v>7</v>
+      <c r="A32" s="25" t="s">
+        <v>10</v>
       </c>
-      <c r="B32" s="27">
+      <c r="B32" s="26">
         <v>55.0</v>
       </c>
-      <c r="C32" s="27">
+      <c r="C32" s="26">
         <v>2.0</v>
       </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="29"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="28"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="19"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35255,14 +35255,14 @@
     </row>
     <row r="34">
       <c r="A34" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B34" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="30">
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="31">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35277,7 +35277,7 @@
     </row>
     <row r="35">
       <c r="A35" s="9" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B35" s="9">
         <v>2.0</v>
@@ -35285,8 +35285,8 @@
       <c r="C35" s="9">
         <v>100.0</v>
       </c>
-      <c r="D35" s="19"/>
-      <c r="E35" s="30">
+      <c r="D35" s="20"/>
+      <c r="E35" s="31">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35301,7 +35301,7 @@
     </row>
     <row r="36">
       <c r="A36" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B36" s="9">
         <v>20.0</v>
@@ -35309,8 +35309,8 @@
       <c r="C36" s="9">
         <v>100.0</v>
       </c>
-      <c r="D36" s="19"/>
-      <c r="E36" s="30">
+      <c r="D36" s="20"/>
+      <c r="E36" s="31">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="19"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="19"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
+      <c r="A38" s="20"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,10 +51132,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -51156,13 +51156,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>6</v>
+      <c r="A2" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
       <c r="D2" s="9"/>
-      <c r="E2" s="7"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51173,19 +51173,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>7</v>
+      <c r="A3" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B3" s="20">
+      <c r="B3" s="11">
         <v>60.0</v>
       </c>
-      <c r="C3" s="20">
+      <c r="C3" s="11">
         <v>20.0</v>
       </c>
       <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="7"/>
+      <c r="E3" s="8"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51197,10 +51197,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="7"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="8"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51212,14 +51212,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="11"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="14"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51230,8 +51230,8 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>6</v>
+      <c r="A6" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B6" s="9">
         <v>6.0</v>
@@ -51240,7 +51240,7 @@
         <v>100.0</v>
       </c>
       <c r="D6" s="9"/>
-      <c r="E6" s="11">
+      <c r="E6" s="14">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51253,8 +51253,8 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="8" t="s">
-        <v>21</v>
+      <c r="A7" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="B7" s="9">
         <v>8.0</v>
@@ -51265,7 +51265,7 @@
       <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="14">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51279,10 +51279,10 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="5"/>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="7"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="8"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51294,12 +51294,12 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
-      <c r="E9" s="7"/>
+      <c r="E9" s="8"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51310,8 +51310,8 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>6</v>
+      <c r="A10" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B10" s="9">
         <v>6.0</v>
@@ -51322,7 +51322,7 @@
       <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="14">
         <v>46266.88342763889</v>
       </c>
       <c r="F10" s="4"/>
@@ -51335,8 +51335,8 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>21</v>
+      <c r="A11" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="B11" s="9">
         <v>13.0</v>
@@ -51347,7 +51347,7 @@
       <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="14">
         <v>46266.88340020833</v>
       </c>
       <c r="F11" s="4"/>
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="31"/>
-      <c r="D12" s="31"/>
-      <c r="E12" s="32"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="29"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,15 +51375,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="s">
-        <v>23</v>
+      <c r="A13" s="32" t="s">
+        <v>20</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="33" t="s">
         <v>25</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="11"/>
+      <c r="E13" s="14"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51394,8 +51394,8 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14" ht="20.25" customHeight="1">
-      <c r="A14" s="8" t="s">
-        <v>16</v>
+      <c r="A14" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="B14" s="9">
         <v>5.0</v>
@@ -51406,7 +51406,7 @@
       <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="14">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51419,8 +51419,8 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>6</v>
+      <c r="A15" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B15" s="9">
         <v>5.0</v>
@@ -51431,7 +51431,7 @@
       <c r="D15" s="9">
         <v>1.0</v>
       </c>
-      <c r="E15" s="11"/>
+      <c r="E15" s="14"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51442,8 +51442,8 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>28</v>
+      <c r="A16" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="B16" s="9">
         <v>5.0</v>
@@ -51454,11 +51454,11 @@
       <c r="D16" s="9">
         <v>4.0</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="14">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="15" t="s">
-        <v>29</v>
+      <c r="F16" s="18" t="s">
+        <v>27</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51469,8 +51469,8 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
-        <v>21</v>
+      <c r="A17" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="B17" s="9">
         <v>12.0</v>
@@ -51481,7 +51481,7 @@
       <c r="D17" s="9">
         <v>1.0</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="14">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="32"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="29"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,12 +51510,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="7"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51526,19 +51526,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>6</v>
+      <c r="A20" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B20" s="20">
+      <c r="B20" s="11">
         <v>6.0</v>
       </c>
-      <c r="C20" s="20">
+      <c r="C20" s="11">
         <v>45.0</v>
       </c>
       <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="14">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51551,19 +51551,19 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>7</v>
+      <c r="A21" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B21" s="20">
+      <c r="B21" s="11">
         <v>18.0</v>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="11">
         <v>20.0</v>
       </c>
       <c r="D21" s="9">
         <v>1.0</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="14">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51576,11 +51576,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="8"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="7"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="8"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51591,15 +51591,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="33" t="s">
-        <v>11</v>
+      <c r="A23" s="32" t="s">
+        <v>12</v>
       </c>
-      <c r="B23" s="34" t="s">
+      <c r="B23" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="11">
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="14">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51612,19 +51612,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>16</v>
+      <c r="A24" s="7" t="s">
+        <v>21</v>
       </c>
-      <c r="B24" s="20">
+      <c r="B24" s="11">
         <v>6.0</v>
       </c>
-      <c r="C24" s="20">
+      <c r="C24" s="11">
         <v>50.0</v>
       </c>
       <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="14">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51637,19 +51637,19 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>6</v>
+      <c r="A25" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="11">
         <v>8.0</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="11">
         <v>30.0</v>
       </c>
       <c r="D25" s="9">
         <v>1.0</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="14">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51662,23 +51662,23 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>21</v>
+      <c r="A26" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B26" s="20">
+      <c r="B26" s="11">
         <v>10.0</v>
       </c>
-      <c r="C26" s="20">
+      <c r="C26" s="11">
         <v>30.0</v>
       </c>
       <c r="D26" s="9">
         <v>4.0</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="14">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="15" t="s">
-        <v>29</v>
+      <c r="F26" s="18" t="s">
+        <v>27</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51689,19 +51689,19 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>21</v>
+      <c r="A27" s="7" t="s">
+        <v>19</v>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="11">
         <v>17.0</v>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="11">
         <v>15.0</v>
       </c>
       <c r="D27" s="9">
         <v>1.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="14">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51714,11 +51714,11 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="7"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51729,15 +51729,15 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="33" t="s">
+      <c r="A29" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B29" s="34" t="s">
+      <c r="B29" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="7"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="8"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51748,19 +51748,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>16</v>
+      <c r="A30" s="7" t="s">
+        <v>21</v>
       </c>
-      <c r="B30" s="20">
+      <c r="B30" s="11">
         <v>6.0</v>
       </c>
-      <c r="C30" s="20">
+      <c r="C30" s="11">
         <v>50.0</v>
       </c>
       <c r="D30" s="9">
         <v>1.0</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="14">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51773,19 +51773,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
-        <v>6</v>
+      <c r="A31" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B31" s="20">
+      <c r="B31" s="11">
         <v>8.0</v>
       </c>
-      <c r="C31" s="20">
+      <c r="C31" s="11">
         <v>30.0</v>
       </c>
       <c r="D31" s="9">
         <v>1.0</v>
       </c>
-      <c r="E31" s="7"/>
+      <c r="E31" s="8"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51796,19 +51796,19 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
-        <v>7</v>
+      <c r="A32" s="7" t="s">
+        <v>10</v>
       </c>
-      <c r="B32" s="20">
+      <c r="B32" s="11">
         <v>15.0</v>
       </c>
-      <c r="C32" s="20">
+      <c r="C32" s="11">
         <v>10.0</v>
       </c>
       <c r="D32" s="9">
         <v>2.0</v>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="14">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51821,11 +51821,11 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="8"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="7"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="8"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51854,7 +51854,7 @@
     </row>
     <row r="35">
       <c r="A35" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B35" s="41" t="s">
         <v>30</v>
@@ -51879,7 +51879,7 @@
     </row>
     <row r="36">
       <c r="A36" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B36" s="41">
         <v>30.0</v>
@@ -51901,8 +51901,8 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>16</v>
+      <c r="A37" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="B37" s="9">
         <v>10.0</v>
@@ -51913,7 +51913,7 @@
       <c r="D37" s="9">
         <v>1.0</v>
       </c>
-      <c r="E37" s="11">
+      <c r="E37" s="14">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51926,11 +51926,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="18"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="7"/>
+      <c r="A38" s="19"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="8"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51944,10 +51944,10 @@
       <c r="A39" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="19"/>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="7"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="8"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51958,8 +51958,8 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="s">
-        <v>7</v>
+      <c r="A40" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B40" s="9">
         <v>40.0</v>
@@ -51970,7 +51970,7 @@
       <c r="D40" s="9">
         <v>1.0</v>
       </c>
-      <c r="E40" s="11">
+      <c r="E40" s="14">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51984,10 +51984,10 @@
     </row>
     <row r="41">
       <c r="A41" s="5"/>
-      <c r="B41" s="19"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="7"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="8"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51999,12 +51999,12 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
-      <c r="B42" s="19"/>
-      <c r="C42" s="19"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="7"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="8"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -52015,8 +52015,8 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="s">
-        <v>6</v>
+      <c r="A43" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B43" s="9">
         <v>9.0</v>
@@ -52027,7 +52027,7 @@
       <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="11">
+      <c r="E43" s="14">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52040,8 +52040,8 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="s">
-        <v>7</v>
+      <c r="A44" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B44" s="9">
         <v>55.0</v>
@@ -52052,7 +52052,7 @@
       <c r="D44" s="9">
         <v>1.0</v>
       </c>
-      <c r="E44" s="11">
+      <c r="E44" s="14">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52065,8 +52065,8 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="s">
-        <v>6</v>
+      <c r="A45" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B45" s="9">
         <v>10.0</v>
@@ -52077,10 +52077,10 @@
       <c r="D45" s="9">
         <v>1.0</v>
       </c>
-      <c r="E45" s="11">
+      <c r="E45" s="14">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="15" t="s">
+      <c r="F45" s="18" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52093,10 +52093,10 @@
     </row>
     <row r="46">
       <c r="A46" s="42"/>
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="7"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="8"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52108,12 +52108,12 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
-      <c r="B47" s="19"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="7"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="8"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52124,8 +52124,8 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="s">
-        <v>7</v>
+      <c r="A48" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B48" s="9">
         <v>55.0</v>
@@ -52136,7 +52136,7 @@
       <c r="D48" s="9">
         <v>1.0</v>
       </c>
-      <c r="E48" s="11">
+      <c r="E48" s="14">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52150,10 +52150,10 @@
     </row>
     <row r="49">
       <c r="A49" s="42"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="7"/>
+      <c r="B49" s="20"/>
+      <c r="C49" s="20"/>
+      <c r="D49" s="20"/>
+      <c r="E49" s="8"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52164,13 +52164,11 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B50" s="19"/>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="7"/>
+      <c r="A50" s="42"/>
+      <c r="B50" s="20"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="20"/>
+      <c r="E50" s="8"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52181,21 +52179,13 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="s">
-        <v>7</v>
+      <c r="A51" s="42" t="s">
+        <v>23</v>
       </c>
-      <c r="B51" s="9">
-        <v>60.0</v>
-      </c>
-      <c r="C51" s="9">
-        <v>10.0</v>
-      </c>
-      <c r="D51" s="9">
-        <v>1.0</v>
-      </c>
-      <c r="E51" s="11">
-        <v>46203.63265940972</v>
-      </c>
+      <c r="B51" s="20"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="8"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52206,20 +52196,20 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="s">
-        <v>6</v>
+      <c r="A52" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B52" s="9">
-        <v>10.0</v>
+        <v>60.0</v>
       </c>
       <c r="C52" s="9">
-        <v>50.0</v>
+        <v>10.0</v>
       </c>
       <c r="D52" s="9">
         <v>1.0</v>
       </c>
-      <c r="E52" s="11">
-        <v>46253.61151159722</v>
+      <c r="E52" s="14">
+        <v>46203.63265940972</v>
       </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -52231,11 +52221,21 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="42"/>
-      <c r="B53" s="19"/>
-      <c r="C53" s="19"/>
-      <c r="D53" s="19"/>
-      <c r="E53" s="7"/>
+      <c r="A53" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B53" s="9">
+        <v>10.0</v>
+      </c>
+      <c r="C53" s="9">
+        <v>50.0</v>
+      </c>
+      <c r="D53" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="E53" s="14">
+        <v>46253.61151159722</v>
+      </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -52246,13 +52246,11 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="42" t="s">
-        <v>33</v>
-      </c>
-      <c r="B54" s="19"/>
-      <c r="C54" s="19"/>
-      <c r="D54" s="19"/>
-      <c r="E54" s="7"/>
+      <c r="A54" s="42"/>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
+      <c r="E54" s="8"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52263,21 +52261,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="s">
-        <v>12</v>
+      <c r="A55" s="42" t="s">
+        <v>33</v>
       </c>
-      <c r="B55" s="20">
-        <v>70.0</v>
-      </c>
-      <c r="C55" s="20">
-        <v>300.0</v>
-      </c>
-      <c r="D55" s="20">
-        <v>1.0</v>
-      </c>
-      <c r="E55" s="11">
-        <v>46223.80899857639</v>
-      </c>
+      <c r="B55" s="20"/>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="8"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52288,20 +52278,20 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="s">
-        <v>6</v>
+      <c r="A56" s="7" t="s">
+        <v>11</v>
       </c>
-      <c r="B56" s="20">
-        <v>10.0</v>
+      <c r="B56" s="11">
+        <v>70.0</v>
       </c>
-      <c r="C56" s="20">
-        <v>20.0</v>
+      <c r="C56" s="11">
+        <v>300.0</v>
       </c>
-      <c r="D56" s="20">
+      <c r="D56" s="11">
         <v>1.0</v>
       </c>
-      <c r="E56" s="11">
-        <v>46223.80911148148</v>
+      <c r="E56" s="14">
+        <v>46223.80899857639</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
@@ -52313,20 +52303,20 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="s">
-        <v>7</v>
+      <c r="A57" s="7" t="s">
+        <v>8</v>
       </c>
-      <c r="B57" s="20">
-        <v>70.0</v>
+      <c r="B57" s="11">
+        <v>10.0</v>
       </c>
-      <c r="C57" s="20">
-        <v>8.0</v>
+      <c r="C57" s="11">
+        <v>20.0</v>
       </c>
-      <c r="D57" s="20">
+      <c r="D57" s="11">
         <v>1.0</v>
       </c>
-      <c r="E57" s="11">
-        <v>46260.758642430555</v>
+      <c r="E57" s="14">
+        <v>46223.80911148148</v>
       </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
@@ -52338,11 +52328,21 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="8"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="7"/>
+      <c r="A58" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B58" s="11">
+        <v>70.0</v>
+      </c>
+      <c r="C58" s="11">
+        <v>8.0</v>
+      </c>
+      <c r="D58" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="E58" s="14">
+        <v>46260.758642430555</v>
+      </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -52353,17 +52353,11 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B59" s="9" t="s">
-        <v>35</v>
-      </c>
+      <c r="A59" s="7"/>
+      <c r="B59" s="9"/>
       <c r="C59" s="9"/>
       <c r="D59" s="9"/>
-      <c r="E59" s="11">
-        <v>45946.87875708334</v>
-      </c>
+      <c r="E59" s="8"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52374,16 +52368,16 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="8">
-        <v>50.0</v>
+      <c r="A60" s="7" t="s">
+        <v>34</v>
       </c>
-      <c r="B60" s="9">
-        <v>100.0</v>
+      <c r="B60" s="9" t="s">
+        <v>35</v>
       </c>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="11">
-        <v>45946.87887299768</v>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="14">
+        <v>45946.87875708334</v>
       </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
@@ -52395,13 +52389,17 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="43" t="s">
-        <v>36</v>
+      <c r="A61" s="7">
+        <v>50.0</v>
       </c>
-      <c r="B61" s="44"/>
-      <c r="C61" s="44"/>
-      <c r="D61" s="44"/>
-      <c r="E61" s="45"/>
+      <c r="B61" s="9">
+        <v>100.0</v>
+      </c>
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="14">
+        <v>45946.87887299768</v>
+      </c>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -52412,21 +52410,13 @@
       <c r="M61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="39" t="s">
-        <v>37</v>
+      <c r="A62" s="43" t="s">
+        <v>36</v>
       </c>
-      <c r="B62" s="39">
-        <v>100.0</v>
-      </c>
-      <c r="C62" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="D62" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="E62" s="46">
-        <v>46009.783484375</v>
-      </c>
+      <c r="B62" s="44"/>
+      <c r="C62" s="44"/>
+      <c r="D62" s="44"/>
+      <c r="E62" s="45"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -52437,11 +52427,21 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="40"/>
-      <c r="B63" s="40"/>
-      <c r="C63" s="4"/>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
+      <c r="A63" s="39" t="s">
+        <v>37</v>
+      </c>
+      <c r="B63" s="39">
+        <v>100.0</v>
+      </c>
+      <c r="C63" s="18">
+        <v>1.0</v>
+      </c>
+      <c r="D63" s="18">
+        <v>2.0</v>
+      </c>
+      <c r="E63" s="46">
+        <v>46009.783484375</v>
+      </c>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -52452,9 +52452,7 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="39" t="s">
-        <v>38</v>
-      </c>
+      <c r="A64" s="40"/>
       <c r="B64" s="40"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
@@ -52469,21 +52467,13 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="s">
-        <v>7</v>
+      <c r="A65" s="39" t="s">
+        <v>38</v>
       </c>
-      <c r="B65" s="39">
-        <v>50.0</v>
-      </c>
-      <c r="C65" s="15">
-        <v>20.0</v>
-      </c>
-      <c r="D65" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E65" s="46">
-        <v>46038.9559609375</v>
-      </c>
+      <c r="B65" s="40"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
@@ -52494,18 +52484,20 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="39" t="s">
-        <v>39</v>
+      <c r="A66" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="B66" s="39">
-        <v>15.0</v>
+        <v>50.0</v>
       </c>
-      <c r="C66" s="15">
-        <v>16.0</v>
+      <c r="C66" s="18">
+        <v>20.0</v>
       </c>
-      <c r="D66" s="4"/>
+      <c r="D66" s="18">
+        <v>1.0</v>
+      </c>
       <c r="E66" s="46">
-        <v>46136.01284993056</v>
+        <v>46038.9559609375</v>
       </c>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
@@ -52517,11 +52509,19 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="40"/>
-      <c r="B67" s="40"/>
-      <c r="C67" s="4"/>
+      <c r="A67" s="39" t="s">
+        <v>39</v>
+      </c>
+      <c r="B67" s="39">
+        <v>15.0</v>
+      </c>
+      <c r="C67" s="18">
+        <v>16.0</v>
+      </c>
       <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
+      <c r="E67" s="46">
+        <v>46136.01284993056</v>
+      </c>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -52532,17 +52532,11 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="B68" s="39" t="s">
-        <v>20</v>
-      </c>
+      <c r="A68" s="40"/>
+      <c r="B68" s="40"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
-      <c r="E68" s="46">
-        <v>46044.0116671875</v>
-      </c>
+      <c r="E68" s="4"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
       <c r="H68" s="4"/>
@@ -52554,19 +52548,15 @@
     </row>
     <row r="69">
       <c r="A69" s="39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
-      <c r="B69" s="39">
-        <v>5.0</v>
+      <c r="B69" s="39" t="s">
+        <v>22</v>
       </c>
-      <c r="C69" s="15">
-        <v>80.0</v>
-      </c>
-      <c r="D69" s="15">
-        <v>1.0</v>
-      </c>
+      <c r="C69" s="4"/>
+      <c r="D69" s="4"/>
       <c r="E69" s="46">
-        <v>46044.01310700232</v>
+        <v>46044.0116671875</v>
       </c>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
@@ -52579,19 +52569,19 @@
     </row>
     <row r="70">
       <c r="A70" s="39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B70" s="39">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
-      <c r="C70" s="15">
-        <v>10.0</v>
+      <c r="C70" s="18">
+        <v>80.0</v>
       </c>
-      <c r="D70" s="15">
+      <c r="D70" s="18">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
-        <v>46044.013194907406</v>
+        <v>46044.01310700232</v>
       </c>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
@@ -52604,19 +52594,19 @@
     </row>
     <row r="71">
       <c r="A71" s="39" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B71" s="39">
-        <v>30.0</v>
+        <v>15.0</v>
       </c>
-      <c r="C71" s="15">
+      <c r="C71" s="18">
         <v>10.0</v>
       </c>
-      <c r="D71" s="15">
+      <c r="D71" s="18">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
-        <v>46056.701985011576</v>
+        <v>46044.013194907406</v>
       </c>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
@@ -52628,11 +52618,21 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="40"/>
-      <c r="B72" s="40"/>
-      <c r="C72" s="4"/>
-      <c r="D72" s="4"/>
-      <c r="E72" s="4"/>
+      <c r="A72" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="B72" s="39">
+        <v>30.0</v>
+      </c>
+      <c r="C72" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="D72" s="18">
+        <v>1.0</v>
+      </c>
+      <c r="E72" s="46">
+        <v>46056.701985011576</v>
+      </c>
       <c r="F72" s="4"/>
       <c r="G72" s="4"/>
       <c r="H72" s="4"/>
@@ -52643,17 +52643,11 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="B73" s="39" t="s">
-        <v>33</v>
-      </c>
+      <c r="A73" s="40"/>
+      <c r="B73" s="40"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
-      <c r="E73" s="46">
-        <v>46044.0136399537</v>
-      </c>
+      <c r="E73" s="4"/>
       <c r="F73" s="4"/>
       <c r="G73" s="4"/>
       <c r="H73" s="4"/>
@@ -52665,18 +52659,16 @@
     </row>
     <row r="74">
       <c r="A74" s="39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
-      <c r="B74" s="39">
-        <v>5.0</v>
+      <c r="B74" s="39" t="s">
+        <v>33</v>
       </c>
-      <c r="C74" s="15">
-        <v>80.0</v>
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="46">
+        <v>46044.0136399537</v>
       </c>
-      <c r="D74" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="E74" s="4"/>
       <c r="F74" s="4"/>
       <c r="G74" s="4"/>
       <c r="H74" s="4"/>
@@ -52688,15 +52680,15 @@
     </row>
     <row r="75">
       <c r="A75" s="39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B75" s="39">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
-      <c r="C75" s="15">
-        <v>10.0</v>
+      <c r="C75" s="18">
+        <v>80.0</v>
       </c>
-      <c r="D75" s="15">
+      <c r="D75" s="18">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52711,20 +52703,18 @@
     </row>
     <row r="76">
       <c r="A76" s="39" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B76" s="39">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
-      <c r="C76" s="15">
+      <c r="C76" s="18">
         <v>10.0</v>
       </c>
-      <c r="D76" s="15">
-        <v>6.0</v>
+      <c r="D76" s="18">
+        <v>1.0</v>
       </c>
-      <c r="E76" s="46">
-        <v>46044.014003055556</v>
-      </c>
+      <c r="E76" s="4"/>
       <c r="F76" s="4"/>
       <c r="G76" s="4"/>
       <c r="H76" s="4"/>
@@ -52735,11 +52725,21 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="40"/>
-      <c r="B77" s="40"/>
-      <c r="C77" s="4"/>
-      <c r="D77" s="4"/>
-      <c r="E77" s="4"/>
+      <c r="A77" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="B77" s="39">
+        <v>20.0</v>
+      </c>
+      <c r="C77" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="D77" s="18">
+        <v>6.0</v>
+      </c>
+      <c r="E77" s="46">
+        <v>46044.014003055556</v>
+      </c>
       <c r="F77" s="4"/>
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
@@ -52750,7 +52750,7 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="39"/>
+      <c r="A78" s="40"/>
       <c r="B78" s="40"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
@@ -52765,7 +52765,7 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="40"/>
+      <c r="A79" s="39"/>
       <c r="B79" s="40"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
@@ -52780,8 +52780,8 @@
       <c r="M79" s="4"/>
     </row>
     <row r="80">
-      <c r="A80" s="4"/>
-      <c r="B80" s="4"/>
+      <c r="A80" s="40"/>
+      <c r="B80" s="40"/>
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
       <c r="E80" s="4"/>
@@ -66849,6 +66849,21 @@
       <c r="L1017" s="4"/>
       <c r="M1017" s="4"/>
     </row>
+    <row r="1018">
+      <c r="A1018" s="4"/>
+      <c r="B1018" s="4"/>
+      <c r="C1018" s="4"/>
+      <c r="D1018" s="4"/>
+      <c r="E1018" s="4"/>
+      <c r="F1018" s="4"/>
+      <c r="G1018" s="4"/>
+      <c r="H1018" s="4"/>
+      <c r="I1018" s="4"/>
+      <c r="J1018" s="4"/>
+      <c r="K1018" s="4"/>
+      <c r="L1018" s="4"/>
+      <c r="M1018" s="4"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-10-23T06:57:43.499Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,12 +14,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="43">
   <si>
     <t>項目</t>
   </si>
   <si>
     <t>功率</t>
+  </si>
+  <si>
+    <t>遮蓋膠紙</t>
   </si>
   <si>
     <t>速度</t>
@@ -31,9 +34,6 @@
     <t>最後更新日期</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>刀壓</t>
   </si>
   <si>
@@ -43,25 +43,13 @@
     <t>Line</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
-  </si>
-  <si>
     <t>Cut-1/2</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>(PS -3)</t>
   </si>
   <si>
     <t>(PS)</t>
   </si>
   <si>
-    <t>1mm</t>
+    <t>Cut(detail)</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -70,16 +58,37 @@
     <t>03mm</t>
   </si>
   <si>
-    <t>2mm</t>
+    <t>0.5mm</t>
   </si>
   <si>
     <t>Cut</t>
+  </si>
+  <si>
+    <t>(PS -3)</t>
+  </si>
+  <si>
+    <t>FILL</t>
   </si>
   <si>
     <t>0.3 mm</t>
   </si>
   <si>
     <t>Fill</t>
+  </si>
+  <si>
+    <t>1mm</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>2mm</t>
+  </si>
+  <si>
+    <t>cut</t>
+  </si>
+  <si>
+    <t>Keep Detail</t>
   </si>
   <si>
     <t>3mm</t>
@@ -91,22 +100,13 @@
     <t>(0.9 Power)</t>
   </si>
   <si>
-    <t>PS</t>
-  </si>
-  <si>
-    <t>cut</t>
-  </si>
-  <si>
-    <t>Keep Detail</t>
-  </si>
-  <si>
     <t>甲板紙</t>
   </si>
   <si>
-    <t>反轉cut, 鏡射</t>
+    <t>６</t>
   </si>
   <si>
-    <t>６</t>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>1.5mm</t>
@@ -327,31 +327,37 @@
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -363,25 +369,32 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -396,26 +409,16 @@
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -429,9 +432,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -688,13 +688,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -710,7 +710,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -725,16 +725,16 @@
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="12">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -749,18 +749,18 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>25.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -773,10 +773,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="6"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -788,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="s">
-        <v>12</v>
+      <c r="A6" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>13</v>
+      <c r="B6" s="16" t="s">
+        <v>16</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="15"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -808,23 +808,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,23 +834,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="s">
-        <v>10</v>
+      <c r="A8" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="19"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="10"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="12"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +877,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="10"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -897,20 +897,20 @@
       <c r="A11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>5.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>5.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -923,16 +923,16 @@
       <c r="A12" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="10">
         <v>5.0</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <v>15.0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="10">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -945,18 +945,18 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>32.0</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>5.0</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -968,11 +968,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="19"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="6"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="9"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -984,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="s">
-        <v>18</v>
+      <c r="A15" s="15" t="s">
+        <v>22</v>
       </c>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="15"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1002,19 +1002,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="15"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,19 +1026,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="s">
-        <v>10</v>
+      <c r="A17" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="15"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,11 +1050,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="19"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="6"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1067,12 +1067,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="6"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1087,16 +1087,16 @@
       <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <v>5.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1109,12 +1109,12 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="6"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1126,11 +1126,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="19"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="6"/>
+      <c r="A22" s="21"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="9"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1142,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="s">
-        <v>23</v>
+      <c r="A23" s="15" t="s">
+        <v>26</v>
       </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="15"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1160,19 +1160,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="13">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="15"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1184,17 +1184,17 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="s">
-        <v>10</v>
+      <c r="A25" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B25" s="26">
+      <c r="B25" s="31">
         <v>55.0</v>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="27"/>
-      <c r="E25" s="28"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="20"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,15 +1222,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
-        <v>16</v>
+      <c r="A27" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>24</v>
+      <c r="B27" s="10" t="s">
+        <v>27</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="31">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1244,17 +1244,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="10">
         <v>100.0</v>
       </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="31">
+      <c r="D28" s="13"/>
+      <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1268,17 +1268,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>19</v>
+      <c r="A29" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="10">
         <v>20.0</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="10">
         <v>100.0</v>
       </c>
-      <c r="D29" s="20"/>
-      <c r="E29" s="31">
+      <c r="D29" s="13"/>
+      <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="20"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17107,13 +17107,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17130,7 +17130,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17146,16 +17146,16 @@
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>3.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="11">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17171,18 +17171,18 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>20.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="8"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17196,12 +17196,12 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="8"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17217,19 +17217,19 @@
       <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>18.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17240,21 +17240,21 @@
     </row>
     <row r="7">
       <c r="A7" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="10">
         <v>18.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>3.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17265,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="14"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="s">
-        <v>12</v>
+      <c r="A9" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="21"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="20"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17300,19 +17300,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="20">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,19 +17327,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="s">
-        <v>10</v>
+      <c r="A11" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="20">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17354,19 +17354,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="s">
-        <v>21</v>
+      <c r="A12" s="18" t="s">
+        <v>19</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="20">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17381,13 +17381,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="s">
-        <v>14</v>
+      <c r="A13" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="23"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="24"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17400,19 +17400,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="23"/>
+      <c r="E14" s="24"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,19 +17425,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="s">
-        <v>10</v>
+      <c r="A15" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="23"/>
+      <c r="E15" s="24"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="30"/>
-      <c r="E16" s="8"/>
+      <c r="A16" s="27"/>
+      <c r="E16" s="6"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17465,14 +17465,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
-      <c r="B17" s="34" t="s">
-        <v>14</v>
+      <c r="B17" s="29" t="s">
+        <v>10</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="8"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="6"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17488,16 +17488,16 @@
       <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17511,18 +17511,18 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>40.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>5.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="8"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="19"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="8"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="s">
-        <v>18</v>
+      <c r="A21" s="15" t="s">
+        <v>22</v>
       </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="23"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="24"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17571,19 +17571,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="13">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="13">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="23"/>
+      <c r="E22" s="24"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,19 +17596,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="s">
-        <v>10</v>
+      <c r="A23" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="23"/>
+      <c r="E23" s="24"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="19"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="8"/>
+      <c r="A24" s="21"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="6"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17639,12 +17639,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="8"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17660,16 +17660,16 @@
       <c r="A26" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <v>10.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="10">
         <v>15.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="8"/>
+      <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17683,18 +17683,18 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <v>60.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="10">
         <v>2.0</v>
       </c>
-      <c r="E27" s="14">
+      <c r="E27" s="11">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="19"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="8"/>
+      <c r="A28" s="21"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="s">
-        <v>23</v>
+      <c r="A29" s="15" t="s">
+        <v>26</v>
       </c>
-      <c r="B29" s="22"/>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="23"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="24"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17745,19 +17745,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="s">
+      <c r="A30" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="13">
+      <c r="B30" s="16">
         <v>18.0</v>
       </c>
-      <c r="C30" s="13">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="13">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="23"/>
+      <c r="E30" s="24"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17770,16 +17770,16 @@
       <c r="O30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="s">
-        <v>10</v>
+      <c r="A31" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="26">
+      <c r="B31" s="31">
         <v>70.0</v>
       </c>
-      <c r="C31" s="26">
+      <c r="C31" s="31">
         <v>5.0</v>
       </c>
-      <c r="D31" s="26">
+      <c r="D31" s="31">
         <v>1.0</v>
       </c>
       <c r="E31" s="35"/>
@@ -17815,30 +17815,30 @@
       <c r="A33" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="37">
+      <c r="B33" s="38">
         <v>5.0</v>
       </c>
-      <c r="C33" s="37">
+      <c r="C33" s="38">
         <v>10.0</v>
       </c>
-      <c r="D33" s="37">
+      <c r="D33" s="38">
         <v>2.0</v>
       </c>
-      <c r="E33" s="38">
+      <c r="E33" s="39">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="39" t="s">
-        <v>29</v>
+      <c r="F33" s="40" t="s">
+        <v>30</v>
       </c>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="40"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="40"/>
-      <c r="N33" s="40"/>
-      <c r="O33" s="40"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
+      <c r="I33" s="41"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17875,14 +17875,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
-        <v>16</v>
+      <c r="A36" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>24</v>
+      <c r="B36" s="10" t="s">
+        <v>27</v>
       </c>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17896,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <v>100.0</v>
       </c>
-      <c r="D37" s="20"/>
+      <c r="D37" s="13"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17919,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="s">
-        <v>19</v>
+      <c r="A38" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="10">
         <v>20.0</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <v>100.0</v>
       </c>
-      <c r="D38" s="20"/>
+      <c r="D38" s="13"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34573,13 +34573,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34595,7 +34595,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34610,16 +34610,16 @@
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>15.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="12">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34634,18 +34634,18 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>10.0</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>10.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <v>2.0</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="12">
         <v>46232.916719409724</v>
       </c>
       <c r="F4" s="4"/>
@@ -34660,18 +34660,18 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="10">
         <v>20.0</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>20.0</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="10">
         <v>1.0</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="12">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34686,18 +34686,18 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>2.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>20.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="12">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34712,10 +34712,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="6"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="9"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34727,15 +34727,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="s">
-        <v>12</v>
+      <c r="A8" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>13</v>
+      <c r="B8" s="16" t="s">
+        <v>16</v>
       </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="15"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="17"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34747,23 +34747,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="16">
         <v>4.0</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="16">
         <v>10.0</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34773,23 +34773,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="s">
-        <v>10</v>
+      <c r="A10" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="16">
         <v>20.0</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="16">
         <v>10.0</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,11 +34799,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="19"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="10"/>
+      <c r="A11" s="21"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="12"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34816,9 +34816,9 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34833,10 +34833,10 @@
       <c r="A13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="12"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34849,18 +34849,18 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>20.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>10.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="12">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34875,12 +34875,12 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34892,11 +34892,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="19"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="10"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="12"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34909,12 +34909,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="12"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34929,20 +34929,20 @@
       <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>5.0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>5.0</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34955,16 +34955,16 @@
       <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>5.0</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>15.0</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34977,18 +34977,18 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <v>32.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <v>5.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -35000,11 +35000,11 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="19"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="6"/>
+      <c r="A21" s="21"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35016,13 +35016,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="s">
-        <v>18</v>
+      <c r="A22" s="15" t="s">
+        <v>22</v>
       </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="15"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35034,19 +35034,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="16">
         <v>5.0</v>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="16">
         <v>1.0</v>
       </c>
-      <c r="E23" s="15"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35058,19 +35058,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="s">
-        <v>10</v>
+      <c r="A24" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="16">
         <v>50.0</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="13">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="15"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,11 +35082,11 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="19"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="6"/>
+      <c r="A25" s="21"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="9"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35099,12 +35099,12 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="6"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="9"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35119,16 +35119,16 @@
       <c r="A27" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <v>5.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="10">
         <v>5.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="10">
         <v>1.0</v>
       </c>
-      <c r="E27" s="6"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35141,12 +35141,12 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="6"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35158,11 +35158,11 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="19"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="6"/>
+      <c r="A29" s="21"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="9"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35174,13 +35174,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="s">
-        <v>23</v>
+      <c r="A30" s="15" t="s">
+        <v>26</v>
       </c>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="15"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35192,19 +35192,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="13">
+      <c r="B31" s="16">
         <v>5.0</v>
       </c>
-      <c r="C31" s="13">
+      <c r="C31" s="16">
         <v>5.0</v>
       </c>
-      <c r="D31" s="13">
+      <c r="D31" s="16">
         <v>1.0</v>
       </c>
-      <c r="E31" s="15"/>
+      <c r="E31" s="17"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35216,17 +35216,17 @@
       <c r="N31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="25" t="s">
-        <v>10</v>
+      <c r="A32" s="30" t="s">
+        <v>9</v>
       </c>
-      <c r="B32" s="26">
+      <c r="B32" s="31">
         <v>55.0</v>
       </c>
-      <c r="C32" s="26">
+      <c r="C32" s="31">
         <v>2.0</v>
       </c>
-      <c r="D32" s="27"/>
-      <c r="E32" s="28"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="33"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35238,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="20"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35254,15 +35254,15 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="s">
-        <v>16</v>
+      <c r="A34" s="10" t="s">
+        <v>12</v>
       </c>
-      <c r="B34" s="9" t="s">
-        <v>24</v>
+      <c r="B34" s="10" t="s">
+        <v>27</v>
       </c>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="31">
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35276,17 +35276,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="10">
         <v>2.0</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="10">
         <v>100.0</v>
       </c>
-      <c r="D35" s="20"/>
-      <c r="E35" s="31">
+      <c r="D35" s="13"/>
+      <c r="E35" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35300,17 +35300,17 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="s">
-        <v>19</v>
+      <c r="A36" s="10" t="s">
+        <v>15</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="10">
         <v>20.0</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="10">
         <v>100.0</v>
       </c>
-      <c r="D36" s="20"/>
-      <c r="E36" s="31">
+      <c r="D36" s="13"/>
+      <c r="E36" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35324,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="20"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="20"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="20"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,19 +51132,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51159,10 +51159,10 @@
       <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51174,18 +51174,18 @@
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="8">
         <v>60.0</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="8">
         <v>20.0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="8"/>
+      <c r="E3" s="6"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51197,10 +51197,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="8"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51212,14 +51212,14 @@
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="14"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="11"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51233,14 +51233,14 @@
       <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>6.0</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>100.0</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="14">
+      <c r="D6" s="10"/>
+      <c r="E6" s="11">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51254,18 +51254,18 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="10">
         <v>8.0</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>60.0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="10">
         <v>1.0</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="11">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51279,10 +51279,10 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="5"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="8"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="6"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51294,12 +51294,12 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="8"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="6"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51313,16 +51313,16 @@
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="10">
         <v>6.0</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="10">
         <v>45.0</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="10">
         <v>1.0</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="11">
         <v>46266.88342763889</v>
       </c>
       <c r="F10" s="4"/>
@@ -51336,18 +51336,18 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>13.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>30.0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="10">
         <v>1.0</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="11">
         <v>46266.88340020833</v>
       </c>
       <c r="F11" s="4"/>
@@ -51361,10 +51361,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="29"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51375,15 +51375,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="s">
-        <v>20</v>
+      <c r="A13" s="25" t="s">
+        <v>18</v>
       </c>
-      <c r="B13" s="33" t="s">
-        <v>25</v>
+      <c r="B13" s="26" t="s">
+        <v>21</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="14"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51395,18 +51395,18 @@
     </row>
     <row r="14" ht="20.25" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>5.0</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>60.0</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="11">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51422,16 +51422,16 @@
       <c r="A15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="10">
         <v>5.0</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="10">
         <v>30.0</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="10">
         <v>1.0</v>
       </c>
-      <c r="E15" s="14"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51443,22 +51443,22 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="10">
         <v>5.0</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="10">
         <v>30.0</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="10">
         <v>4.0</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="11">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="18" t="s">
-        <v>27</v>
+      <c r="F16" s="14" t="s">
+        <v>24</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51470,18 +51470,18 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="10">
         <v>12.0</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="10">
         <v>20.0</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="10">
         <v>1.0</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="11">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51495,10 +51495,10 @@
     </row>
     <row r="18">
       <c r="A18" s="5"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="29"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51510,12 +51510,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="8"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51529,16 +51529,16 @@
       <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="8">
         <v>6.0</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="8">
         <v>45.0</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="11">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51552,18 +51552,18 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="8">
         <v>18.0</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="8">
         <v>20.0</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="10">
         <v>1.0</v>
       </c>
-      <c r="E21" s="14">
+      <c r="E21" s="11">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51577,10 +51577,10 @@
     </row>
     <row r="22">
       <c r="A22" s="7"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="8"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51591,15 +51591,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="s">
-        <v>12</v>
+      <c r="A23" s="25" t="s">
+        <v>14</v>
       </c>
-      <c r="B23" s="33" t="s">
-        <v>25</v>
+      <c r="B23" s="26" t="s">
+        <v>21</v>
       </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="14">
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="11">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51613,18 +51613,18 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="8">
         <v>6.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="8">
         <v>50.0</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="10">
         <v>1.0</v>
       </c>
-      <c r="E24" s="14">
+      <c r="E24" s="11">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51640,16 +51640,16 @@
       <c r="A25" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="8">
         <v>8.0</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="8">
         <v>30.0</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="10">
         <v>1.0</v>
       </c>
-      <c r="E25" s="14">
+      <c r="E25" s="11">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51663,22 +51663,22 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="8">
         <v>10.0</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="8">
         <v>30.0</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>4.0</v>
       </c>
-      <c r="E26" s="14">
+      <c r="E26" s="11">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="18" t="s">
-        <v>27</v>
+      <c r="F26" s="14" t="s">
+        <v>24</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51690,18 +51690,18 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="8">
         <v>17.0</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="8">
         <v>15.0</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="10">
         <v>1.0</v>
       </c>
-      <c r="E27" s="14">
+      <c r="E27" s="11">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51715,10 +51715,10 @@
     </row>
     <row r="28">
       <c r="A28" s="7"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="8"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51729,15 +51729,15 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="32" t="s">
-        <v>15</v>
+      <c r="A29" s="25" t="s">
+        <v>20</v>
       </c>
-      <c r="B29" s="33" t="s">
-        <v>25</v>
+      <c r="B29" s="26" t="s">
+        <v>21</v>
       </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="8"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51749,18 +51749,18 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="8">
         <v>6.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="8">
         <v>50.0</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="14">
+      <c r="E30" s="11">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51776,16 +51776,16 @@
       <c r="A31" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="8">
         <v>8.0</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="8">
         <v>30.0</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="10">
         <v>1.0</v>
       </c>
-      <c r="E31" s="8"/>
+      <c r="E31" s="6"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51797,18 +51797,18 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="8">
         <v>15.0</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="8">
         <v>10.0</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="10">
         <v>2.0</v>
       </c>
-      <c r="E32" s="14">
+      <c r="E32" s="11">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51822,10 +51822,10 @@
     </row>
     <row r="33">
       <c r="A33" s="7"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="8"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="6"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51836,13 +51836,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="s">
-        <v>15</v>
+      <c r="A34" s="15" t="s">
+        <v>20</v>
       </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="23"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="24"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51853,19 +51853,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="41" t="s">
-        <v>30</v>
+      <c r="B35" s="37" t="s">
+        <v>29</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="37">
         <v>40.0</v>
       </c>
-      <c r="D35" s="41">
+      <c r="D35" s="37">
         <v>1.0</v>
       </c>
-      <c r="E35" s="21">
+      <c r="E35" s="20">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51878,19 +51878,19 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="s">
-        <v>10</v>
+      <c r="A36" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B36" s="41">
+      <c r="B36" s="37">
         <v>30.0</v>
       </c>
-      <c r="C36" s="41">
+      <c r="C36" s="37">
         <v>15.0</v>
       </c>
-      <c r="D36" s="41">
+      <c r="D36" s="37">
         <v>1.0</v>
       </c>
-      <c r="E36" s="23"/>
+      <c r="E36" s="24"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51902,18 +51902,18 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="10">
         <v>10.0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <v>150.0</v>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="10">
         <v>1.0</v>
       </c>
-      <c r="E37" s="14">
+      <c r="E37" s="11">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51926,11 +51926,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="19"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="8"/>
+      <c r="A38" s="21"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="6"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51944,10 +51944,10 @@
       <c r="A39" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="8"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="6"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51959,18 +51959,18 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="10">
         <v>40.0</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="10">
         <v>15.0</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="10">
         <v>1.0</v>
       </c>
-      <c r="E40" s="14">
+      <c r="E40" s="11">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51984,10 +51984,10 @@
     </row>
     <row r="41">
       <c r="A41" s="5"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="8"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="6"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51999,12 +51999,12 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="8"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="6"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -52018,16 +52018,16 @@
       <c r="A43" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="10">
         <v>9.0</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C43" s="10">
         <v>20.0</v>
       </c>
-      <c r="D43" s="9">
+      <c r="D43" s="10">
         <v>1.0</v>
       </c>
-      <c r="E43" s="14">
+      <c r="E43" s="11">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52041,18 +52041,18 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="10">
         <v>55.0</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="10">
         <v>20.0</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="10">
         <v>1.0</v>
       </c>
-      <c r="E44" s="14">
+      <c r="E44" s="11">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52068,19 +52068,19 @@
       <c r="A45" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B45" s="10">
         <v>10.0</v>
       </c>
-      <c r="C45" s="9">
+      <c r="C45" s="10">
         <v>250.0</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45" s="10">
         <v>1.0</v>
       </c>
-      <c r="E45" s="14">
+      <c r="E45" s="11">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="18" t="s">
+      <c r="F45" s="14" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52093,10 +52093,10 @@
     </row>
     <row r="46">
       <c r="A46" s="42"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="8"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="6"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52108,12 +52108,12 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="8"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="6"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52125,18 +52125,18 @@
     </row>
     <row r="48">
       <c r="A48" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="10">
         <v>55.0</v>
       </c>
-      <c r="C48" s="9">
+      <c r="C48" s="10">
         <v>10.0</v>
       </c>
-      <c r="D48" s="9">
+      <c r="D48" s="10">
         <v>1.0</v>
       </c>
-      <c r="E48" s="14">
+      <c r="E48" s="11">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52149,11 +52149,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="42"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="8"/>
+      <c r="A49" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="8">
+        <v>70.0</v>
+      </c>
+      <c r="C49" s="8">
+        <v>300.0</v>
+      </c>
+      <c r="D49" s="8">
+        <v>1.0</v>
+      </c>
+      <c r="E49" s="6"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52165,10 +52173,10 @@
     </row>
     <row r="50">
       <c r="A50" s="42"/>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="8"/>
+      <c r="B50" s="13"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="6"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52180,12 +52188,12 @@
     </row>
     <row r="51">
       <c r="A51" s="42" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
-      <c r="B51" s="20"/>
-      <c r="C51" s="20"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="8"/>
+      <c r="B51" s="13"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="6"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52197,18 +52205,18 @@
     </row>
     <row r="52">
       <c r="A52" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B52" s="9">
+      <c r="B52" s="10">
         <v>60.0</v>
       </c>
-      <c r="C52" s="9">
+      <c r="C52" s="10">
         <v>10.0</v>
       </c>
-      <c r="D52" s="9">
+      <c r="D52" s="10">
         <v>1.0</v>
       </c>
-      <c r="E52" s="14">
+      <c r="E52" s="11">
         <v>46203.63265940972</v>
       </c>
       <c r="F52" s="4"/>
@@ -52224,16 +52232,16 @@
       <c r="A53" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B53" s="9">
+      <c r="B53" s="10">
         <v>10.0</v>
       </c>
-      <c r="C53" s="9">
+      <c r="C53" s="10">
         <v>50.0</v>
       </c>
-      <c r="D53" s="9">
+      <c r="D53" s="10">
         <v>1.0</v>
       </c>
-      <c r="E53" s="14">
+      <c r="E53" s="11">
         <v>46253.61151159722</v>
       </c>
       <c r="F53" s="4"/>
@@ -52247,10 +52255,10 @@
     </row>
     <row r="54">
       <c r="A54" s="42"/>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="8"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="6"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52264,10 +52272,10 @@
       <c r="A55" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B55" s="20"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="8"/>
+      <c r="B55" s="13"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="6"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52279,18 +52287,18 @@
     </row>
     <row r="56">
       <c r="A56" s="7" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
-      <c r="B56" s="11">
+      <c r="B56" s="8">
         <v>70.0</v>
       </c>
-      <c r="C56" s="11">
+      <c r="C56" s="8">
         <v>300.0</v>
       </c>
-      <c r="D56" s="11">
+      <c r="D56" s="8">
         <v>1.0</v>
       </c>
-      <c r="E56" s="14">
+      <c r="E56" s="11">
         <v>46223.80899857639</v>
       </c>
       <c r="F56" s="4"/>
@@ -52306,16 +52314,16 @@
       <c r="A57" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B57" s="11">
+      <c r="B57" s="8">
         <v>10.0</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="8">
         <v>20.0</v>
       </c>
-      <c r="D57" s="11">
+      <c r="D57" s="8">
         <v>1.0</v>
       </c>
-      <c r="E57" s="14">
+      <c r="E57" s="11">
         <v>46223.80911148148</v>
       </c>
       <c r="F57" s="4"/>
@@ -52329,18 +52337,18 @@
     </row>
     <row r="58">
       <c r="A58" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B58" s="11">
+      <c r="B58" s="8">
         <v>70.0</v>
       </c>
-      <c r="C58" s="11">
+      <c r="C58" s="8">
         <v>8.0</v>
       </c>
-      <c r="D58" s="11">
+      <c r="D58" s="8">
         <v>1.0</v>
       </c>
-      <c r="E58" s="14">
+      <c r="E58" s="11">
         <v>46260.758642430555</v>
       </c>
       <c r="F58" s="4"/>
@@ -52354,10 +52362,10 @@
     </row>
     <row r="59">
       <c r="A59" s="7"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="8"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="10"/>
+      <c r="E59" s="6"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52371,12 +52379,12 @@
       <c r="A60" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B60" s="9" t="s">
+      <c r="B60" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="14">
+      <c r="C60" s="10"/>
+      <c r="D60" s="10"/>
+      <c r="E60" s="11">
         <v>45946.87875708334</v>
       </c>
       <c r="F60" s="4"/>
@@ -52392,12 +52400,12 @@
       <c r="A61" s="7">
         <v>50.0</v>
       </c>
-      <c r="B61" s="9">
+      <c r="B61" s="10">
         <v>100.0</v>
       </c>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="14">
+      <c r="C61" s="13"/>
+      <c r="D61" s="13"/>
+      <c r="E61" s="11">
         <v>45946.87887299768</v>
       </c>
       <c r="F61" s="4"/>
@@ -52427,16 +52435,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="39" t="s">
+      <c r="A63" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B63" s="39">
+      <c r="B63" s="40">
         <v>100.0</v>
       </c>
-      <c r="C63" s="18">
+      <c r="C63" s="14">
         <v>1.0</v>
       </c>
-      <c r="D63" s="18">
+      <c r="D63" s="14">
         <v>2.0</v>
       </c>
       <c r="E63" s="46">
@@ -52452,8 +52460,8 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="40"/>
-      <c r="B64" s="40"/>
+      <c r="A64" s="41"/>
+      <c r="B64" s="41"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
@@ -52467,10 +52475,10 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="39" t="s">
+      <c r="A65" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B65" s="40"/>
+      <c r="B65" s="41"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
@@ -52485,15 +52493,15 @@
     </row>
     <row r="66">
       <c r="A66" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B66" s="39">
+      <c r="B66" s="40">
         <v>50.0</v>
       </c>
-      <c r="C66" s="18">
+      <c r="C66" s="14">
         <v>20.0</v>
       </c>
-      <c r="D66" s="18">
+      <c r="D66" s="14">
         <v>1.0</v>
       </c>
       <c r="E66" s="46">
@@ -52509,13 +52517,13 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="39" t="s">
+      <c r="A67" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B67" s="39">
+      <c r="B67" s="40">
         <v>15.0</v>
       </c>
-      <c r="C67" s="18">
+      <c r="C67" s="14">
         <v>16.0</v>
       </c>
       <c r="D67" s="4"/>
@@ -52532,8 +52540,8 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="40"/>
-      <c r="B68" s="40"/>
+      <c r="A68" s="41"/>
+      <c r="B68" s="41"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
       <c r="E68" s="4"/>
@@ -52547,11 +52555,11 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="39" t="s">
+      <c r="A69" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B69" s="39" t="s">
-        <v>22</v>
+      <c r="B69" s="40" t="s">
+        <v>25</v>
       </c>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
@@ -52568,16 +52576,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="39" t="s">
+      <c r="A70" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B70" s="39">
+      <c r="B70" s="40">
         <v>5.0</v>
       </c>
-      <c r="C70" s="18">
+      <c r="C70" s="14">
         <v>80.0</v>
       </c>
-      <c r="D70" s="18">
+      <c r="D70" s="14">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52593,16 +52601,16 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="39" t="s">
+      <c r="A71" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B71" s="39">
+      <c r="B71" s="40">
         <v>15.0</v>
       </c>
-      <c r="C71" s="18">
+      <c r="C71" s="14">
         <v>10.0</v>
       </c>
-      <c r="D71" s="18">
+      <c r="D71" s="14">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52618,16 +52626,16 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="39" t="s">
-        <v>19</v>
+      <c r="A72" s="40" t="s">
+        <v>15</v>
       </c>
-      <c r="B72" s="39">
+      <c r="B72" s="40">
         <v>30.0</v>
       </c>
-      <c r="C72" s="18">
+      <c r="C72" s="14">
         <v>10.0</v>
       </c>
-      <c r="D72" s="18">
+      <c r="D72" s="14">
         <v>1.0</v>
       </c>
       <c r="E72" s="46">
@@ -52643,8 +52651,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="40"/>
-      <c r="B73" s="40"/>
+      <c r="A73" s="41"/>
+      <c r="B73" s="41"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
@@ -52658,10 +52666,10 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="39" t="s">
+      <c r="A74" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B74" s="39" t="s">
+      <c r="B74" s="40" t="s">
         <v>33</v>
       </c>
       <c r="C74" s="4"/>
@@ -52679,16 +52687,16 @@
       <c r="M74" s="4"/>
     </row>
     <row r="75">
-      <c r="A75" s="39" t="s">
+      <c r="A75" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B75" s="39">
+      <c r="B75" s="40">
         <v>5.0</v>
       </c>
-      <c r="C75" s="18">
+      <c r="C75" s="14">
         <v>80.0</v>
       </c>
-      <c r="D75" s="18">
+      <c r="D75" s="14">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52702,16 +52710,16 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76">
-      <c r="A76" s="39" t="s">
+      <c r="A76" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B76" s="39">
+      <c r="B76" s="40">
         <v>15.0</v>
       </c>
-      <c r="C76" s="18">
+      <c r="C76" s="14">
         <v>10.0</v>
       </c>
-      <c r="D76" s="18">
+      <c r="D76" s="14">
         <v>1.0</v>
       </c>
       <c r="E76" s="4"/>
@@ -52725,16 +52733,16 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="39" t="s">
-        <v>19</v>
+      <c r="A77" s="40" t="s">
+        <v>15</v>
       </c>
-      <c r="B77" s="39">
+      <c r="B77" s="40">
         <v>20.0</v>
       </c>
-      <c r="C77" s="18">
+      <c r="C77" s="14">
         <v>10.0</v>
       </c>
-      <c r="D77" s="18">
+      <c r="D77" s="14">
         <v>6.0</v>
       </c>
       <c r="E77" s="46">
@@ -52750,8 +52758,8 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="40"/>
-      <c r="B78" s="40"/>
+      <c r="A78" s="41"/>
+      <c r="B78" s="41"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
@@ -52765,8 +52773,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="39"/>
-      <c r="B79" s="40"/>
+      <c r="A79" s="40"/>
+      <c r="B79" s="41"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
@@ -52780,8 +52788,8 @@
       <c r="M79" s="4"/>
     </row>
     <row r="80">
-      <c r="A80" s="40"/>
-      <c r="B80" s="40"/>
+      <c r="A80" s="41"/>
+      <c r="B80" s="41"/>
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
       <c r="E80" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-10-23T06:57:48.302Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -19,10 +19,13 @@
     <t>項目</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>功率</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
+    <t>刀壓</t>
   </si>
   <si>
     <t>速度</t>
@@ -34,9 +37,6 @@
     <t>最後更新日期</t>
   </si>
   <si>
-    <t>刀壓</t>
-  </si>
-  <si>
     <t>0.3mm</t>
   </si>
   <si>
@@ -46,22 +46,19 @@
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>Cut(detail)</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
+    <t>0.5mm</t>
   </si>
   <si>
     <t>A4紙</t>
   </si>
   <si>
-    <t>03mm</t>
+    <t>(PS)</t>
   </si>
   <si>
-    <t>0.5mm</t>
-  </si>
-  <si>
-    <t>Cut</t>
+    <t>03mm</t>
   </si>
   <si>
     <t>(PS -3)</t>
@@ -70,19 +67,25 @@
     <t>FILL</t>
   </si>
   <si>
+    <t>Cut</t>
+  </si>
+  <si>
     <t>0.3 mm</t>
+  </si>
+  <si>
+    <t>1mm</t>
+  </si>
+  <si>
+    <t>2mm</t>
   </si>
   <si>
     <t>Fill</t>
   </si>
   <si>
-    <t>1mm</t>
-  </si>
-  <si>
     <t>PS</t>
   </si>
   <si>
-    <t>2mm</t>
+    <t>3mm</t>
   </si>
   <si>
     <t>cut</t>
@@ -91,25 +94,22 @@
     <t>Keep Detail</t>
   </si>
   <si>
-    <t>3mm</t>
-  </si>
-  <si>
     <t>4mm</t>
   </si>
   <si>
     <t>(0.9 Power)</t>
   </si>
   <si>
+    <t>６</t>
+  </si>
+  <si>
+    <t>1.5mm</t>
+  </si>
+  <si>
     <t>甲板紙</t>
   </si>
   <si>
-    <t>６</t>
-  </si>
-  <si>
     <t>反轉cut, 鏡射</t>
-  </si>
-  <si>
-    <t>1.5mm</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
@@ -327,32 +327,29 @@
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -369,11 +366,14 @@
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -381,7 +381,7 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -390,10 +390,10 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -412,13 +412,13 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -685,16 +685,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -710,7 +710,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -734,7 +734,7 @@
       <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -760,7 +760,7 @@
       <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -776,7 +776,7 @@
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
-      <c r="E5" s="9"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -788,15 +788,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="s">
-        <v>14</v>
+      <c r="A6" s="14" t="s">
+        <v>11</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>16</v>
+      <c r="B6" s="15" t="s">
+        <v>15</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -808,23 +808,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="15">
         <v>4.0</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="15">
         <v>10.0</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="15">
         <v>1.0</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="18">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,23 +834,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <v>25.0</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="15">
         <v>5.0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="15">
         <v>1.0</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="18">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="21"/>
+      <c r="A9" s="20"/>
       <c r="B9" s="10"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="12"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +877,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
       <c r="D10" s="10"/>
-      <c r="E10" s="12"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -906,11 +906,11 @@
       <c r="D11" s="10">
         <v>1.0</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -932,7 +932,7 @@
       <c r="D12" s="10">
         <v>1.0</v>
       </c>
-      <c r="E12" s="9"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -956,7 +956,7 @@
       <c r="D13" s="10">
         <v>1.0</v>
       </c>
-      <c r="E13" s="9"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -968,11 +968,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="21"/>
+      <c r="A14" s="20"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="9"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -984,13 +984,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
-        <v>22</v>
+      <c r="A15" s="14" t="s">
+        <v>20</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="17"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="16"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1002,19 +1002,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="15">
         <v>5.0</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="15">
         <v>5.0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="15">
         <v>1.0</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="16"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,19 +1026,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="15">
         <v>50.0</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="15">
         <v>5.0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="15">
         <v>1.0</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,11 +1050,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="21"/>
+      <c r="A18" s="20"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="9"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1067,12 +1067,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="9"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1096,7 +1096,7 @@
       <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="9"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1114,7 +1114,7 @@
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1126,11 +1126,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="21"/>
+      <c r="A22" s="20"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="9"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1142,13 +1142,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1160,19 +1160,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="15">
         <v>5.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="16"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1269,7 +1269,7 @@
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B29" s="10">
         <v>20.0</v>
@@ -17104,16 +17104,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17130,7 +17130,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17155,7 +17155,7 @@
       <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17182,7 +17182,7 @@
       <c r="D4" s="10">
         <v>1.0</v>
       </c>
-      <c r="E4" s="6"/>
+      <c r="E4" s="8"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17196,12 +17196,12 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
-      <c r="E5" s="6"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17226,10 +17226,10 @@
       <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17251,10 +17251,10 @@
       <c r="D7" s="10">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17268,7 +17268,7 @@
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
-      <c r="E8" s="11"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,13 +17281,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="s">
-        <v>14</v>
+      <c r="A9" s="14" t="s">
+        <v>11</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="20"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="21"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17300,19 +17300,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <v>4.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <v>15.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="21">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,19 +17327,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="15">
         <v>25.0</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="15">
         <v>10.0</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="15">
         <v>1.0</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="21">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17354,19 +17354,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="s">
-        <v>19</v>
+      <c r="A12" s="17" t="s">
+        <v>21</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <v>4.0</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="15">
         <v>10.0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="15">
         <v>1.0</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="21">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17381,13 +17381,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="s">
-        <v>10</v>
+      <c r="A13" s="17" t="s">
+        <v>13</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="24"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="27"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17400,19 +17400,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="15">
         <v>2.0</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="15">
         <v>18.0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="15">
         <v>1.0</v>
       </c>
-      <c r="E14" s="24"/>
+      <c r="E14" s="27"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,19 +17425,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="15">
         <v>18.0</v>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="15">
         <v>4.0</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="15">
         <v>1.0</v>
       </c>
-      <c r="E15" s="24"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="27"/>
-      <c r="E16" s="6"/>
+      <c r="A16" s="28"/>
+      <c r="E16" s="8"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17465,14 +17465,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
-      <c r="E17" s="6"/>
+      <c r="E17" s="8"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17497,7 +17497,7 @@
       <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="6"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17522,7 +17522,7 @@
       <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="21"/>
+      <c r="A20" s="20"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="6"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,13 +17552,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
-        <v>22</v>
+      <c r="A21" s="14" t="s">
+        <v>20</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="24"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="27"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17571,19 +17571,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="15">
         <v>8.0</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="15">
         <v>15.0</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="15">
         <v>1.0</v>
       </c>
-      <c r="E22" s="24"/>
+      <c r="E22" s="27"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,19 +17596,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <v>55.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="15">
         <v>2.0</v>
       </c>
-      <c r="E23" s="24"/>
+      <c r="E23" s="27"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="21"/>
+      <c r="A24" s="20"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="6"/>
+      <c r="E24" s="8"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17639,12 +17639,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="6"/>
+      <c r="E25" s="8"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17669,7 +17669,7 @@
       <c r="D26" s="10">
         <v>1.0</v>
       </c>
-      <c r="E26" s="6"/>
+      <c r="E26" s="8"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17694,7 +17694,7 @@
       <c r="D27" s="10">
         <v>2.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="12">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="21"/>
+      <c r="A28" s="20"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="6"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,13 +17726,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="24"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17745,19 +17745,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="15">
         <v>18.0</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="15">
         <v>5.0</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="15">
         <v>1.0</v>
       </c>
-      <c r="E30" s="24"/>
+      <c r="E30" s="27"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17782,7 +17782,7 @@
       <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="35"/>
+      <c r="E31" s="36"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17812,8 +17812,8 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="36" t="s">
-        <v>28</v>
+      <c r="A33" s="37" t="s">
+        <v>30</v>
       </c>
       <c r="B33" s="38">
         <v>5.0</v>
@@ -17828,7 +17828,7 @@
         <v>46043.55545597222</v>
       </c>
       <c r="F33" s="40" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G33" s="41"/>
       <c r="H33" s="41"/>
@@ -17920,7 +17920,7 @@
     </row>
     <row r="38">
       <c r="A38" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B38" s="10">
         <v>20.0</v>
@@ -34570,16 +34570,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34595,7 +34595,7 @@
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="9"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34619,7 +34619,7 @@
       <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34634,7 +34634,7 @@
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="10">
         <v>10.0</v>
@@ -34645,7 +34645,7 @@
       <c r="D4" s="10">
         <v>2.0</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="11">
         <v>46232.916719409724</v>
       </c>
       <c r="F4" s="4"/>
@@ -34671,7 +34671,7 @@
       <c r="D5" s="10">
         <v>1.0</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="11">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34686,7 +34686,7 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" s="10">
         <v>2.0</v>
@@ -34697,7 +34697,7 @@
       <c r="D6" s="10">
         <v>1.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="11">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34715,7 +34715,7 @@
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
-      <c r="E7" s="9"/>
+      <c r="E7" s="6"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34727,15 +34727,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="s">
-        <v>14</v>
+      <c r="A8" s="14" t="s">
+        <v>11</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>16</v>
+      <c r="B8" s="15" t="s">
+        <v>15</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="17"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="16"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34747,23 +34747,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="15">
         <v>4.0</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="15">
         <v>10.0</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="15">
         <v>1.0</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="18">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34773,23 +34773,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <v>20.0</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <v>10.0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="15">
         <v>1.0</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="18">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,11 +34799,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="21"/>
+      <c r="A11" s="20"/>
       <c r="B11" s="10"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
-      <c r="E11" s="12"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34816,9 +34816,9 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
-      <c r="E12" s="9"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34836,7 +34836,7 @@
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
-      <c r="E13" s="12"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34860,7 +34860,7 @@
       <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="11">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34875,12 +34875,12 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
-      <c r="E15" s="12"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34892,11 +34892,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="21"/>
+      <c r="A16" s="20"/>
       <c r="B16" s="10"/>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
-      <c r="E16" s="12"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34909,12 +34909,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
       <c r="D17" s="10"/>
-      <c r="E17" s="12"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34938,11 +34938,11 @@
       <c r="D18" s="10">
         <v>1.0</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34964,7 +34964,7 @@
       <c r="D19" s="10">
         <v>1.0</v>
       </c>
-      <c r="E19" s="9"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34988,7 +34988,7 @@
       <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="9"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -35000,11 +35000,11 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="21"/>
+      <c r="A21" s="20"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="9"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35016,13 +35016,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="s">
-        <v>22</v>
+      <c r="A22" s="14" t="s">
+        <v>20</v>
       </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="17"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="16"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35034,19 +35034,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <v>5.0</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="15">
         <v>5.0</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="15">
         <v>1.0</v>
       </c>
-      <c r="E23" s="17"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35058,19 +35058,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="15">
         <v>50.0</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="15">
         <v>5.0</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="15">
         <v>1.0</v>
       </c>
-      <c r="E24" s="17"/>
+      <c r="E24" s="16"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,11 +35082,11 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="21"/>
+      <c r="A25" s="20"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35099,12 +35099,12 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
-      <c r="E26" s="9"/>
+      <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35128,7 +35128,7 @@
       <c r="D27" s="10">
         <v>1.0</v>
       </c>
-      <c r="E27" s="9"/>
+      <c r="E27" s="6"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35146,7 +35146,7 @@
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="9"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35158,11 +35158,11 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="21"/>
+      <c r="A29" s="20"/>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
-      <c r="E29" s="9"/>
+      <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35174,13 +35174,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="17"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35192,19 +35192,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="15">
         <v>5.0</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="15">
         <v>5.0</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="15">
         <v>1.0</v>
       </c>
-      <c r="E31" s="17"/>
+      <c r="E31" s="16"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35301,7 +35301,7 @@
     </row>
     <row r="36">
       <c r="A36" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B36" s="10">
         <v>20.0</v>
@@ -51132,19 +51132,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51159,10 +51159,10 @@
       <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
       <c r="D2" s="10"/>
-      <c r="E2" s="6"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51176,16 +51176,16 @@
       <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <v>60.0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
       <c r="D3" s="10">
         <v>1.0</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="8"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51200,7 +51200,7 @@
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="6"/>
+      <c r="E4" s="8"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51215,11 +51215,11 @@
         <v>12</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
-      <c r="E5" s="11"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51240,7 +51240,7 @@
         <v>100.0</v>
       </c>
       <c r="D6" s="10"/>
-      <c r="E6" s="11">
+      <c r="E6" s="12">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51254,7 +51254,7 @@
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="10">
         <v>8.0</v>
@@ -51265,7 +51265,7 @@
       <c r="D7" s="10">
         <v>1.0</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="12">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51282,7 +51282,7 @@
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
-      <c r="E8" s="6"/>
+      <c r="E8" s="8"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51299,7 +51299,7 @@
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
-      <c r="E9" s="6"/>
+      <c r="E9" s="8"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51322,7 +51322,7 @@
       <c r="D10" s="10">
         <v>1.0</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="12">
         <v>46266.88342763889</v>
       </c>
       <c r="F10" s="4"/>
@@ -51336,7 +51336,7 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11" s="10">
         <v>13.0</v>
@@ -51347,7 +51347,7 @@
       <c r="D11" s="10">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="12">
         <v>46266.88340020833</v>
       </c>
       <c r="F11" s="4"/>
@@ -51379,11 +51379,11 @@
         <v>18</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
+      <c r="E13" s="12"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51395,7 +51395,7 @@
     </row>
     <row r="14" ht="20.25" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B14" s="10">
         <v>5.0</v>
@@ -51406,7 +51406,7 @@
       <c r="D14" s="10">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="12">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51431,7 +51431,7 @@
       <c r="D15" s="10">
         <v>1.0</v>
       </c>
-      <c r="E15" s="11"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51443,7 +51443,7 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" s="10">
         <v>5.0</v>
@@ -51454,11 +51454,11 @@
       <c r="D16" s="10">
         <v>4.0</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="12">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="14" t="s">
-        <v>24</v>
+      <c r="F16" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51470,7 +51470,7 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B17" s="10">
         <v>12.0</v>
@@ -51481,7 +51481,7 @@
       <c r="D17" s="10">
         <v>1.0</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="12">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51510,12 +51510,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="6"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51529,16 +51529,16 @@
       <c r="A20" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="9">
         <v>6.0</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="9">
         <v>45.0</v>
       </c>
       <c r="D20" s="10">
         <v>1.0</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="12">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51554,16 +51554,16 @@
       <c r="A21" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="9">
         <v>18.0</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="9">
         <v>20.0</v>
       </c>
       <c r="D21" s="10">
         <v>1.0</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="12">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51580,7 +51580,7 @@
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="6"/>
+      <c r="E22" s="8"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51592,14 +51592,14 @@
     </row>
     <row r="23">
       <c r="A23" s="25" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
-      <c r="E23" s="11">
+      <c r="E23" s="12">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51613,18 +51613,18 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="9">
         <v>6.0</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C24" s="9">
         <v>50.0</v>
       </c>
       <c r="D24" s="10">
         <v>1.0</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="12">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51640,16 +51640,16 @@
       <c r="A25" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="9">
         <v>8.0</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="9">
         <v>30.0</v>
       </c>
       <c r="D25" s="10">
         <v>1.0</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="12">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51663,22 +51663,22 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="9">
         <v>30.0</v>
       </c>
       <c r="D26" s="10">
         <v>4.0</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="12">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="14" t="s">
-        <v>24</v>
+      <c r="F26" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51690,18 +51690,18 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <v>17.0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="9">
         <v>15.0</v>
       </c>
       <c r="D27" s="10">
         <v>1.0</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="12">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51718,7 +51718,7 @@
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="6"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51730,14 +51730,14 @@
     </row>
     <row r="29">
       <c r="A29" s="25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
-      <c r="E29" s="6"/>
+      <c r="E29" s="8"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51749,18 +51749,18 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="9">
         <v>6.0</v>
       </c>
-      <c r="C30" s="8">
+      <c r="C30" s="9">
         <v>50.0</v>
       </c>
       <c r="D30" s="10">
         <v>1.0</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="12">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51776,16 +51776,16 @@
       <c r="A31" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="9">
         <v>8.0</v>
       </c>
-      <c r="C31" s="8">
+      <c r="C31" s="9">
         <v>30.0</v>
       </c>
       <c r="D31" s="10">
         <v>1.0</v>
       </c>
-      <c r="E31" s="6"/>
+      <c r="E31" s="8"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51799,16 +51799,16 @@
       <c r="A32" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="9">
         <v>15.0</v>
       </c>
-      <c r="C32" s="8">
+      <c r="C32" s="9">
         <v>10.0</v>
       </c>
       <c r="D32" s="10">
         <v>2.0</v>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="12">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51825,7 +51825,7 @@
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
-      <c r="E33" s="6"/>
+      <c r="E33" s="8"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51836,13 +51836,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="s">
-        <v>20</v>
+      <c r="A34" s="14" t="s">
+        <v>19</v>
       </c>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="24"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="27"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51853,19 +51853,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="37" t="s">
-        <v>29</v>
+      <c r="B35" s="35" t="s">
+        <v>28</v>
       </c>
-      <c r="C35" s="37">
+      <c r="C35" s="35">
         <v>40.0</v>
       </c>
-      <c r="D35" s="37">
+      <c r="D35" s="35">
         <v>1.0</v>
       </c>
-      <c r="E35" s="20">
+      <c r="E35" s="21">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51878,19 +51878,19 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="s">
+      <c r="A36" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B36" s="37">
+      <c r="B36" s="35">
         <v>30.0</v>
       </c>
-      <c r="C36" s="37">
+      <c r="C36" s="35">
         <v>15.0</v>
       </c>
-      <c r="D36" s="37">
+      <c r="D36" s="35">
         <v>1.0</v>
       </c>
-      <c r="E36" s="24"/>
+      <c r="E36" s="27"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51902,7 +51902,7 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B37" s="10">
         <v>10.0</v>
@@ -51913,7 +51913,7 @@
       <c r="D37" s="10">
         <v>1.0</v>
       </c>
-      <c r="E37" s="11">
+      <c r="E37" s="12">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51926,11 +51926,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="21"/>
+      <c r="A38" s="20"/>
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
       <c r="D38" s="13"/>
-      <c r="E38" s="6"/>
+      <c r="E38" s="8"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51942,12 +51942,12 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="6"/>
+      <c r="E39" s="8"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51970,7 +51970,7 @@
       <c r="D40" s="10">
         <v>1.0</v>
       </c>
-      <c r="E40" s="11">
+      <c r="E40" s="12">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51987,7 +51987,7 @@
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
       <c r="D41" s="13"/>
-      <c r="E41" s="6"/>
+      <c r="E41" s="8"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51999,12 +51999,12 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B42" s="13"/>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
-      <c r="E42" s="6"/>
+      <c r="E42" s="8"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -52027,7 +52027,7 @@
       <c r="D43" s="10">
         <v>1.0</v>
       </c>
-      <c r="E43" s="11">
+      <c r="E43" s="12">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52052,7 +52052,7 @@
       <c r="D44" s="10">
         <v>1.0</v>
       </c>
-      <c r="E44" s="11">
+      <c r="E44" s="12">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52077,10 +52077,10 @@
       <c r="D45" s="10">
         <v>1.0</v>
       </c>
-      <c r="E45" s="11">
+      <c r="E45" s="12">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="14" t="s">
+      <c r="F45" s="19" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="4"/>
@@ -52096,7 +52096,7 @@
       <c r="B46" s="13"/>
       <c r="C46" s="13"/>
       <c r="D46" s="13"/>
-      <c r="E46" s="6"/>
+      <c r="E46" s="8"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52108,12 +52108,12 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="6"/>
+      <c r="E47" s="8"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52136,7 +52136,7 @@
       <c r="D48" s="10">
         <v>1.0</v>
       </c>
-      <c r="E48" s="11">
+      <c r="E48" s="12">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52150,18 +52150,20 @@
     </row>
     <row r="49">
       <c r="A49" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
-      <c r="B49" s="8">
-        <v>70.0</v>
+      <c r="B49" s="9">
+        <v>40.0</v>
       </c>
-      <c r="C49" s="8">
+      <c r="C49" s="9">
         <v>300.0</v>
       </c>
-      <c r="D49" s="8">
+      <c r="D49" s="9">
         <v>1.0</v>
       </c>
-      <c r="E49" s="6"/>
+      <c r="E49" s="12">
+        <v>46318.6234527662</v>
+      </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -52176,7 +52178,7 @@
       <c r="B50" s="13"/>
       <c r="C50" s="13"/>
       <c r="D50" s="13"/>
-      <c r="E50" s="6"/>
+      <c r="E50" s="8"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52193,7 +52195,7 @@
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
       <c r="D51" s="13"/>
-      <c r="E51" s="6"/>
+      <c r="E51" s="8"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52216,7 +52218,7 @@
       <c r="D52" s="10">
         <v>1.0</v>
       </c>
-      <c r="E52" s="11">
+      <c r="E52" s="12">
         <v>46203.63265940972</v>
       </c>
       <c r="F52" s="4"/>
@@ -52241,7 +52243,7 @@
       <c r="D53" s="10">
         <v>1.0</v>
       </c>
-      <c r="E53" s="11">
+      <c r="E53" s="12">
         <v>46253.61151159722</v>
       </c>
       <c r="F53" s="4"/>
@@ -52258,7 +52260,7 @@
       <c r="B54" s="13"/>
       <c r="C54" s="13"/>
       <c r="D54" s="13"/>
-      <c r="E54" s="6"/>
+      <c r="E54" s="8"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52275,7 +52277,7 @@
       <c r="B55" s="13"/>
       <c r="C55" s="13"/>
       <c r="D55" s="13"/>
-      <c r="E55" s="6"/>
+      <c r="E55" s="8"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52287,18 +52289,18 @@
     </row>
     <row r="56">
       <c r="A56" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
-      <c r="B56" s="8">
+      <c r="B56" s="9">
         <v>70.0</v>
       </c>
-      <c r="C56" s="8">
+      <c r="C56" s="9">
         <v>300.0</v>
       </c>
-      <c r="D56" s="8">
+      <c r="D56" s="9">
         <v>1.0</v>
       </c>
-      <c r="E56" s="11">
+      <c r="E56" s="12">
         <v>46223.80899857639</v>
       </c>
       <c r="F56" s="4"/>
@@ -52314,16 +52316,16 @@
       <c r="A57" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B57" s="8">
+      <c r="B57" s="9">
         <v>10.0</v>
       </c>
-      <c r="C57" s="8">
+      <c r="C57" s="9">
         <v>20.0</v>
       </c>
-      <c r="D57" s="8">
+      <c r="D57" s="9">
         <v>1.0</v>
       </c>
-      <c r="E57" s="11">
+      <c r="E57" s="12">
         <v>46223.80911148148</v>
       </c>
       <c r="F57" s="4"/>
@@ -52339,16 +52341,16 @@
       <c r="A58" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B58" s="8">
+      <c r="B58" s="9">
         <v>70.0</v>
       </c>
-      <c r="C58" s="8">
+      <c r="C58" s="9">
         <v>8.0</v>
       </c>
-      <c r="D58" s="8">
+      <c r="D58" s="9">
         <v>1.0</v>
       </c>
-      <c r="E58" s="11">
+      <c r="E58" s="12">
         <v>46260.758642430555</v>
       </c>
       <c r="F58" s="4"/>
@@ -52365,7 +52367,7 @@
       <c r="B59" s="10"/>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
-      <c r="E59" s="6"/>
+      <c r="E59" s="8"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52384,7 +52386,7 @@
       </c>
       <c r="C60" s="10"/>
       <c r="D60" s="10"/>
-      <c r="E60" s="11">
+      <c r="E60" s="12">
         <v>45946.87875708334</v>
       </c>
       <c r="F60" s="4"/>
@@ -52405,7 +52407,7 @@
       </c>
       <c r="C61" s="13"/>
       <c r="D61" s="13"/>
-      <c r="E61" s="11">
+      <c r="E61" s="12">
         <v>45946.87887299768</v>
       </c>
       <c r="F61" s="4"/>
@@ -52441,10 +52443,10 @@
       <c r="B63" s="40">
         <v>100.0</v>
       </c>
-      <c r="C63" s="14">
+      <c r="C63" s="19">
         <v>1.0</v>
       </c>
-      <c r="D63" s="14">
+      <c r="D63" s="19">
         <v>2.0</v>
       </c>
       <c r="E63" s="46">
@@ -52498,10 +52500,10 @@
       <c r="B66" s="40">
         <v>50.0</v>
       </c>
-      <c r="C66" s="14">
+      <c r="C66" s="19">
         <v>20.0</v>
       </c>
-      <c r="D66" s="14">
+      <c r="D66" s="19">
         <v>1.0</v>
       </c>
       <c r="E66" s="46">
@@ -52523,7 +52525,7 @@
       <c r="B67" s="40">
         <v>15.0</v>
       </c>
-      <c r="C67" s="14">
+      <c r="C67" s="19">
         <v>16.0</v>
       </c>
       <c r="D67" s="4"/>
@@ -52559,7 +52561,7 @@
         <v>40</v>
       </c>
       <c r="B69" s="40" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
@@ -52582,10 +52584,10 @@
       <c r="B70" s="40">
         <v>5.0</v>
       </c>
-      <c r="C70" s="14">
+      <c r="C70" s="19">
         <v>80.0</v>
       </c>
-      <c r="D70" s="14">
+      <c r="D70" s="19">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52607,10 +52609,10 @@
       <c r="B71" s="40">
         <v>15.0</v>
       </c>
-      <c r="C71" s="14">
+      <c r="C71" s="19">
         <v>10.0</v>
       </c>
-      <c r="D71" s="14">
+      <c r="D71" s="19">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52627,15 +52629,15 @@
     </row>
     <row r="72">
       <c r="A72" s="40" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B72" s="40">
         <v>30.0</v>
       </c>
-      <c r="C72" s="14">
+      <c r="C72" s="19">
         <v>10.0</v>
       </c>
-      <c r="D72" s="14">
+      <c r="D72" s="19">
         <v>1.0</v>
       </c>
       <c r="E72" s="46">
@@ -52693,10 +52695,10 @@
       <c r="B75" s="40">
         <v>5.0</v>
       </c>
-      <c r="C75" s="14">
+      <c r="C75" s="19">
         <v>80.0</v>
       </c>
-      <c r="D75" s="14">
+      <c r="D75" s="19">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52716,10 +52718,10 @@
       <c r="B76" s="40">
         <v>15.0</v>
       </c>
-      <c r="C76" s="14">
+      <c r="C76" s="19">
         <v>10.0</v>
       </c>
-      <c r="D76" s="14">
+      <c r="D76" s="19">
         <v>1.0</v>
       </c>
       <c r="E76" s="4"/>
@@ -52734,15 +52736,15 @@
     </row>
     <row r="77">
       <c r="A77" s="40" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B77" s="40">
         <v>20.0</v>
       </c>
-      <c r="C77" s="14">
+      <c r="C77" s="19">
         <v>10.0</v>
       </c>
-      <c r="D77" s="14">
+      <c r="D77" s="19">
         <v>6.0</v>
       </c>
       <c r="E77" s="46">

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-10-24T12:54:08.928Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,18 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="44">
   <si>
     <t>項目</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
-  </si>
-  <si>
     <t>功率</t>
-  </si>
-  <si>
-    <t>刀壓</t>
   </si>
   <si>
     <t>速度</t>
@@ -37,7 +31,16 @@
     <t>最後更新日期</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>0.3mm</t>
+  </si>
+  <si>
+    <t>刀壓</t>
+  </si>
+  <si>
+    <t>``````</t>
   </si>
   <si>
     <t>Line</t>
@@ -46,28 +49,31 @@
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
+    <t>(PS)</t>
+  </si>
+  <si>
+    <t>A4紙</t>
+  </si>
+  <si>
+    <t>03mm</t>
   </si>
   <si>
     <t>0.5mm</t>
   </si>
   <si>
-    <t>A4紙</t>
+    <t>Cut(detail)</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>Cut</t>
   </si>
   <si>
-    <t>03mm</t>
+    <t>FILL</t>
   </si>
   <si>
     <t>(PS -3)</t>
   </si>
   <si>
-    <t>FILL</t>
-  </si>
-  <si>
-    <t>Cut</t>
+    <t>Fill</t>
   </si>
   <si>
     <t>0.3 mm</t>
@@ -76,16 +82,10 @@
     <t>1mm</t>
   </si>
   <si>
-    <t>2mm</t>
-  </si>
-  <si>
-    <t>Fill</t>
-  </si>
-  <si>
     <t>PS</t>
   </si>
   <si>
-    <t>3mm</t>
+    <t>2mm</t>
   </si>
   <si>
     <t>cut</t>
@@ -94,22 +94,25 @@
     <t>Keep Detail</t>
   </si>
   <si>
-    <t>4mm</t>
+    <t>3mm</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
-  </si>
-  <si>
-    <t>６</t>
-  </si>
-  <si>
-    <t>1.5mm</t>
+    <t>4mm</t>
   </si>
   <si>
     <t>甲板紙</t>
   </si>
   <si>
     <t>反轉cut, 鏡射</t>
+  </si>
+  <si>
+    <t>６</t>
+  </si>
+  <si>
+    <t>(0.9 Power)</t>
+  </si>
+  <si>
+    <t>1.5mm</t>
   </si>
   <si>
     <t>吉翁號刻線參數</t>
@@ -209,14 +212,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -327,25 +330,28 @@
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -357,22 +363,19 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -381,21 +384,21 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -403,23 +406,17 @@
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -432,6 +429,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -685,16 +688,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -708,9 +711,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -722,19 +725,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>8</v>
+      <c r="A3" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -748,19 +751,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>9</v>
+      <c r="A4" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>25.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -773,10 +776,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="6"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="7"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -788,15 +791,15 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="s">
-        <v>11</v>
+      <c r="A6" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>15</v>
+      <c r="B6" s="16" t="s">
+        <v>18</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="19"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -808,23 +811,23 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="s">
-        <v>8</v>
+      <c r="A7" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <v>4.0</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <v>10.0</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="21">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -834,23 +837,23 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="s">
-        <v>9</v>
+      <c r="A8" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>25.0</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <v>5.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="21">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -860,11 +863,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="20"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="11"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="12"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -877,12 +880,12 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="11"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -894,23 +897,23 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>8</v>
+      <c r="A11" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>5.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="9">
         <v>5.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -920,19 +923,19 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>8</v>
+      <c r="A12" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="9">
         <v>5.0</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="9">
         <v>15.0</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="9">
         <v>1.0</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="7"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -944,19 +947,19 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>9</v>
+      <c r="A13" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>32.0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>5.0</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="7"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -968,11 +971,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="6"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="7"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -984,13 +987,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="s">
-        <v>20</v>
+      <c r="A15" s="15" t="s">
+        <v>23</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="16"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1002,19 +1005,19 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="s">
-        <v>8</v>
+      <c r="A16" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <v>5.0</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <v>5.0</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="16"/>
+      <c r="E16" s="19"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1026,19 +1029,19 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="s">
-        <v>9</v>
+      <c r="A17" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <v>50.0</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="16">
         <v>5.0</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="19"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1050,11 +1053,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="20"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="6"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1067,12 +1070,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="6"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1084,19 +1087,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>8</v>
+      <c r="A20" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>5.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1108,13 +1111,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>9</v>
+      <c r="A21" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="6"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1126,11 +1129,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="20"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="6"/>
+      <c r="A22" s="25"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="7"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1142,13 +1145,13 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="s">
-        <v>26</v>
+      <c r="A23" s="15" t="s">
+        <v>27</v>
       </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="16"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="19"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1160,19 +1163,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="s">
-        <v>8</v>
+      <c r="A24" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <v>5.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="16"/>
+      <c r="E24" s="19"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1185,7 +1188,7 @@
     </row>
     <row r="25">
       <c r="A25" s="30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B25" s="31">
         <v>55.0</v>
@@ -1193,8 +1196,8 @@
       <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="33"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="35"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1206,11 +1209,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1222,15 +1225,15 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>27</v>
+      <c r="B27" s="9" t="s">
+        <v>31</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="34">
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="41">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1244,17 +1247,17 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>8</v>
+      <c r="A28" s="9" t="s">
+        <v>9</v>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="9">
         <v>2.0</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="34">
+      <c r="D28" s="14"/>
+      <c r="E28" s="41">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1268,17 +1271,17 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
-        <v>17</v>
+      <c r="A29" s="9" t="s">
+        <v>16</v>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="9">
         <v>20.0</v>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="34">
+      <c r="D29" s="14"/>
+      <c r="E29" s="41">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1292,11 +1295,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1308,11 +1311,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17104,16 +17107,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17128,9 +17131,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="E2" s="8"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17143,19 +17146,19 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>8</v>
+      <c r="A3" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>3.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="10">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17170,19 +17173,19 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>9</v>
+      <c r="A4" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>20.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="8"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17195,13 +17198,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>13</v>
+      <c r="A5" s="8" t="s">
+        <v>11</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17214,22 +17217,22 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>8</v>
+      <c r="A6" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>18.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17239,22 +17242,22 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>9</v>
+      <c r="A7" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <v>18.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>3.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17265,10 +17268,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="12"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17281,13 +17284,13 @@
       <c r="O8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="s">
-        <v>11</v>
+      <c r="A9" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="21"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="17"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17300,19 +17303,19 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="s">
-        <v>8</v>
+      <c r="A10" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <v>4.0</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>15.0</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="17">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17327,19 +17330,19 @@
       <c r="O10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="s">
-        <v>9</v>
+      <c r="A11" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="16">
         <v>25.0</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <v>10.0</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="17">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17354,19 +17357,19 @@
       <c r="O11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="s">
-        <v>21</v>
+      <c r="A12" s="18" t="s">
+        <v>19</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <v>4.0</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <v>10.0</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="17">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17381,13 +17384,13 @@
       <c r="O12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="s">
-        <v>13</v>
+      <c r="A13" s="18" t="s">
+        <v>11</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="27"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="20"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17400,19 +17403,19 @@
       <c r="O13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="s">
-        <v>8</v>
+      <c r="A14" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <v>2.0</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <v>18.0</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="27"/>
+      <c r="E14" s="20"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17425,19 +17428,19 @@
       <c r="O14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="s">
-        <v>9</v>
+      <c r="A15" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <v>18.0</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <v>4.0</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="27"/>
+      <c r="E15" s="20"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17450,8 +17453,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="28"/>
-      <c r="E16" s="8"/>
+      <c r="A16" s="24"/>
+      <c r="E16" s="6"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17465,14 +17468,14 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
-      <c r="B17" s="29" t="s">
-        <v>13</v>
+      <c r="B17" s="26" t="s">
+        <v>11</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="8"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="6"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17485,19 +17488,19 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>8</v>
+      <c r="A18" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17510,19 +17513,19 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>9</v>
+      <c r="A19" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>40.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>5.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="8"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17535,11 +17538,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="8"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17552,13 +17555,13 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
-        <v>20</v>
+      <c r="A21" s="15" t="s">
+        <v>23</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="27"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="20"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17571,19 +17574,19 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="s">
-        <v>8</v>
+      <c r="A22" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <v>8.0</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <v>15.0</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="20"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17596,19 +17599,19 @@
       <c r="O22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="s">
-        <v>9</v>
+      <c r="A23" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>55.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="27"/>
+      <c r="E23" s="20"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17621,11 +17624,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="20"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="8"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="6"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17639,12 +17642,12 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="8"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17657,19 +17660,19 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>8</v>
+      <c r="A26" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="9">
         <v>10.0</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="9">
         <v>15.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="8"/>
+      <c r="E26" s="6"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17682,19 +17685,19 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>9</v>
+      <c r="A27" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>60.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="10">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17709,11 +17712,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="20"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="8"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17726,13 +17729,13 @@
       <c r="O28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="s">
-        <v>26</v>
+      <c r="A29" s="15" t="s">
+        <v>27</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="27"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="20"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17745,19 +17748,19 @@
       <c r="O29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="s">
-        <v>8</v>
+      <c r="A30" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <v>18.0</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <v>5.0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="27"/>
+      <c r="E30" s="20"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17771,7 +17774,7 @@
     </row>
     <row r="31">
       <c r="A31" s="30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B31" s="31">
         <v>70.0</v>
@@ -17782,7 +17785,7 @@
       <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="36"/>
+      <c r="E31" s="32"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17812,33 +17815,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="37" t="s">
-        <v>30</v>
+      <c r="A33" s="33" t="s">
+        <v>28</v>
       </c>
-      <c r="B33" s="38">
+      <c r="B33" s="36">
         <v>5.0</v>
       </c>
-      <c r="C33" s="38">
+      <c r="C33" s="36">
         <v>10.0</v>
       </c>
-      <c r="D33" s="38">
+      <c r="D33" s="36">
         <v>2.0</v>
       </c>
-      <c r="E33" s="39">
+      <c r="E33" s="37">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="40" t="s">
-        <v>31</v>
+      <c r="F33" s="38" t="s">
+        <v>29</v>
       </c>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="39"/>
+      <c r="I33" s="39"/>
+      <c r="J33" s="39"/>
+      <c r="K33" s="39"/>
+      <c r="L33" s="39"/>
+      <c r="M33" s="39"/>
+      <c r="N33" s="39"/>
+      <c r="O33" s="39"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17875,14 +17878,14 @@
       <c r="O35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>27</v>
+      <c r="B36" s="9" t="s">
+        <v>31</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17896,16 +17899,16 @@
       <c r="O36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="s">
-        <v>8</v>
+      <c r="A37" s="9" t="s">
+        <v>9</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="9">
         <v>2.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="13"/>
+      <c r="D37" s="14"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17919,16 +17922,16 @@
       <c r="O37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="s">
-        <v>17</v>
+      <c r="A38" s="9" t="s">
+        <v>16</v>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="9">
         <v>20.0</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="14"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34567,19 +34570,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34593,9 +34596,9 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34607,19 +34610,19 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>8</v>
+      <c r="A3" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>2.0</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>15.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34633,19 +34636,19 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>10</v>
+      <c r="A4" s="8" t="s">
+        <v>15</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>10.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>10.0</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>2.0</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="12">
         <v>46232.916719409724</v>
       </c>
       <c r="F4" s="4"/>
@@ -34659,19 +34662,19 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>9</v>
+      <c r="A5" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>20.0</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>20.0</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>1.0</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="12">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34685,19 +34688,19 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>16</v>
+      <c r="A6" s="8" t="s">
+        <v>17</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>2.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>20.0</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="12">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34712,10 +34715,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="6"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34727,15 +34730,15 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="s">
-        <v>11</v>
+      <c r="A8" s="15" t="s">
+        <v>14</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>15</v>
+      <c r="B8" s="16" t="s">
+        <v>18</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="19"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34747,23 +34750,23 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="s">
-        <v>8</v>
+      <c r="A9" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="16">
         <v>4.0</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="16">
         <v>10.0</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="21">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34773,23 +34776,23 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="s">
-        <v>9</v>
+      <c r="A10" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <v>20.0</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <v>10.0</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="21">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34799,11 +34802,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="20"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="11"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="12"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34816,9 +34819,9 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" s="7"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34830,13 +34833,13 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>8</v>
+      <c r="A13" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="12"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34848,19 +34851,19 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>9</v>
+      <c r="A14" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>20.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>10.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="12">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34874,13 +34877,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>16</v>
+      <c r="A15" s="8" t="s">
+        <v>17</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="11"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="12"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34892,11 +34895,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="20"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="11"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="12"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34909,12 +34912,12 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="11"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="12"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34926,23 +34929,23 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>8</v>
+      <c r="A18" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="9">
         <v>5.0</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>5.0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="12">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34952,19 +34955,19 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>8</v>
+      <c r="A19" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="9">
         <v>5.0</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>15.0</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34976,19 +34979,19 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>9</v>
+      <c r="A20" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="9">
         <v>32.0</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>5.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -35000,11 +35003,11 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="20"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="6"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35016,13 +35019,13 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="s">
-        <v>20</v>
+      <c r="A22" s="15" t="s">
+        <v>23</v>
       </c>
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="16"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="19"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35034,19 +35037,19 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="s">
-        <v>8</v>
+      <c r="A23" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <v>5.0</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <v>5.0</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <v>1.0</v>
       </c>
-      <c r="E23" s="16"/>
+      <c r="E23" s="19"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35058,19 +35061,19 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="s">
-        <v>9</v>
+      <c r="A24" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <v>50.0</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <v>5.0</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="16"/>
+      <c r="E24" s="19"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35082,11 +35085,11 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="6"/>
+      <c r="A25" s="25"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35099,12 +35102,12 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="6"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35116,19 +35119,19 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>8</v>
+      <c r="A27" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="9">
         <v>5.0</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="9">
         <v>5.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>1.0</v>
       </c>
-      <c r="E27" s="6"/>
+      <c r="E27" s="7"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35140,13 +35143,13 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>9</v>
+      <c r="A28" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="6"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35158,11 +35161,11 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="20"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="6"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="7"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35174,13 +35177,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="s">
-        <v>26</v>
+      <c r="A30" s="15" t="s">
+        <v>27</v>
       </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="16"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="19"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35192,19 +35195,19 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="s">
-        <v>8</v>
+      <c r="A31" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="15">
+      <c r="B31" s="16">
         <v>5.0</v>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="16">
         <v>5.0</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="16">
         <v>1.0</v>
       </c>
-      <c r="E31" s="16"/>
+      <c r="E31" s="19"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35217,7 +35220,7 @@
     </row>
     <row r="32">
       <c r="A32" s="30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B32" s="31">
         <v>55.0</v>
@@ -35225,8 +35228,8 @@
       <c r="C32" s="31">
         <v>2.0</v>
       </c>
-      <c r="D32" s="32"/>
-      <c r="E32" s="33"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="35"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35238,11 +35241,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35254,15 +35257,15 @@
       <c r="N33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="s">
+      <c r="A34" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="10" t="s">
-        <v>27</v>
+      <c r="B34" s="9" t="s">
+        <v>31</v>
       </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="34">
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="41">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35276,17 +35279,17 @@
       <c r="N34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="s">
-        <v>8</v>
+      <c r="A35" s="9" t="s">
+        <v>9</v>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="9">
         <v>2.0</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="9">
         <v>100.0</v>
       </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="34">
+      <c r="D35" s="14"/>
+      <c r="E35" s="41">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35300,17 +35303,17 @@
       <c r="N35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="s">
-        <v>17</v>
+      <c r="A36" s="9" t="s">
+        <v>16</v>
       </c>
-      <c r="B36" s="10">
+      <c r="B36" s="9">
         <v>20.0</v>
       </c>
-      <c r="C36" s="10">
+      <c r="C36" s="9">
         <v>100.0</v>
       </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="34">
+      <c r="D36" s="14"/>
+      <c r="E36" s="41">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35324,11 +35327,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35340,11 +35343,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="13"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51132,19 +51135,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51156,13 +51159,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="s">
-        <v>8</v>
+      <c r="A2" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="8"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51173,19 +51176,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>9</v>
+      <c r="A3" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="11">
         <v>60.0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="11">
         <v>20.0</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="8"/>
+      <c r="E3" s="6"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51197,10 +51200,10 @@
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="5"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="8"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51215,11 +51218,11 @@
         <v>12</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51230,17 +51233,17 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="7" t="s">
-        <v>8</v>
+      <c r="A6" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>6.0</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>100.0</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="12">
+      <c r="D6" s="9"/>
+      <c r="E6" s="10">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51253,19 +51256,19 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="7" t="s">
-        <v>17</v>
+      <c r="A7" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <v>8.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>60.0</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="10">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51279,10 +51282,10 @@
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="5"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="8"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="6"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51294,12 +51297,12 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="8"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="6"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51310,19 +51313,19 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>8</v>
+      <c r="A10" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="9">
         <v>6.0</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="9">
         <v>45.0</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="10">
         <v>46266.88342763889</v>
       </c>
       <c r="F10" s="4"/>
@@ -51335,19 +51338,19 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>17</v>
+      <c r="A11" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>13.0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="9">
         <v>30.0</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="10">
         <v>46266.88340020833</v>
       </c>
       <c r="F11" s="4"/>
@@ -51375,15 +51378,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="s">
-        <v>18</v>
+      <c r="A13" s="27" t="s">
+        <v>20</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="12"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="10"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51394,19 +51397,19 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14" ht="20.25" customHeight="1">
-      <c r="A14" s="7" t="s">
-        <v>21</v>
+      <c r="A14" s="8" t="s">
+        <v>19</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>5.0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>60.0</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="10">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51419,19 +51422,19 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>8</v>
+      <c r="A15" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="9">
         <v>5.0</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="9">
         <v>30.0</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="9">
         <v>1.0</v>
       </c>
-      <c r="E15" s="12"/>
+      <c r="E15" s="10"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51442,22 +51445,22 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="9">
         <v>5.0</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="9">
         <v>30.0</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="9">
         <v>4.0</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="10">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G16" s="4"/>
@@ -51469,19 +51472,19 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="s">
-        <v>17</v>
+      <c r="A17" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="9">
         <v>12.0</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="9">
         <v>20.0</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="9">
         <v>1.0</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="10">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51510,12 +51513,12 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="8"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51526,19 +51529,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>8</v>
+      <c r="A20" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="11">
         <v>6.0</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="11">
         <v>45.0</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="10">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51551,19 +51554,19 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>9</v>
+      <c r="A21" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B21" s="9">
+      <c r="B21" s="11">
         <v>18.0</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="11">
         <v>20.0</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="9">
         <v>1.0</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="10">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51576,11 +51579,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="7"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="8"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51591,15 +51594,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="s">
-        <v>11</v>
+      <c r="A23" s="27" t="s">
+        <v>14</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="12">
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="10">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51612,19 +51615,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>21</v>
+      <c r="A24" s="8" t="s">
+        <v>19</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="11">
         <v>6.0</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="11">
         <v>50.0</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="10">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51637,19 +51640,19 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>8</v>
+      <c r="A25" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="11">
         <v>8.0</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="11">
         <v>30.0</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="9">
         <v>1.0</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="10">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51662,22 +51665,22 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>17</v>
+      <c r="A26" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="11">
         <v>10.0</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="11">
         <v>30.0</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <v>4.0</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="10">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="19" t="s">
+      <c r="F26" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G26" s="4"/>
@@ -51689,19 +51692,19 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>17</v>
+      <c r="A27" s="8" t="s">
+        <v>16</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="11">
         <v>17.0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="11">
         <v>15.0</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <v>1.0</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="10">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51714,11 +51717,11 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="7"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="8"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51729,15 +51732,15 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="25" t="s">
-        <v>19</v>
+      <c r="A29" s="27" t="s">
+        <v>21</v>
       </c>
-      <c r="B29" s="26" t="s">
+      <c r="B29" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="8"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="6"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51748,19 +51751,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>21</v>
+      <c r="A30" s="8" t="s">
+        <v>19</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="11">
         <v>6.0</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="11">
         <v>50.0</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="9">
         <v>1.0</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="10">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51773,19 +51776,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>8</v>
+      <c r="A31" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="11">
         <v>8.0</v>
       </c>
-      <c r="C31" s="9">
+      <c r="C31" s="11">
         <v>30.0</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="9">
         <v>1.0</v>
       </c>
-      <c r="E31" s="8"/>
+      <c r="E31" s="6"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51796,19 +51799,19 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="s">
-        <v>9</v>
+      <c r="A32" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="11">
         <v>15.0</v>
       </c>
-      <c r="C32" s="9">
+      <c r="C32" s="11">
         <v>10.0</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="9">
         <v>2.0</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="10">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51821,11 +51824,11 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="7"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="8"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="6"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51836,13 +51839,13 @@
       <c r="M33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="s">
-        <v>19</v>
+      <c r="A34" s="15" t="s">
+        <v>21</v>
       </c>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="27"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="20"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51853,19 +51856,19 @@
       <c r="M34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="s">
-        <v>8</v>
+      <c r="A35" s="18" t="s">
+        <v>9</v>
       </c>
-      <c r="B35" s="35" t="s">
-        <v>28</v>
+      <c r="B35" s="40" t="s">
+        <v>30</v>
       </c>
-      <c r="C35" s="35">
+      <c r="C35" s="40">
         <v>40.0</v>
       </c>
-      <c r="D35" s="35">
+      <c r="D35" s="40">
         <v>1.0</v>
       </c>
-      <c r="E35" s="21">
+      <c r="E35" s="17">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51878,19 +51881,19 @@
       <c r="M35" s="4"/>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="s">
-        <v>9</v>
+      <c r="A36" s="18" t="s">
+        <v>10</v>
       </c>
-      <c r="B36" s="35">
+      <c r="B36" s="40">
         <v>30.0</v>
       </c>
-      <c r="C36" s="35">
+      <c r="C36" s="40">
         <v>15.0</v>
       </c>
-      <c r="D36" s="35">
+      <c r="D36" s="40">
         <v>1.0</v>
       </c>
-      <c r="E36" s="27"/>
+      <c r="E36" s="20"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51901,19 +51904,19 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="s">
-        <v>21</v>
+      <c r="A37" s="8" t="s">
+        <v>19</v>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="9">
         <v>10.0</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="9">
         <v>150.0</v>
       </c>
-      <c r="D37" s="10">
+      <c r="D37" s="9">
         <v>1.0</v>
       </c>
-      <c r="E37" s="12">
+      <c r="E37" s="10">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51926,11 +51929,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="20"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="8"/>
+      <c r="A38" s="25"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="6"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51942,12 +51945,12 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="8"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="6"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51958,19 +51961,19 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="s">
-        <v>9</v>
+      <c r="A40" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B40" s="10">
+      <c r="B40" s="9">
         <v>40.0</v>
       </c>
-      <c r="C40" s="10">
+      <c r="C40" s="9">
         <v>15.0</v>
       </c>
-      <c r="D40" s="10">
+      <c r="D40" s="9">
         <v>1.0</v>
       </c>
-      <c r="E40" s="12">
+      <c r="E40" s="10">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51984,10 +51987,10 @@
     </row>
     <row r="41">
       <c r="A41" s="5"/>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="8"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="6"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -51999,12 +52002,12 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="8"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="6"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -52015,19 +52018,19 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="s">
-        <v>8</v>
+      <c r="A43" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="9">
         <v>9.0</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="9">
         <v>20.0</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="10">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52040,19 +52043,19 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="s">
-        <v>9</v>
+      <c r="A44" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B44" s="10">
+      <c r="B44" s="9">
         <v>55.0</v>
       </c>
-      <c r="C44" s="10">
+      <c r="C44" s="9">
         <v>20.0</v>
       </c>
-      <c r="D44" s="10">
+      <c r="D44" s="9">
         <v>1.0</v>
       </c>
-      <c r="E44" s="12">
+      <c r="E44" s="10">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52065,23 +52068,23 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="s">
-        <v>8</v>
+      <c r="A45" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B45" s="10">
+      <c r="B45" s="9">
         <v>10.0</v>
       </c>
-      <c r="C45" s="10">
+      <c r="C45" s="9">
         <v>250.0</v>
       </c>
-      <c r="D45" s="10">
+      <c r="D45" s="9">
         <v>1.0</v>
       </c>
-      <c r="E45" s="12">
+      <c r="E45" s="10">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="19" t="s">
-        <v>32</v>
+      <c r="F45" s="13" t="s">
+        <v>33</v>
       </c>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52093,10 +52096,10 @@
     </row>
     <row r="46">
       <c r="A46" s="42"/>
-      <c r="B46" s="13"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="8"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="6"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52108,12 +52111,12 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
-      <c r="B47" s="13"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="8"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="6"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52124,19 +52127,19 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="s">
-        <v>9</v>
+      <c r="A48" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B48" s="10">
+      <c r="B48" s="9">
         <v>55.0</v>
       </c>
-      <c r="C48" s="10">
+      <c r="C48" s="9">
         <v>10.0</v>
       </c>
-      <c r="D48" s="10">
+      <c r="D48" s="9">
         <v>1.0</v>
       </c>
-      <c r="E48" s="12">
+      <c r="E48" s="10">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52149,19 +52152,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="s">
-        <v>16</v>
+      <c r="A49" s="8" t="s">
+        <v>17</v>
       </c>
-      <c r="B49" s="9">
+      <c r="B49" s="11">
         <v>40.0</v>
       </c>
-      <c r="C49" s="9">
+      <c r="C49" s="11">
         <v>300.0</v>
       </c>
-      <c r="D49" s="9">
+      <c r="D49" s="11">
         <v>1.0</v>
       </c>
-      <c r="E49" s="12">
+      <c r="E49" s="10">
         <v>46318.6234527662</v>
       </c>
       <c r="F49" s="4"/>
@@ -52175,10 +52178,10 @@
     </row>
     <row r="50">
       <c r="A50" s="42"/>
-      <c r="B50" s="13"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="8"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="14"/>
+      <c r="E50" s="6"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52190,12 +52193,12 @@
     </row>
     <row r="51">
       <c r="A51" s="42" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
-      <c r="B51" s="13"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="8"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="6"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52206,19 +52209,19 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="s">
-        <v>9</v>
+      <c r="A52" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B52" s="10">
+      <c r="B52" s="9">
         <v>60.0</v>
       </c>
-      <c r="C52" s="10">
+      <c r="C52" s="9">
         <v>10.0</v>
       </c>
-      <c r="D52" s="10">
+      <c r="D52" s="9">
         <v>1.0</v>
       </c>
-      <c r="E52" s="12">
+      <c r="E52" s="10">
         <v>46203.63265940972</v>
       </c>
       <c r="F52" s="4"/>
@@ -52231,19 +52234,19 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="s">
-        <v>8</v>
+      <c r="A53" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B53" s="10">
+      <c r="B53" s="9">
         <v>10.0</v>
       </c>
-      <c r="C53" s="10">
+      <c r="C53" s="9">
         <v>50.0</v>
       </c>
-      <c r="D53" s="10">
+      <c r="D53" s="9">
         <v>1.0</v>
       </c>
-      <c r="E53" s="12">
+      <c r="E53" s="10">
         <v>46253.61151159722</v>
       </c>
       <c r="F53" s="4"/>
@@ -52257,10 +52260,10 @@
     </row>
     <row r="54">
       <c r="A54" s="42"/>
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="8"/>
+      <c r="B54" s="14"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="6"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52272,12 +52275,12 @@
     </row>
     <row r="55">
       <c r="A55" s="42" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
-      <c r="B55" s="13"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="8"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="6"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52288,19 +52291,19 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="s">
-        <v>16</v>
+      <c r="A56" s="8" t="s">
+        <v>17</v>
       </c>
-      <c r="B56" s="9">
+      <c r="B56" s="11">
         <v>70.0</v>
       </c>
-      <c r="C56" s="9">
+      <c r="C56" s="11">
         <v>300.0</v>
       </c>
-      <c r="D56" s="9">
+      <c r="D56" s="11">
         <v>1.0</v>
       </c>
-      <c r="E56" s="12">
+      <c r="E56" s="10">
         <v>46223.80899857639</v>
       </c>
       <c r="F56" s="4"/>
@@ -52313,19 +52316,19 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="s">
-        <v>8</v>
+      <c r="A57" s="8" t="s">
+        <v>9</v>
       </c>
-      <c r="B57" s="9">
+      <c r="B57" s="11">
         <v>10.0</v>
       </c>
-      <c r="C57" s="9">
+      <c r="C57" s="11">
         <v>20.0</v>
       </c>
-      <c r="D57" s="9">
+      <c r="D57" s="11">
         <v>1.0</v>
       </c>
-      <c r="E57" s="12">
+      <c r="E57" s="10">
         <v>46223.80911148148</v>
       </c>
       <c r="F57" s="4"/>
@@ -52338,19 +52341,19 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="s">
-        <v>9</v>
+      <c r="A58" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B58" s="9">
+      <c r="B58" s="11">
         <v>70.0</v>
       </c>
-      <c r="C58" s="9">
+      <c r="C58" s="11">
         <v>8.0</v>
       </c>
-      <c r="D58" s="9">
+      <c r="D58" s="11">
         <v>1.0</v>
       </c>
-      <c r="E58" s="12">
+      <c r="E58" s="10">
         <v>46260.758642430555</v>
       </c>
       <c r="F58" s="4"/>
@@ -52363,11 +52366,11 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="7"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="8"/>
+      <c r="A59" s="8"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="6"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52378,15 +52381,15 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B60" s="10" t="s">
+      <c r="A60" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="12">
+      <c r="B60" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="10">
         <v>45946.87875708334</v>
       </c>
       <c r="F60" s="4"/>
@@ -52399,15 +52402,15 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="7">
+      <c r="A61" s="8">
         <v>50.0</v>
       </c>
-      <c r="B61" s="10">
+      <c r="B61" s="9">
         <v>100.0</v>
       </c>
-      <c r="C61" s="13"/>
-      <c r="D61" s="13"/>
-      <c r="E61" s="12">
+      <c r="C61" s="14"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="10">
         <v>45946.87887299768</v>
       </c>
       <c r="F61" s="4"/>
@@ -52421,7 +52424,7 @@
     </row>
     <row r="62">
       <c r="A62" s="43" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B62" s="44"/>
       <c r="C62" s="44"/>
@@ -52437,16 +52440,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="40" t="s">
-        <v>37</v>
+      <c r="A63" s="38" t="s">
+        <v>38</v>
       </c>
-      <c r="B63" s="40">
+      <c r="B63" s="38">
         <v>100.0</v>
       </c>
-      <c r="C63" s="19">
+      <c r="C63" s="13">
         <v>1.0</v>
       </c>
-      <c r="D63" s="19">
+      <c r="D63" s="13">
         <v>2.0</v>
       </c>
       <c r="E63" s="46">
@@ -52462,8 +52465,8 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="41"/>
-      <c r="B64" s="41"/>
+      <c r="A64" s="39"/>
+      <c r="B64" s="39"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
@@ -52477,10 +52480,10 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="40" t="s">
-        <v>38</v>
+      <c r="A65" s="38" t="s">
+        <v>39</v>
       </c>
-      <c r="B65" s="41"/>
+      <c r="B65" s="39"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
@@ -52494,16 +52497,16 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="7" t="s">
-        <v>9</v>
+      <c r="A66" s="8" t="s">
+        <v>10</v>
       </c>
-      <c r="B66" s="40">
+      <c r="B66" s="38">
         <v>50.0</v>
       </c>
-      <c r="C66" s="19">
+      <c r="C66" s="13">
         <v>20.0</v>
       </c>
-      <c r="D66" s="19">
+      <c r="D66" s="13">
         <v>1.0</v>
       </c>
       <c r="E66" s="46">
@@ -52519,13 +52522,13 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="40" t="s">
-        <v>39</v>
+      <c r="A67" s="38" t="s">
+        <v>40</v>
       </c>
-      <c r="B67" s="40">
+      <c r="B67" s="38">
         <v>15.0</v>
       </c>
-      <c r="C67" s="19">
+      <c r="C67" s="13">
         <v>16.0</v>
       </c>
       <c r="D67" s="4"/>
@@ -52542,8 +52545,8 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="41"/>
-      <c r="B68" s="41"/>
+      <c r="A68" s="39"/>
+      <c r="B68" s="39"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
       <c r="E68" s="4"/>
@@ -52557,11 +52560,11 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="40" t="s">
-        <v>40</v>
+      <c r="A69" s="38" t="s">
+        <v>41</v>
       </c>
-      <c r="B69" s="40" t="s">
-        <v>23</v>
+      <c r="B69" s="38" t="s">
+        <v>26</v>
       </c>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
@@ -52578,16 +52581,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="40" t="s">
-        <v>41</v>
+      <c r="A70" s="38" t="s">
+        <v>42</v>
       </c>
-      <c r="B70" s="40">
+      <c r="B70" s="38">
         <v>5.0</v>
       </c>
-      <c r="C70" s="19">
+      <c r="C70" s="13">
         <v>80.0</v>
       </c>
-      <c r="D70" s="19">
+      <c r="D70" s="13">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52603,16 +52606,16 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="40" t="s">
-        <v>42</v>
+      <c r="A71" s="38" t="s">
+        <v>43</v>
       </c>
-      <c r="B71" s="40">
+      <c r="B71" s="38">
         <v>15.0</v>
       </c>
-      <c r="C71" s="19">
+      <c r="C71" s="13">
         <v>10.0</v>
       </c>
-      <c r="D71" s="19">
+      <c r="D71" s="13">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52628,16 +52631,16 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="40" t="s">
-        <v>17</v>
+      <c r="A72" s="38" t="s">
+        <v>16</v>
       </c>
-      <c r="B72" s="40">
+      <c r="B72" s="38">
         <v>30.0</v>
       </c>
-      <c r="C72" s="19">
+      <c r="C72" s="13">
         <v>10.0</v>
       </c>
-      <c r="D72" s="19">
+      <c r="D72" s="13">
         <v>1.0</v>
       </c>
       <c r="E72" s="46">
@@ -52653,8 +52656,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="41"/>
-      <c r="B73" s="41"/>
+      <c r="A73" s="39"/>
+      <c r="B73" s="39"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
@@ -52668,11 +52671,11 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="40" t="s">
-        <v>40</v>
+      <c r="A74" s="38" t="s">
+        <v>41</v>
       </c>
-      <c r="B74" s="40" t="s">
-        <v>33</v>
+      <c r="B74" s="38" t="s">
+        <v>34</v>
       </c>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
@@ -52689,16 +52692,16 @@
       <c r="M74" s="4"/>
     </row>
     <row r="75">
-      <c r="A75" s="40" t="s">
-        <v>41</v>
+      <c r="A75" s="38" t="s">
+        <v>42</v>
       </c>
-      <c r="B75" s="40">
+      <c r="B75" s="38">
         <v>5.0</v>
       </c>
-      <c r="C75" s="19">
+      <c r="C75" s="13">
         <v>80.0</v>
       </c>
-      <c r="D75" s="19">
+      <c r="D75" s="13">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52712,16 +52715,16 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76">
-      <c r="A76" s="40" t="s">
-        <v>42</v>
+      <c r="A76" s="38" t="s">
+        <v>43</v>
       </c>
-      <c r="B76" s="40">
+      <c r="B76" s="38">
         <v>15.0</v>
       </c>
-      <c r="C76" s="19">
+      <c r="C76" s="13">
         <v>10.0</v>
       </c>
-      <c r="D76" s="19">
+      <c r="D76" s="13">
         <v>1.0</v>
       </c>
       <c r="E76" s="4"/>
@@ -52735,16 +52738,16 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="40" t="s">
-        <v>17</v>
+      <c r="A77" s="38" t="s">
+        <v>16</v>
       </c>
-      <c r="B77" s="40">
+      <c r="B77" s="38">
         <v>20.0</v>
       </c>
-      <c r="C77" s="19">
+      <c r="C77" s="13">
         <v>10.0</v>
       </c>
-      <c r="D77" s="19">
+      <c r="D77" s="13">
         <v>6.0</v>
       </c>
       <c r="E77" s="46">
@@ -52760,8 +52763,8 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="41"/>
-      <c r="B78" s="41"/>
+      <c r="A78" s="39"/>
+      <c r="B78" s="39"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
@@ -52775,8 +52778,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="40"/>
-      <c r="B79" s="41"/>
+      <c r="A79" s="38"/>
+      <c r="B79" s="39"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
@@ -52790,8 +52793,8 @@
       <c r="M79" s="4"/>
     </row>
     <row r="80">
-      <c r="A80" s="41"/>
-      <c r="B80" s="41"/>
+      <c r="A80" s="39"/>
+      <c r="B80" s="39"/>
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
       <c r="E80" s="4"/>

</xml_diff>

<commit_message>
Update Laser.xlsx from Google Sheets @ 2026-10-24T12:54:11.421Z
</commit_message>
<xml_diff>
--- a/Laser.xlsx
+++ b/Laser.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="43">
   <si>
     <t>項目</t>
   </si>
@@ -25,31 +25,28 @@
     <t>速度</t>
   </si>
   <si>
+    <t>遮蓋膠紙</t>
+  </si>
+  <si>
     <t>次數</t>
+  </si>
+  <si>
+    <t>刀壓</t>
   </si>
   <si>
     <t>最後更新日期</t>
   </si>
   <si>
-    <t>遮蓋膠紙</t>
+    <t>Line</t>
   </si>
   <si>
     <t>0.3mm</t>
   </si>
   <si>
-    <t>刀壓</t>
-  </si>
-  <si>
-    <t>``````</t>
-  </si>
-  <si>
-    <t>Line</t>
-  </si>
-  <si>
     <t>Cut-1/2</t>
   </si>
   <si>
-    <t>(PS)</t>
+    <t>Cut(detail)</t>
   </si>
   <si>
     <t>A4紙</t>
@@ -58,34 +55,28 @@
     <t>03mm</t>
   </si>
   <si>
-    <t>0.5mm</t>
+    <t>FILL</t>
   </si>
   <si>
-    <t>Cut(detail)</t>
+    <t>(PS)</t>
   </si>
   <si>
     <t>Cut</t>
   </si>
   <si>
-    <t>FILL</t>
+    <t>0.5mm</t>
+  </si>
+  <si>
+    <t>0.3 mm</t>
   </si>
   <si>
     <t>(PS -3)</t>
   </si>
   <si>
-    <t>Fill</t>
-  </si>
-  <si>
-    <t>0.3 mm</t>
-  </si>
-  <si>
-    <t>1mm</t>
-  </si>
-  <si>
     <t>PS</t>
   </si>
   <si>
-    <t>2mm</t>
+    <t>Fill</t>
   </si>
   <si>
     <t>cut</t>
@@ -94,28 +85,34 @@
     <t>Keep Detail</t>
   </si>
   <si>
+    <t>1mm</t>
+  </si>
+  <si>
+    <t>2mm</t>
+  </si>
+  <si>
     <t>3mm</t>
   </si>
   <si>
     <t>4mm</t>
   </si>
   <si>
-    <t>甲板紙</t>
-  </si>
-  <si>
-    <t>反轉cut, 鏡射</t>
+    <t>(0.9 Power)</t>
   </si>
   <si>
     <t>６</t>
   </si>
   <si>
-    <t>(0.9 Power)</t>
-  </si>
-  <si>
     <t>1.5mm</t>
   </si>
   <si>
+    <t>甲板紙</t>
+  </si>
+  <si>
     <t>吉翁號刻線參數</t>
+  </si>
+  <si>
+    <t>反轉cut, 鏡射</t>
   </si>
   <si>
     <t>5mm</t>
@@ -212,14 +209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FF00FFFF"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <fgColor rgb="FF00FFFF"/>
+        <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -327,35 +324,35 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -363,17 +360,11 @@
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -384,26 +375,44 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -412,13 +421,10 @@
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="7" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="11" fillId="0" fontId="5" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -429,15 +435,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -694,10 +691,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -710,10 +707,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>6</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -725,8 +722,8 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>9</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B3" s="9">
         <v>2.0</v>
@@ -737,7 +734,7 @@
       <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -751,8 +748,8 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>10</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B4" s="9">
         <v>25.0</v>
@@ -763,7 +760,7 @@
       <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -775,11 +772,11 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="5"/>
+      <c r="A5" s="6"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="7"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -792,14 +789,14 @@
     </row>
     <row r="6">
       <c r="A6" s="15" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
-      <c r="E6" s="19"/>
+      <c r="E6" s="17"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -812,7 +809,7 @@
     </row>
     <row r="7">
       <c r="A7" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7" s="16">
         <v>4.0</v>
@@ -823,11 +820,11 @@
       <c r="D7" s="16">
         <v>1.0</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -838,7 +835,7 @@
     </row>
     <row r="8">
       <c r="A8" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="16">
         <v>25.0</v>
@@ -849,11 +846,11 @@
       <c r="D8" s="16">
         <v>1.0</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="19">
         <v>45954.915123425926</v>
       </c>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -863,11 +860,11 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="25"/>
+      <c r="A9" s="23"/>
       <c r="B9" s="9"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="12"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -879,13 +876,13 @@
       <c r="N9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>21</v>
+      <c r="A10" s="6" t="s">
+        <v>23</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
       <c r="D10" s="9"/>
-      <c r="E10" s="12"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -897,8 +894,8 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>9</v>
+      <c r="A11" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B11" s="9">
         <v>5.0</v>
@@ -909,11 +906,11 @@
       <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -923,8 +920,8 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
-        <v>9</v>
+      <c r="A12" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B12" s="9">
         <v>5.0</v>
@@ -935,7 +932,7 @@
       <c r="D12" s="9">
         <v>1.0</v>
       </c>
-      <c r="E12" s="7"/>
+      <c r="E12" s="8"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -947,8 +944,8 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>10</v>
+      <c r="A13" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B13" s="9">
         <v>32.0</v>
@@ -959,7 +956,7 @@
       <c r="D13" s="9">
         <v>1.0</v>
       </c>
-      <c r="E13" s="7"/>
+      <c r="E13" s="8"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -971,11 +968,11 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="25"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="7"/>
+      <c r="A14" s="23"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="8"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -988,12 +985,12 @@
     </row>
     <row r="15">
       <c r="A15" s="15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="19"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1006,7 +1003,7 @@
     </row>
     <row r="16">
       <c r="A16" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B16" s="16">
         <v>5.0</v>
@@ -1017,7 +1014,7 @@
       <c r="D16" s="16">
         <v>1.0</v>
       </c>
-      <c r="E16" s="19"/>
+      <c r="E16" s="17"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1030,7 +1027,7 @@
     </row>
     <row r="17">
       <c r="A17" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" s="16">
         <v>50.0</v>
@@ -1041,7 +1038,7 @@
       <c r="D17" s="16">
         <v>1.0</v>
       </c>
-      <c r="E17" s="19"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1053,11 +1050,11 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="25"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="7"/>
+      <c r="A18" s="23"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="8"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -1069,13 +1066,13 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>26</v>
+      <c r="A19" s="6" t="s">
+        <v>25</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="7"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1087,8 +1084,8 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>9</v>
+      <c r="A20" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B20" s="9">
         <v>5.0</v>
@@ -1099,7 +1096,7 @@
       <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="7"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1111,13 +1108,13 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>10</v>
+      <c r="A21" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="7"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1129,11 +1126,11 @@
       <c r="N21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="25"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="7"/>
+      <c r="A22" s="23"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="8"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1146,12 +1143,12 @@
     </row>
     <row r="23">
       <c r="A23" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="19"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -1164,7 +1161,7 @@
     </row>
     <row r="24">
       <c r="A24" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B24" s="16">
         <v>5.0</v>
@@ -1175,7 +1172,7 @@
       <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="19"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1188,7 +1185,7 @@
     </row>
     <row r="25">
       <c r="A25" s="30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B25" s="31">
         <v>55.0</v>
@@ -1196,8 +1193,8 @@
       <c r="C25" s="31">
         <v>2.0</v>
       </c>
-      <c r="D25" s="34"/>
-      <c r="E25" s="35"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1209,11 +1206,11 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
+      <c r="A26" s="12"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -1226,14 +1223,14 @@
     </row>
     <row r="27">
       <c r="A27" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="41">
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F27" s="4"/>
@@ -1248,7 +1245,7 @@
     </row>
     <row r="28">
       <c r="A28" s="9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B28" s="9">
         <v>2.0</v>
@@ -1256,8 +1253,8 @@
       <c r="C28" s="9">
         <v>100.0</v>
       </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="41">
+      <c r="D28" s="12"/>
+      <c r="E28" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F28" s="4"/>
@@ -1272,7 +1269,7 @@
     </row>
     <row r="29">
       <c r="A29" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B29" s="9">
         <v>20.0</v>
@@ -1280,8 +1277,8 @@
       <c r="C29" s="9">
         <v>100.0</v>
       </c>
-      <c r="D29" s="14"/>
-      <c r="E29" s="41">
+      <c r="D29" s="12"/>
+      <c r="E29" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F29" s="4"/>
@@ -1295,11 +1292,11 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="14"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1311,11 +1308,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="14"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17113,10 +17110,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -17130,10 +17127,10 @@
       <c r="O1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>6</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -17146,8 +17143,8 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>9</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B3" s="9">
         <v>3.0</v>
@@ -17158,7 +17155,7 @@
       <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="13">
         <v>46037.00168581019</v>
       </c>
       <c r="F3" s="4"/>
@@ -17173,8 +17170,8 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>10</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B4" s="9">
         <v>20.0</v>
@@ -17185,7 +17182,7 @@
       <c r="D4" s="9">
         <v>1.0</v>
       </c>
-      <c r="E4" s="6"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -17198,13 +17195,13 @@
       <c r="O4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>11</v>
+      <c r="A5" s="5" t="s">
+        <v>14</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="6"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -17217,8 +17214,8 @@
       <c r="O5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>9</v>
+      <c r="A6" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B6" s="9">
         <v>2.0</v>
@@ -17229,10 +17226,10 @@
       <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -17242,8 +17239,8 @@
       <c r="O6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>10</v>
+      <c r="A7" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B7" s="9">
         <v>18.0</v>
@@ -17254,10 +17251,10 @@
       <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -17267,11 +17264,11 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="5"/>
+      <c r="A8" s="6"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
-      <c r="E8" s="10"/>
+      <c r="E8" s="13"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17285,12 +17282,12 @@
     </row>
     <row r="9">
       <c r="A9" s="15" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
-      <c r="E9" s="17"/>
+      <c r="E9" s="22"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17304,7 +17301,7 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10" s="16">
         <v>4.0</v>
@@ -17315,7 +17312,7 @@
       <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="22">
         <v>46223.647590416665</v>
       </c>
       <c r="F10" s="4"/>
@@ -17331,7 +17328,7 @@
     </row>
     <row r="11">
       <c r="A11" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="16">
         <v>25.0</v>
@@ -17342,7 +17339,7 @@
       <c r="D11" s="16">
         <v>1.0</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="22">
         <v>46031.84505053241</v>
       </c>
       <c r="F11" s="4"/>
@@ -17358,7 +17355,7 @@
     </row>
     <row r="12">
       <c r="A12" s="18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" s="16">
         <v>4.0</v>
@@ -17369,7 +17366,7 @@
       <c r="D12" s="16">
         <v>1.0</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="22">
         <v>45960.0</v>
       </c>
       <c r="F12" s="4"/>
@@ -17385,12 +17382,12 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
-      <c r="E13" s="20"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17404,7 +17401,7 @@
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B14" s="16">
         <v>2.0</v>
@@ -17415,7 +17412,7 @@
       <c r="D14" s="16">
         <v>1.0</v>
       </c>
-      <c r="E14" s="20"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17429,7 +17426,7 @@
     </row>
     <row r="15">
       <c r="A15" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="16">
         <v>18.0</v>
@@ -17440,7 +17437,7 @@
       <c r="D15" s="16">
         <v>1.0</v>
       </c>
-      <c r="E15" s="20"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17453,8 +17450,8 @@
       <c r="O15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="24"/>
-      <c r="E16" s="6"/>
+      <c r="A16" s="28"/>
+      <c r="E16" s="10"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17467,15 +17464,15 @@
       <c r="O16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>21</v>
+      <c r="A17" s="6" t="s">
+        <v>23</v>
       </c>
-      <c r="B17" s="26" t="s">
-        <v>11</v>
+      <c r="B17" s="29" t="s">
+        <v>14</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
-      <c r="E17" s="6"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17488,8 +17485,8 @@
       <c r="O17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>9</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B18" s="9">
         <v>5.0</v>
@@ -17500,7 +17497,7 @@
       <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="6"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17513,8 +17510,8 @@
       <c r="O18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>10</v>
+      <c r="A19" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B19" s="9">
         <v>40.0</v>
@@ -17525,7 +17522,7 @@
       <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17538,11 +17535,11 @@
       <c r="O19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="25"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="6"/>
+      <c r="A20" s="23"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="10"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17556,12 +17553,12 @@
     </row>
     <row r="21">
       <c r="A21" s="15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="20"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17575,7 +17572,7 @@
     </row>
     <row r="22">
       <c r="A22" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B22" s="16">
         <v>8.0</v>
@@ -17586,7 +17583,7 @@
       <c r="D22" s="16">
         <v>1.0</v>
       </c>
-      <c r="E22" s="20"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17600,7 +17597,7 @@
     </row>
     <row r="23">
       <c r="A23" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B23" s="16">
         <v>55.0</v>
@@ -17611,7 +17608,7 @@
       <c r="D23" s="16">
         <v>2.0</v>
       </c>
-      <c r="E23" s="20"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17624,11 +17621,11 @@
       <c r="O23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="25"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="6"/>
+      <c r="A24" s="23"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="10"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17641,13 +17638,13 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>26</v>
+      <c r="A25" s="6" t="s">
+        <v>25</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="6"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="10"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17660,8 +17657,8 @@
       <c r="O25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>9</v>
+      <c r="A26" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B26" s="9">
         <v>10.0</v>
@@ -17672,7 +17669,7 @@
       <c r="D26" s="9">
         <v>1.0</v>
       </c>
-      <c r="E26" s="6"/>
+      <c r="E26" s="10"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17685,8 +17682,8 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>10</v>
+      <c r="A27" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B27" s="9">
         <v>60.0</v>
@@ -17697,7 +17694,7 @@
       <c r="D27" s="9">
         <v>2.0</v>
       </c>
-      <c r="E27" s="10">
+      <c r="E27" s="13">
         <v>45974.8842990625</v>
       </c>
       <c r="F27" s="4"/>
@@ -17712,11 +17709,11 @@
       <c r="O27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="25"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="6"/>
+      <c r="A28" s="23"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17730,12 +17727,12 @@
     </row>
     <row r="29">
       <c r="A29" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="20"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17749,7 +17746,7 @@
     </row>
     <row r="30">
       <c r="A30" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B30" s="16">
         <v>18.0</v>
@@ -17760,7 +17757,7 @@
       <c r="D30" s="16">
         <v>1.0</v>
       </c>
-      <c r="E30" s="20"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17774,7 +17771,7 @@
     </row>
     <row r="31">
       <c r="A31" s="30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B31" s="31">
         <v>70.0</v>
@@ -17785,7 +17782,7 @@
       <c r="D31" s="31">
         <v>1.0</v>
       </c>
-      <c r="E31" s="32"/>
+      <c r="E31" s="36"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17815,33 +17812,33 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" ht="20.25" customHeight="1">
-      <c r="A33" s="33" t="s">
-        <v>28</v>
+      <c r="A33" s="37" t="s">
+        <v>30</v>
       </c>
-      <c r="B33" s="36">
+      <c r="B33" s="38">
         <v>5.0</v>
       </c>
-      <c r="C33" s="36">
+      <c r="C33" s="38">
         <v>10.0</v>
       </c>
-      <c r="D33" s="36">
+      <c r="D33" s="38">
         <v>2.0</v>
       </c>
-      <c r="E33" s="37">
+      <c r="E33" s="40">
         <v>46043.55545597222</v>
       </c>
-      <c r="F33" s="38" t="s">
-        <v>29</v>
+      <c r="F33" s="41" t="s">
+        <v>32</v>
       </c>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="39"/>
-      <c r="J33" s="39"/>
-      <c r="K33" s="39"/>
-      <c r="L33" s="39"/>
-      <c r="M33" s="39"/>
-      <c r="N33" s="39"/>
-      <c r="O33" s="39"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42"/>
+      <c r="O33" s="42"/>
     </row>
     <row r="34">
       <c r="A34" s="4"/>
@@ -17879,13 +17876,13 @@
     </row>
     <row r="36">
       <c r="A36" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -17900,7 +17897,7 @@
     </row>
     <row r="37">
       <c r="A37" s="9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B37" s="9">
         <v>2.0</v>
@@ -17908,7 +17905,7 @@
       <c r="C37" s="9">
         <v>100.0</v>
       </c>
-      <c r="D37" s="14"/>
+      <c r="D37" s="12"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -17923,7 +17920,7 @@
     </row>
     <row r="38">
       <c r="A38" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B38" s="9">
         <v>20.0</v>
@@ -17931,7 +17928,7 @@
       <c r="C38" s="9">
         <v>100.0</v>
       </c>
-      <c r="D38" s="14"/>
+      <c r="D38" s="12"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -34570,7 +34567,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -34579,10 +34576,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -34595,10 +34592,10 @@
       <c r="N1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>6</v>
+      <c r="A2" s="6" t="s">
+        <v>8</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="8"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -34610,8 +34607,8 @@
       <c r="N2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>9</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B3" s="9">
         <v>2.0</v>
@@ -34622,7 +34619,7 @@
       <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>46106.732072326384</v>
       </c>
       <c r="F3" s="4"/>
@@ -34636,8 +34633,8 @@
       <c r="N3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>15</v>
+      <c r="A4" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="B4" s="9">
         <v>10.0</v>
@@ -34648,7 +34645,7 @@
       <c r="D4" s="9">
         <v>2.0</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="11">
         <v>46232.916719409724</v>
       </c>
       <c r="F4" s="4"/>
@@ -34662,8 +34659,8 @@
       <c r="N4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>10</v>
+      <c r="A5" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B5" s="9">
         <v>20.0</v>
@@ -34674,7 +34671,7 @@
       <c r="D5" s="9">
         <v>1.0</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="11">
         <v>46147.893450902775</v>
       </c>
       <c r="F5" s="4"/>
@@ -34688,8 +34685,8 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>17</v>
+      <c r="A6" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="B6" s="9">
         <v>2.0</v>
@@ -34700,7 +34697,7 @@
       <c r="D6" s="9">
         <v>1.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="11">
         <v>46182.71399388889</v>
       </c>
       <c r="F6" s="4"/>
@@ -34714,11 +34711,11 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="5"/>
+      <c r="A7" s="6"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
-      <c r="E7" s="7"/>
+      <c r="E7" s="8"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -34731,14 +34728,14 @@
     </row>
     <row r="8">
       <c r="A8" s="15" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
-      <c r="E8" s="19"/>
+      <c r="E8" s="17"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -34751,7 +34748,7 @@
     </row>
     <row r="9">
       <c r="A9" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9" s="16">
         <v>4.0</v>
@@ -34762,11 +34759,11 @@
       <c r="D9" s="16">
         <v>1.0</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="19">
         <v>45957.92965825232</v>
       </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -34777,7 +34774,7 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="16">
         <v>20.0</v>
@@ -34788,11 +34785,11 @@
       <c r="D10" s="16">
         <v>1.0</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="19">
         <v>46116.685309016204</v>
       </c>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -34802,11 +34799,11 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="25"/>
+      <c r="A11" s="23"/>
       <c r="B11" s="9"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -34818,10 +34815,10 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>14</v>
+      <c r="A12" s="6" t="s">
+        <v>16</v>
       </c>
-      <c r="E12" s="7"/>
+      <c r="E12" s="8"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -34833,13 +34830,13 @@
       <c r="N12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>9</v>
+      <c r="A13" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="12"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -34851,8 +34848,8 @@
       <c r="N13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
-        <v>10</v>
+      <c r="A14" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B14" s="9">
         <v>20.0</v>
@@ -34863,7 +34860,7 @@
       <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="11">
         <v>46228.70790929398</v>
       </c>
       <c r="F14" s="4"/>
@@ -34877,13 +34874,13 @@
       <c r="N14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>17</v>
+      <c r="A15" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
-      <c r="E15" s="12"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -34895,11 +34892,11 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="25"/>
+      <c r="A16" s="23"/>
       <c r="B16" s="9"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -34911,13 +34908,13 @@
       <c r="N16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>21</v>
+      <c r="A17" s="6" t="s">
+        <v>23</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
       <c r="D17" s="9"/>
-      <c r="E17" s="12"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -34929,8 +34926,8 @@
       <c r="N17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>9</v>
+      <c r="A18" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B18" s="9">
         <v>5.0</v>
@@ -34941,11 +34938,11 @@
       <c r="D18" s="9">
         <v>1.0</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="11">
         <v>46042.0</v>
       </c>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
@@ -34955,8 +34952,8 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>9</v>
+      <c r="A19" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B19" s="9">
         <v>5.0</v>
@@ -34967,7 +34964,7 @@
       <c r="D19" s="9">
         <v>1.0</v>
       </c>
-      <c r="E19" s="7"/>
+      <c r="E19" s="8"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -34979,8 +34976,8 @@
       <c r="N19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>10</v>
+      <c r="A20" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B20" s="9">
         <v>32.0</v>
@@ -34991,7 +34988,7 @@
       <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="7"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -35003,11 +35000,11 @@
       <c r="N20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="25"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="7"/>
+      <c r="A21" s="23"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -35020,12 +35017,12 @@
     </row>
     <row r="22">
       <c r="A22" s="15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="19"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="17"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -35038,7 +35035,7 @@
     </row>
     <row r="23">
       <c r="A23" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B23" s="16">
         <v>5.0</v>
@@ -35049,7 +35046,7 @@
       <c r="D23" s="16">
         <v>1.0</v>
       </c>
-      <c r="E23" s="19"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -35062,7 +35059,7 @@
     </row>
     <row r="24">
       <c r="A24" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B24" s="16">
         <v>50.0</v>
@@ -35073,7 +35070,7 @@
       <c r="D24" s="16">
         <v>1.0</v>
       </c>
-      <c r="E24" s="19"/>
+      <c r="E24" s="17"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -35085,11 +35082,11 @@
       <c r="N24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="25"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="7"/>
+      <c r="A25" s="23"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="8"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -35101,13 +35098,13 @@
       <c r="N25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>26</v>
+      <c r="A26" s="6" t="s">
+        <v>25</v>
       </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="7"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="8"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -35119,8 +35116,8 @@
       <c r="N26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>9</v>
+      <c r="A27" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B27" s="9">
         <v>5.0</v>
@@ -35131,7 +35128,7 @@
       <c r="D27" s="9">
         <v>1.0</v>
       </c>
-      <c r="E27" s="7"/>
+      <c r="E27" s="8"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -35143,13 +35140,13 @@
       <c r="N27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>10</v>
+      <c r="A28" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="7"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="8"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -35161,11 +35158,11 @@
       <c r="N28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="25"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="7"/>
+      <c r="A29" s="23"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="8"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -35178,12 +35175,12 @@
     </row>
     <row r="30">
       <c r="A30" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="19"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -35196,7 +35193,7 @@
     </row>
     <row r="31">
       <c r="A31" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B31" s="16">
         <v>5.0</v>
@@ -35207,7 +35204,7 @@
       <c r="D31" s="16">
         <v>1.0</v>
       </c>
-      <c r="E31" s="19"/>
+      <c r="E31" s="17"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -35220,7 +35217,7 @@
     </row>
     <row r="32">
       <c r="A32" s="30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B32" s="31">
         <v>55.0</v>
@@ -35228,8 +35225,8 @@
       <c r="C32" s="31">
         <v>2.0</v>
       </c>
-      <c r="D32" s="34"/>
-      <c r="E32" s="35"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="33"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -35241,11 +35238,11 @@
       <c r="N32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="14"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
+      <c r="A33" s="12"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -35258,14 +35255,14 @@
     </row>
     <row r="34">
       <c r="A34" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="41">
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="34">
         <v>46051.96156388889</v>
       </c>
       <c r="F34" s="4"/>
@@ -35280,7 +35277,7 @@
     </row>
     <row r="35">
       <c r="A35" s="9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B35" s="9">
         <v>2.0</v>
@@ -35288,8 +35285,8 @@
       <c r="C35" s="9">
         <v>100.0</v>
       </c>
-      <c r="D35" s="14"/>
-      <c r="E35" s="41">
+      <c r="D35" s="12"/>
+      <c r="E35" s="34">
         <v>46100.83597384259</v>
       </c>
       <c r="F35" s="4"/>
@@ -35304,7 +35301,7 @@
     </row>
     <row r="36">
       <c r="A36" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B36" s="9">
         <v>20.0</v>
@@ -35312,8 +35309,8 @@
       <c r="C36" s="9">
         <v>100.0</v>
       </c>
-      <c r="D36" s="14"/>
-      <c r="E36" s="41">
+      <c r="D36" s="12"/>
+      <c r="E36" s="34">
         <v>46100.83604224537</v>
       </c>
       <c r="F36" s="4"/>
@@ -35327,11 +35324,11 @@
       <c r="N36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
+      <c r="A37" s="12"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -35343,11 +35340,11 @@
       <c r="N37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
+      <c r="A38" s="12"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51135,19 +51132,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -51159,13 +51156,13 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>9</v>
+      <c r="A2" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
       <c r="D2" s="9"/>
-      <c r="E2" s="6"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -51176,19 +51173,19 @@
       <c r="M2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>10</v>
+      <c r="A3" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="7">
         <v>60.0</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="7">
         <v>20.0</v>
       </c>
       <c r="D3" s="9">
         <v>1.0</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -51199,11 +51196,11 @@
       <c r="M3" s="4"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="6"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -51214,15 +51211,15 @@
       <c r="M4" s="4"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="10"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="13"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -51233,8 +51230,8 @@
       <c r="M5" s="4"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>9</v>
+      <c r="A6" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B6" s="9">
         <v>6.0</v>
@@ -51243,7 +51240,7 @@
         <v>100.0</v>
       </c>
       <c r="D6" s="9"/>
-      <c r="E6" s="10">
+      <c r="E6" s="13">
         <v>46241.84478354167</v>
       </c>
       <c r="F6" s="4"/>
@@ -51256,8 +51253,8 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="8" t="s">
-        <v>16</v>
+      <c r="A7" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="B7" s="9">
         <v>8.0</v>
@@ -51268,7 +51265,7 @@
       <c r="D7" s="9">
         <v>1.0</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="13">
         <v>46241.876225625005</v>
       </c>
       <c r="F7" s="4"/>
@@ -51281,11 +51278,11 @@
       <c r="M7" s="4"/>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="5"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="6"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -51296,13 +51293,13 @@
       <c r="M8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>20</v>
+      <c r="A9" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
-      <c r="E9" s="6"/>
+      <c r="E9" s="10"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -51313,8 +51310,8 @@
       <c r="M9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>9</v>
+      <c r="A10" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B10" s="9">
         <v>6.0</v>
@@ -51325,7 +51322,7 @@
       <c r="D10" s="9">
         <v>1.0</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="13">
         <v>46266.88342763889</v>
       </c>
       <c r="F10" s="4"/>
@@ -51338,8 +51335,8 @@
       <c r="M10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>16</v>
+      <c r="A11" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="B11" s="9">
         <v>13.0</v>
@@ -51350,7 +51347,7 @@
       <c r="D11" s="9">
         <v>1.0</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="13">
         <v>46266.88340020833</v>
       </c>
       <c r="F11" s="4"/>
@@ -51363,11 +51360,11 @@
       <c r="M11" s="4"/>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="5"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="21"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -51378,15 +51375,15 @@
       <c r="M12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="s">
-        <v>20</v>
+      <c r="A13" s="24" t="s">
+        <v>17</v>
       </c>
-      <c r="B13" s="28" t="s">
-        <v>22</v>
+      <c r="B13" s="25" t="s">
+        <v>19</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="10"/>
+      <c r="E13" s="13"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -51397,8 +51394,8 @@
       <c r="M13" s="4"/>
     </row>
     <row r="14" ht="20.25" customHeight="1">
-      <c r="A14" s="8" t="s">
-        <v>19</v>
+      <c r="A14" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="B14" s="9">
         <v>5.0</v>
@@ -51409,7 +51406,7 @@
       <c r="D14" s="9">
         <v>1.0</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="13">
         <v>46160.881155752315</v>
       </c>
       <c r="F14" s="4"/>
@@ -51422,8 +51419,8 @@
       <c r="M14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>9</v>
+      <c r="A15" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B15" s="9">
         <v>5.0</v>
@@ -51434,7 +51431,7 @@
       <c r="D15" s="9">
         <v>1.0</v>
       </c>
-      <c r="E15" s="10"/>
+      <c r="E15" s="13"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -51445,8 +51442,8 @@
       <c r="M15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>24</v>
+      <c r="A16" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="B16" s="9">
         <v>5.0</v>
@@ -51457,11 +51454,11 @@
       <c r="D16" s="9">
         <v>4.0</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="13">
         <v>46160.85381630787</v>
       </c>
-      <c r="F16" s="13" t="s">
-        <v>25</v>
+      <c r="F16" s="14" t="s">
+        <v>22</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -51472,8 +51469,8 @@
       <c r="M16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
-        <v>16</v>
+      <c r="A17" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="B17" s="9">
         <v>12.0</v>
@@ -51484,7 +51481,7 @@
       <c r="D17" s="9">
         <v>1.0</v>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="13">
         <v>46158.840069502316</v>
       </c>
       <c r="F17" s="4"/>
@@ -51497,11 +51494,11 @@
       <c r="M17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="5"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="21"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -51512,13 +51509,13 @@
       <c r="M18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>14</v>
+      <c r="A19" s="6" t="s">
+        <v>16</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="6"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="10"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -51529,19 +51526,19 @@
       <c r="M19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>9</v>
+      <c r="A20" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="7">
         <v>6.0</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="7">
         <v>45.0</v>
       </c>
       <c r="D20" s="9">
         <v>1.0</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="13">
         <v>46203.65718435185</v>
       </c>
       <c r="F20" s="4"/>
@@ -51554,19 +51551,19 @@
       <c r="M20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>10</v>
+      <c r="A21" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="7">
         <v>18.0</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="7">
         <v>20.0</v>
       </c>
       <c r="D21" s="9">
         <v>1.0</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="13">
         <v>46155.874796793985</v>
       </c>
       <c r="F21" s="4"/>
@@ -51579,11 +51576,11 @@
       <c r="M21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="8"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="6"/>
+      <c r="A22" s="5"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="10"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -51594,15 +51591,15 @@
       <c r="M22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="s">
-        <v>14</v>
+      <c r="A23" s="24" t="s">
+        <v>16</v>
       </c>
-      <c r="B23" s="28" t="s">
-        <v>22</v>
+      <c r="B23" s="25" t="s">
+        <v>19</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="10">
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="13">
         <v>46155.850816817125</v>
       </c>
       <c r="F23" s="4"/>
@@ -51615,19 +51612,19 @@
       <c r="M23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>19</v>
+      <c r="A24" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="7">
         <v>6.0</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="7">
         <v>50.0</v>
       </c>
       <c r="D24" s="9">
         <v>1.0</v>
       </c>
-      <c r="E24" s="10">
+      <c r="E24" s="13">
         <v>46155.86764509259</v>
       </c>
       <c r="F24" s="4"/>
@@ -51640,19 +51637,19 @@
       <c r="M24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>9</v>
+      <c r="A25" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="7">
         <v>8.0</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="7">
         <v>30.0</v>
       </c>
       <c r="D25" s="9">
         <v>1.0</v>
       </c>
-      <c r="E25" s="10">
+      <c r="E25" s="13">
         <v>46155.86212506944</v>
       </c>
       <c r="F25" s="4"/>
@@ -51665,23 +51662,23 @@
       <c r="M25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>16</v>
+      <c r="A26" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="7">
         <v>10.0</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="7">
         <v>30.0</v>
       </c>
       <c r="D26" s="9">
         <v>4.0</v>
       </c>
-      <c r="E26" s="10">
+      <c r="E26" s="13">
         <v>46156.84678416667</v>
       </c>
-      <c r="F26" s="13" t="s">
-        <v>25</v>
+      <c r="F26" s="14" t="s">
+        <v>22</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -51692,19 +51689,19 @@
       <c r="M26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>16</v>
+      <c r="A27" s="5" t="s">
+        <v>15</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="7">
         <v>17.0</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="7">
         <v>15.0</v>
       </c>
       <c r="D27" s="9">
         <v>1.0</v>
       </c>
-      <c r="E27" s="10">
+      <c r="E27" s="13">
         <v>46155.877253784725</v>
       </c>
       <c r="F27" s="4"/>
@@ -51717,11 +51714,11 @@
       <c r="M27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="8"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="6"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -51732,15 +51729,15 @@
       <c r="M28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="s">
-        <v>21</v>
+      <c r="A29" s="24" t="s">
+        <v>23</v>
       </c>
-      <c r="B29" s="28" t="s">
-        <v>22</v>
+      <c r="B29" s="25" t="s">
+        <v>19</v>
       </c>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="6"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="10"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -51751,19 +51748,19 @@
       <c r="M29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>19</v>
+      <c r="A30" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="7">
         <v>6.0</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="7">
         <v>50.0</v>
       </c>
       <c r="D30" s="9">
         <v>1.0</v>
       </c>
-      <c r="E30" s="10">
+      <c r="E30" s="13">
         <v>46155.89164559028</v>
       </c>
       <c r="F30" s="4"/>
@@ -51776,19 +51773,19 @@
       <c r="M30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
-        <v>9</v>
+      <c r="A31" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="7">
         <v>8.0</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="7">
         <v>30.0</v>
       </c>
       <c r="D31" s="9">
         <v>1.0</v>
       </c>
-      <c r="E31" s="6"/>
+      <c r="E31" s="10"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -51799,19 +51796,19 @@
       <c r="M31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
-        <v>10</v>
+      <c r="A32" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="7">
         <v>15.0</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="7">
         <v>10.0</v>
       </c>
       <c r="D32" s="9">
         <v>2.0</v>
       </c>
-      <c r="E32" s="10">
+      <c r="E32" s="13">
         <v>46176.957761134254</v>
       </c>
       <c r="F32" s="4"/>
@@ -51824,11 +51821,11 @@
       <c r="M32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="8"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="6"/>
+      <c r="A33" s="5"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="10"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -51840,12 +51837,12 @@
     </row>
     <row r="34">
       <c r="A34" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
       <c r="D34" s="16"/>
-      <c r="E34" s="20"/>
+      <c r="E34" s="26"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -51857,18 +51854,18 @@
     </row>
     <row r="35">
       <c r="A35" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
-      <c r="B35" s="40" t="s">
-        <v>30</v>
+      <c r="B35" s="35" t="s">
+        <v>28</v>
       </c>
-      <c r="C35" s="40">
+      <c r="C35" s="35">
         <v>40.0</v>
       </c>
-      <c r="D35" s="40">
+      <c r="D35" s="35">
         <v>1.0</v>
       </c>
-      <c r="E35" s="17">
+      <c r="E35" s="22">
         <v>46213.75115673611</v>
       </c>
       <c r="F35" s="4"/>
@@ -51882,18 +51879,18 @@
     </row>
     <row r="36">
       <c r="A36" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="B36" s="40">
+      <c r="B36" s="35">
         <v>30.0</v>
       </c>
-      <c r="C36" s="40">
+      <c r="C36" s="35">
         <v>15.0</v>
       </c>
-      <c r="D36" s="40">
+      <c r="D36" s="35">
         <v>1.0</v>
       </c>
-      <c r="E36" s="20"/>
+      <c r="E36" s="26"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -51904,8 +51901,8 @@
       <c r="M36" s="4"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>19</v>
+      <c r="A37" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="B37" s="9">
         <v>10.0</v>
@@ -51916,7 +51913,7 @@
       <c r="D37" s="9">
         <v>1.0</v>
       </c>
-      <c r="E37" s="10">
+      <c r="E37" s="13">
         <v>46233.612064189816</v>
       </c>
       <c r="F37" s="4"/>
@@ -51929,11 +51926,11 @@
       <c r="M37" s="4"/>
     </row>
     <row r="38">
-      <c r="A38" s="25"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="6"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="10"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -51944,13 +51941,13 @@
       <c r="M38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="s">
-        <v>32</v>
+      <c r="A39" s="6" t="s">
+        <v>29</v>
       </c>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="6"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="10"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -51961,8 +51958,8 @@
       <c r="M39" s="4"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="s">
-        <v>10</v>
+      <c r="A40" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B40" s="9">
         <v>40.0</v>
@@ -51973,7 +51970,7 @@
       <c r="D40" s="9">
         <v>1.0</v>
       </c>
-      <c r="E40" s="10">
+      <c r="E40" s="13">
         <v>46203.63427946759</v>
       </c>
       <c r="F40" s="4"/>
@@ -51986,11 +51983,11 @@
       <c r="M40" s="4"/>
     </row>
     <row r="41">
-      <c r="A41" s="5"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="6"/>
+      <c r="A41" s="6"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="10"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -52001,13 +51998,13 @@
       <c r="M41" s="4"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="s">
-        <v>23</v>
+      <c r="A42" s="6" t="s">
+        <v>24</v>
       </c>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="6"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="10"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -52018,8 +52015,8 @@
       <c r="M42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="s">
-        <v>9</v>
+      <c r="A43" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B43" s="9">
         <v>9.0</v>
@@ -52030,7 +52027,7 @@
       <c r="D43" s="9">
         <v>1.0</v>
       </c>
-      <c r="E43" s="10">
+      <c r="E43" s="13">
         <v>46006.95620635417</v>
       </c>
       <c r="F43" s="4"/>
@@ -52043,8 +52040,8 @@
       <c r="M43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="s">
-        <v>10</v>
+      <c r="A44" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B44" s="9">
         <v>55.0</v>
@@ -52055,7 +52052,7 @@
       <c r="D44" s="9">
         <v>1.0</v>
       </c>
-      <c r="E44" s="10">
+      <c r="E44" s="13">
         <v>46006.95627618056</v>
       </c>
       <c r="F44" s="4"/>
@@ -52068,8 +52065,8 @@
       <c r="M44" s="4"/>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="s">
-        <v>9</v>
+      <c r="A45" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B45" s="9">
         <v>10.0</v>
@@ -52080,11 +52077,11 @@
       <c r="D45" s="9">
         <v>1.0</v>
       </c>
-      <c r="E45" s="10">
+      <c r="E45" s="13">
         <v>46038.439073761576</v>
       </c>
-      <c r="F45" s="13" t="s">
-        <v>33</v>
+      <c r="F45" s="14" t="s">
+        <v>31</v>
       </c>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -52095,11 +52092,11 @@
       <c r="M45" s="4"/>
     </row>
     <row r="46">
-      <c r="A46" s="42"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="6"/>
+      <c r="A46" s="39"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="10"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -52110,13 +52107,13 @@
       <c r="M46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="s">
-        <v>26</v>
+      <c r="A47" s="6" t="s">
+        <v>25</v>
       </c>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="6"/>
+      <c r="B47" s="12"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="10"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -52127,8 +52124,8 @@
       <c r="M47" s="4"/>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="s">
-        <v>10</v>
+      <c r="A48" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B48" s="9">
         <v>55.0</v>
@@ -52139,7 +52136,7 @@
       <c r="D48" s="9">
         <v>1.0</v>
       </c>
-      <c r="E48" s="10">
+      <c r="E48" s="13">
         <v>46233.62550483797</v>
       </c>
       <c r="F48" s="4"/>
@@ -52152,19 +52149,19 @@
       <c r="M48" s="4"/>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="s">
-        <v>17</v>
+      <c r="A49" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="7">
         <v>40.0</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="7">
         <v>300.0</v>
       </c>
-      <c r="D49" s="11">
+      <c r="D49" s="7">
         <v>1.0</v>
       </c>
-      <c r="E49" s="10">
+      <c r="E49" s="13">
         <v>46318.6234527662</v>
       </c>
       <c r="F49" s="4"/>
@@ -52177,11 +52174,11 @@
       <c r="M49" s="4"/>
     </row>
     <row r="50">
-      <c r="A50" s="42"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="6"/>
+      <c r="A50" s="39"/>
+      <c r="B50" s="12"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="10"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -52192,13 +52189,13 @@
       <c r="M50" s="4"/>
     </row>
     <row r="51">
-      <c r="A51" s="42" t="s">
-        <v>27</v>
+      <c r="A51" s="39" t="s">
+        <v>26</v>
       </c>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="6"/>
+      <c r="B51" s="12"/>
+      <c r="C51" s="12"/>
+      <c r="D51" s="12"/>
+      <c r="E51" s="10"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -52209,8 +52206,8 @@
       <c r="M51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="s">
-        <v>10</v>
+      <c r="A52" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="B52" s="9">
         <v>60.0</v>
@@ -52221,7 +52218,7 @@
       <c r="D52" s="9">
         <v>1.0</v>
       </c>
-      <c r="E52" s="10">
+      <c r="E52" s="13">
         <v>46203.63265940972</v>
       </c>
       <c r="F52" s="4"/>
@@ -52234,8 +52231,8 @@
       <c r="M52" s="4"/>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="s">
-        <v>9</v>
+      <c r="A53" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B53" s="9">
         <v>10.0</v>
@@ -52246,7 +52243,7 @@
       <c r="D53" s="9">
         <v>1.0</v>
       </c>
-      <c r="E53" s="10">
+      <c r="E53" s="13">
         <v>46253.61151159722</v>
       </c>
       <c r="F53" s="4"/>
@@ -52259,11 +52256,11 @@
       <c r="M53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="42"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="6"/>
+      <c r="A54" s="39"/>
+      <c r="B54" s="12"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="10"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -52274,13 +52271,13 @@
       <c r="M54" s="4"/>
     </row>
     <row r="55">
-      <c r="A55" s="42" t="s">
-        <v>34</v>
+      <c r="A55" s="39" t="s">
+        <v>33</v>
       </c>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="6"/>
+      <c r="B55" s="12"/>
+      <c r="C55" s="12"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="10"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -52291,19 +52288,19 @@
       <c r="M55" s="4"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="s">
-        <v>17</v>
+      <c r="A56" s="5" t="s">
+        <v>13</v>
       </c>
-      <c r="B56" s="11">
+      <c r="B56" s="7">
         <v>70.0</v>
       </c>
-      <c r="C56" s="11">
+      <c r="C56" s="7">
         <v>300.0</v>
       </c>
-      <c r="D56" s="11">
+      <c r="D56" s="7">
         <v>1.0</v>
       </c>
-      <c r="E56" s="10">
+      <c r="E56" s="13">
         <v>46223.80899857639</v>
       </c>
       <c r="F56" s="4"/>
@@ -52316,19 +52313,19 @@
       <c r="M56" s="4"/>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="s">
-        <v>9</v>
+      <c r="A57" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="B57" s="11">
+      <c r="B57" s="7">
         <v>10.0</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="7">
         <v>20.0</v>
       </c>
-      <c r="D57" s="11">
+      <c r="D57" s="7">
         <v>1.0</v>
       </c>
-      <c r="E57" s="10">
+      <c r="E57" s="13">
         <v>46223.80911148148</v>
       </c>
       <c r="F57" s="4"/>
@@ -52341,19 +52338,19 @@
       <c r="M57" s="4"/>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="s">
-        <v>10</v>
+      <c r="A58" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B58" s="11">
+      <c r="B58" s="7">
         <v>70.0</v>
       </c>
-      <c r="C58" s="11">
+      <c r="C58" s="7">
         <v>8.0</v>
       </c>
-      <c r="D58" s="11">
+      <c r="D58" s="7">
         <v>1.0</v>
       </c>
-      <c r="E58" s="10">
+      <c r="E58" s="13">
         <v>46260.758642430555</v>
       </c>
       <c r="F58" s="4"/>
@@ -52366,11 +52363,11 @@
       <c r="M58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="8"/>
+      <c r="A59" s="5"/>
       <c r="B59" s="9"/>
       <c r="C59" s="9"/>
       <c r="D59" s="9"/>
-      <c r="E59" s="6"/>
+      <c r="E59" s="10"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -52381,15 +52378,15 @@
       <c r="M59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="s">
-        <v>35</v>
+      <c r="A60" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C60" s="9"/>
       <c r="D60" s="9"/>
-      <c r="E60" s="10">
+      <c r="E60" s="13">
         <v>45946.87875708334</v>
       </c>
       <c r="F60" s="4"/>
@@ -52402,15 +52399,15 @@
       <c r="M60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="8">
+      <c r="A61" s="5">
         <v>50.0</v>
       </c>
       <c r="B61" s="9">
         <v>100.0</v>
       </c>
-      <c r="C61" s="14"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="10">
+      <c r="C61" s="12"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="13">
         <v>45946.87887299768</v>
       </c>
       <c r="F61" s="4"/>
@@ -52424,7 +52421,7 @@
     </row>
     <row r="62">
       <c r="A62" s="43" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B62" s="44"/>
       <c r="C62" s="44"/>
@@ -52440,16 +52437,16 @@
       <c r="M62" s="4"/>
     </row>
     <row r="63">
-      <c r="A63" s="38" t="s">
-        <v>38</v>
+      <c r="A63" s="41" t="s">
+        <v>37</v>
       </c>
-      <c r="B63" s="38">
+      <c r="B63" s="41">
         <v>100.0</v>
       </c>
-      <c r="C63" s="13">
+      <c r="C63" s="14">
         <v>1.0</v>
       </c>
-      <c r="D63" s="13">
+      <c r="D63" s="14">
         <v>2.0</v>
       </c>
       <c r="E63" s="46">
@@ -52465,8 +52462,8 @@
       <c r="M63" s="4"/>
     </row>
     <row r="64">
-      <c r="A64" s="39"/>
-      <c r="B64" s="39"/>
+      <c r="A64" s="42"/>
+      <c r="B64" s="42"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
@@ -52480,10 +52477,10 @@
       <c r="M64" s="4"/>
     </row>
     <row r="65">
-      <c r="A65" s="38" t="s">
-        <v>39</v>
+      <c r="A65" s="41" t="s">
+        <v>38</v>
       </c>
-      <c r="B65" s="39"/>
+      <c r="B65" s="42"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
@@ -52497,16 +52494,16 @@
       <c r="M65" s="4"/>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="s">
-        <v>10</v>
+      <c r="A66" s="5" t="s">
+        <v>9</v>
       </c>
-      <c r="B66" s="38">
+      <c r="B66" s="41">
         <v>50.0</v>
       </c>
-      <c r="C66" s="13">
+      <c r="C66" s="14">
         <v>20.0</v>
       </c>
-      <c r="D66" s="13">
+      <c r="D66" s="14">
         <v>1.0</v>
       </c>
       <c r="E66" s="46">
@@ -52522,13 +52519,13 @@
       <c r="M66" s="4"/>
     </row>
     <row r="67">
-      <c r="A67" s="38" t="s">
-        <v>40</v>
+      <c r="A67" s="41" t="s">
+        <v>39</v>
       </c>
-      <c r="B67" s="38">
+      <c r="B67" s="41">
         <v>15.0</v>
       </c>
-      <c r="C67" s="13">
+      <c r="C67" s="14">
         <v>16.0</v>
       </c>
       <c r="D67" s="4"/>
@@ -52545,8 +52542,8 @@
       <c r="M67" s="4"/>
     </row>
     <row r="68">
-      <c r="A68" s="39"/>
-      <c r="B68" s="39"/>
+      <c r="A68" s="42"/>
+      <c r="B68" s="42"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
       <c r="E68" s="4"/>
@@ -52560,11 +52557,11 @@
       <c r="M68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="38" t="s">
-        <v>41</v>
+      <c r="A69" s="41" t="s">
+        <v>40</v>
       </c>
-      <c r="B69" s="38" t="s">
-        <v>26</v>
+      <c r="B69" s="41" t="s">
+        <v>25</v>
       </c>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
@@ -52581,16 +52578,16 @@
       <c r="M69" s="4"/>
     </row>
     <row r="70">
-      <c r="A70" s="38" t="s">
-        <v>42</v>
+      <c r="A70" s="41" t="s">
+        <v>41</v>
       </c>
-      <c r="B70" s="38">
+      <c r="B70" s="41">
         <v>5.0</v>
       </c>
-      <c r="C70" s="13">
+      <c r="C70" s="14">
         <v>80.0</v>
       </c>
-      <c r="D70" s="13">
+      <c r="D70" s="14">
         <v>1.0</v>
       </c>
       <c r="E70" s="46">
@@ -52606,16 +52603,16 @@
       <c r="M70" s="4"/>
     </row>
     <row r="71">
-      <c r="A71" s="38" t="s">
-        <v>43</v>
+      <c r="A71" s="41" t="s">
+        <v>42</v>
       </c>
-      <c r="B71" s="38">
+      <c r="B71" s="41">
         <v>15.0</v>
       </c>
-      <c r="C71" s="13">
+      <c r="C71" s="14">
         <v>10.0</v>
       </c>
-      <c r="D71" s="13">
+      <c r="D71" s="14">
         <v>1.0</v>
       </c>
       <c r="E71" s="46">
@@ -52631,16 +52628,16 @@
       <c r="M71" s="4"/>
     </row>
     <row r="72">
-      <c r="A72" s="38" t="s">
-        <v>16</v>
+      <c r="A72" s="41" t="s">
+        <v>15</v>
       </c>
-      <c r="B72" s="38">
+      <c r="B72" s="41">
         <v>30.0</v>
       </c>
-      <c r="C72" s="13">
+      <c r="C72" s="14">
         <v>10.0</v>
       </c>
-      <c r="D72" s="13">
+      <c r="D72" s="14">
         <v>1.0</v>
       </c>
       <c r="E72" s="46">
@@ -52656,8 +52653,8 @@
       <c r="M72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="39"/>
-      <c r="B73" s="39"/>
+      <c r="A73" s="42"/>
+      <c r="B73" s="42"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
@@ -52671,11 +52668,11 @@
       <c r="M73" s="4"/>
     </row>
     <row r="74">
-      <c r="A74" s="38" t="s">
-        <v>41</v>
+      <c r="A74" s="41" t="s">
+        <v>40</v>
       </c>
-      <c r="B74" s="38" t="s">
-        <v>34</v>
+      <c r="B74" s="41" t="s">
+        <v>33</v>
       </c>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
@@ -52692,16 +52689,16 @@
       <c r="M74" s="4"/>
     </row>
     <row r="75">
-      <c r="A75" s="38" t="s">
-        <v>42</v>
+      <c r="A75" s="41" t="s">
+        <v>41</v>
       </c>
-      <c r="B75" s="38">
+      <c r="B75" s="41">
         <v>5.0</v>
       </c>
-      <c r="C75" s="13">
+      <c r="C75" s="14">
         <v>80.0</v>
       </c>
-      <c r="D75" s="13">
+      <c r="D75" s="14">
         <v>1.0</v>
       </c>
       <c r="E75" s="4"/>
@@ -52715,16 +52712,16 @@
       <c r="M75" s="4"/>
     </row>
     <row r="76">
-      <c r="A76" s="38" t="s">
-        <v>43</v>
+      <c r="A76" s="41" t="s">
+        <v>42</v>
       </c>
-      <c r="B76" s="38">
+      <c r="B76" s="41">
         <v>15.0</v>
       </c>
-      <c r="C76" s="13">
+      <c r="C76" s="14">
         <v>10.0</v>
       </c>
-      <c r="D76" s="13">
+      <c r="D76" s="14">
         <v>1.0</v>
       </c>
       <c r="E76" s="4"/>
@@ -52738,16 +52735,16 @@
       <c r="M76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="38" t="s">
-        <v>16</v>
+      <c r="A77" s="41" t="s">
+        <v>15</v>
       </c>
-      <c r="B77" s="38">
+      <c r="B77" s="41">
         <v>20.0</v>
       </c>
-      <c r="C77" s="13">
+      <c r="C77" s="14">
         <v>10.0</v>
       </c>
-      <c r="D77" s="13">
+      <c r="D77" s="14">
         <v>6.0</v>
       </c>
       <c r="E77" s="46">
@@ -52763,8 +52760,8 @@
       <c r="M77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="39"/>
-      <c r="B78" s="39"/>
+      <c r="A78" s="42"/>
+      <c r="B78" s="42"/>
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
@@ -52778,8 +52775,8 @@
       <c r="M78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="38"/>
-      <c r="B79" s="39"/>
+      <c r="A79" s="41"/>
+      <c r="B79" s="42"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
@@ -52793,8 +52790,8 @@
       <c r="M79" s="4"/>
     </row>
     <row r="80">
-      <c r="A80" s="39"/>
-      <c r="B80" s="39"/>
+      <c r="A80" s="42"/>
+      <c r="B80" s="42"/>
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
       <c r="E80" s="4"/>

</xml_diff>